<commit_message>
auto: modify 01-Projects (1)
</commit_message>
<xml_diff>
--- a/01-Projects/family-hub/credit-card-management/信用卡主控表.xlsx
+++ b/01-Projects/family-hub/credit-card-management/信用卡主控表.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyFile\AI\ContextStack\01-Projects\family-hub\credit-card-management\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ProjectGroup\AI\ContextStack\01-Projects\family-hub\credit-card-management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F60DEDA-A14A-47F7-9F29-5E6D1339C1EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="1-卡片信息" sheetId="1" r:id="rId1"/>
@@ -25,7 +24,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1-卡片信息'!$A$2:$G$19</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1199,7 +1198,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="20">
     <font>
       <sz val="11"/>
@@ -1726,6 +1725,9 @@
     <xf numFmtId="0" fontId="11" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1753,9 +1755,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -2154,7 +2153,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF4472C4"/>
   </sheetPr>
@@ -2170,15 +2169,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="63" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63"/>
-      <c r="F1" s="63"/>
-      <c r="G1" s="63"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
     </row>
     <row r="2" spans="1:8" ht="24.95" customHeight="1">
       <c r="A2" s="1" t="s">
@@ -2321,7 +2320,7 @@
         <v>41000</v>
       </c>
       <c r="F7" s="2">
-        <v>59000</v>
+        <v>109000</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>23</v>
@@ -2391,10 +2390,10 @@
       <c r="D10" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="77">
+      <c r="E10" s="62">
         <v>80000</v>
       </c>
-      <c r="F10" s="77">
+      <c r="F10" s="62">
         <v>72000</v>
       </c>
       <c r="G10" s="8" t="s">
@@ -2597,44 +2596,44 @@
       <c r="H18" s="26"/>
     </row>
     <row r="19" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A19" s="68" t="s">
+      <c r="A19" s="69" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="66"/>
-      <c r="C19" s="66"/>
-      <c r="D19" s="67"/>
+      <c r="B19" s="67"/>
+      <c r="C19" s="67"/>
+      <c r="D19" s="68"/>
       <c r="E19" s="3">
         <f>SUM(E3:E18)</f>
         <v>831000</v>
       </c>
       <c r="F19" s="3">
         <f>SUM(F3:F18)</f>
-        <v>1055500</v>
+        <v>1105500</v>
       </c>
       <c r="G19" s="11"/>
       <c r="H19" s="26"/>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A21" s="64" t="s">
+      <c r="A21" s="65" t="s">
         <v>56</v>
       </c>
-      <c r="B21" s="63"/>
-      <c r="C21" s="63"/>
-      <c r="D21" s="63"/>
-      <c r="E21" s="63"/>
-      <c r="F21" s="63"/>
-      <c r="G21" s="63"/>
+      <c r="B21" s="64"/>
+      <c r="C21" s="64"/>
+      <c r="D21" s="64"/>
+      <c r="E21" s="64"/>
+      <c r="F21" s="64"/>
+      <c r="G21" s="64"/>
     </row>
     <row r="24" spans="1:8" ht="21" customHeight="1">
-      <c r="A24" s="62" t="s">
+      <c r="A24" s="63" t="s">
         <v>57</v>
       </c>
-      <c r="B24" s="63"/>
-      <c r="C24" s="63"/>
-      <c r="D24" s="63"/>
-      <c r="E24" s="63"/>
-      <c r="F24" s="63"/>
-      <c r="G24" s="63"/>
+      <c r="B24" s="64"/>
+      <c r="C24" s="64"/>
+      <c r="D24" s="64"/>
+      <c r="E24" s="64"/>
+      <c r="F24" s="64"/>
+      <c r="G24" s="64"/>
     </row>
     <row r="25" spans="1:8" ht="21" customHeight="1">
       <c r="A25" s="38" t="s">
@@ -2917,12 +2916,12 @@
       <c r="H37" s="53"/>
     </row>
     <row r="38" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A38" s="65" t="s">
+      <c r="A38" s="66" t="s">
         <v>73</v>
       </c>
-      <c r="B38" s="66"/>
-      <c r="C38" s="66"/>
-      <c r="D38" s="67"/>
+      <c r="B38" s="67"/>
+      <c r="C38" s="67"/>
+      <c r="D38" s="68"/>
       <c r="E38" s="41">
         <f>SUM(E26:E37)</f>
         <v>11000</v>
@@ -2935,7 +2934,7 @@
       <c r="H38" s="53"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:G19" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A2:G19"/>
   <mergeCells count="5">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A21:G21"/>
@@ -2950,7 +2949,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FFED7D31"/>
   </sheetPr>
@@ -2969,28 +2968,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="63" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63"/>
-      <c r="F1" s="63"/>
-      <c r="G1" s="63"/>
-      <c r="H1" s="63"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1">
-      <c r="A3" s="70" t="s">
+      <c r="A3" s="71" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="66"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="67"/>
+      <c r="B3" s="67"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="68"/>
       <c r="I3" s="24"/>
     </row>
     <row r="4" spans="1:9" ht="33" customHeight="1">
@@ -3150,16 +3149,16 @@
       <c r="I9" s="13"/>
     </row>
     <row r="10" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A10" s="70" t="s">
+      <c r="A10" s="71" t="s">
         <v>94</v>
       </c>
-      <c r="B10" s="66"/>
-      <c r="C10" s="66"/>
-      <c r="D10" s="66"/>
-      <c r="E10" s="66"/>
-      <c r="F10" s="66"/>
-      <c r="G10" s="66"/>
-      <c r="H10" s="67"/>
+      <c r="B10" s="67"/>
+      <c r="C10" s="67"/>
+      <c r="D10" s="67"/>
+      <c r="E10" s="67"/>
+      <c r="F10" s="67"/>
+      <c r="G10" s="67"/>
+      <c r="H10" s="68"/>
       <c r="I10" s="24"/>
     </row>
     <row r="11" spans="1:9" ht="16.5" customHeight="1">
@@ -3367,16 +3366,16 @@
       <c r="I18" s="13"/>
     </row>
     <row r="19" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A19" s="70" t="s">
+      <c r="A19" s="71" t="s">
         <v>109</v>
       </c>
-      <c r="B19" s="66"/>
-      <c r="C19" s="66"/>
-      <c r="D19" s="66"/>
-      <c r="E19" s="66"/>
-      <c r="F19" s="66"/>
-      <c r="G19" s="66"/>
-      <c r="H19" s="67"/>
+      <c r="B19" s="67"/>
+      <c r="C19" s="67"/>
+      <c r="D19" s="67"/>
+      <c r="E19" s="67"/>
+      <c r="F19" s="67"/>
+      <c r="G19" s="67"/>
+      <c r="H19" s="68"/>
       <c r="I19" s="24"/>
     </row>
     <row r="20" spans="1:9" ht="16.5" customHeight="1">
@@ -3501,16 +3500,16 @@
       <c r="I24" s="13"/>
     </row>
     <row r="25" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A25" s="70" t="s">
+      <c r="A25" s="71" t="s">
         <v>117</v>
       </c>
-      <c r="B25" s="66"/>
-      <c r="C25" s="66"/>
-      <c r="D25" s="66"/>
-      <c r="E25" s="66"/>
-      <c r="F25" s="66"/>
-      <c r="G25" s="66"/>
-      <c r="H25" s="67"/>
+      <c r="B25" s="67"/>
+      <c r="C25" s="67"/>
+      <c r="D25" s="67"/>
+      <c r="E25" s="67"/>
+      <c r="F25" s="67"/>
+      <c r="G25" s="67"/>
+      <c r="H25" s="68"/>
       <c r="I25" s="24"/>
     </row>
     <row r="26" spans="1:9" ht="16.5" customHeight="1">
@@ -3626,16 +3625,16 @@
       </c>
     </row>
     <row r="32" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A32" s="69" t="s">
+      <c r="A32" s="70" t="s">
         <v>133</v>
       </c>
-      <c r="B32" s="63"/>
-      <c r="C32" s="63"/>
-      <c r="D32" s="63"/>
-      <c r="E32" s="63"/>
-      <c r="F32" s="63"/>
-      <c r="G32" s="63"/>
-      <c r="H32" s="63"/>
+      <c r="B32" s="64"/>
+      <c r="C32" s="64"/>
+      <c r="D32" s="64"/>
+      <c r="E32" s="64"/>
+      <c r="F32" s="64"/>
+      <c r="G32" s="64"/>
+      <c r="H32" s="64"/>
     </row>
     <row r="35" spans="1:9" ht="14.25" customHeight="1">
       <c r="A35" s="36" t="s">
@@ -4028,7 +4027,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF70AD47"/>
   </sheetPr>
@@ -4043,24 +4042,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="63" t="s">
         <v>153</v>
       </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63"/>
-      <c r="F1" s="63"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
     </row>
     <row r="2" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="65" t="s">
         <v>154</v>
       </c>
-      <c r="B2" s="63"/>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
+      <c r="B2" s="64"/>
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
+      <c r="E2" s="64"/>
+      <c r="F2" s="64"/>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -4381,14 +4380,14 @@
       <c r="F19" s="8"/>
     </row>
     <row r="21" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A21" s="64" t="s">
+      <c r="A21" s="65" t="s">
         <v>159</v>
       </c>
-      <c r="B21" s="63"/>
-      <c r="C21" s="63"/>
-      <c r="D21" s="63"/>
-      <c r="E21" s="63"/>
-      <c r="F21" s="63"/>
+      <c r="B21" s="64"/>
+      <c r="C21" s="64"/>
+      <c r="D21" s="64"/>
+      <c r="E21" s="64"/>
+      <c r="F21" s="64"/>
     </row>
     <row r="24" spans="1:6" ht="14.25">
       <c r="A24" s="36" t="s">
@@ -4613,7 +4612,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
@@ -4629,28 +4628,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="63" t="s">
         <v>164</v>
       </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63"/>
-      <c r="F1" s="63"/>
-      <c r="G1" s="63"/>
-      <c r="H1" s="63"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
-      <c r="A3" s="71" t="s">
+      <c r="A3" s="72" t="s">
         <v>165</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63"/>
+      <c r="B3" s="64"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -4965,26 +4964,26 @@
       </c>
     </row>
     <row r="16" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A16" s="72" t="s">
+      <c r="A16" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="66"/>
-      <c r="C16" s="66"/>
-      <c r="D16" s="66"/>
-      <c r="E16" s="67"/>
-      <c r="F16" s="72" t="s">
+      <c r="B16" s="67"/>
+      <c r="C16" s="67"/>
+      <c r="D16" s="67"/>
+      <c r="E16" s="68"/>
+      <c r="F16" s="73" t="s">
         <v>178</v>
       </c>
-      <c r="G16" s="67"/>
+      <c r="G16" s="68"/>
       <c r="H16" s="8" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A17" s="73" t="s">
+      <c r="A17" s="74" t="s">
         <v>205</v>
       </c>
-      <c r="B17" s="67"/>
+      <c r="B17" s="68"/>
       <c r="C17">
         <f>SUM(C5:C15)</f>
         <v>39</v>
@@ -4997,21 +4996,21 @@
         <f>SUM(E5:E15)</f>
         <v>39</v>
       </c>
-      <c r="F17" s="73" t="s">
+      <c r="F17" s="74" t="s">
         <v>206</v>
       </c>
-      <c r="G17" s="67"/>
+      <c r="G17" s="68"/>
       <c r="H17" s="21"/>
     </row>
     <row r="18" spans="1:8" ht="15" customHeight="1">
-      <c r="A18" s="63"/>
-      <c r="B18" s="63"/>
-      <c r="C18" s="63"/>
-      <c r="D18" s="63"/>
-      <c r="E18" s="63"/>
-      <c r="F18" s="63"/>
-      <c r="G18" s="63"/>
-      <c r="H18" s="63"/>
+      <c r="A18" s="64"/>
+      <c r="B18" s="64"/>
+      <c r="C18" s="64"/>
+      <c r="D18" s="64"/>
+      <c r="E18" s="64"/>
+      <c r="F18" s="64"/>
+      <c r="G18" s="64"/>
+      <c r="H18" s="64"/>
     </row>
     <row r="19" spans="1:8" ht="15" customHeight="1">
       <c r="A19" s="33" t="s">
@@ -5391,7 +5390,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FFA5A5A5"/>
   </sheetPr>
@@ -5405,25 +5404,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="63" t="s">
         <v>230</v>
       </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63"/>
-      <c r="F1" s="63"/>
-      <c r="G1" s="63"/>
-      <c r="H1" s="63"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
-      <c r="A3" s="71" t="s">
+      <c r="A3" s="72" t="s">
         <v>231</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
+      <c r="B3" s="64"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -5511,16 +5510,16 @@
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
-      <c r="A11" s="71" t="s">
+      <c r="A11" s="72" t="s">
         <v>251</v>
       </c>
-      <c r="B11" s="63"/>
-      <c r="C11" s="63"/>
-      <c r="D11" s="63"/>
-      <c r="E11" s="63"/>
-      <c r="F11" s="63"/>
-      <c r="G11" s="63"/>
-      <c r="H11" s="63"/>
+      <c r="B11" s="64"/>
+      <c r="C11" s="64"/>
+      <c r="D11" s="64"/>
+      <c r="E11" s="64"/>
+      <c r="F11" s="64"/>
+      <c r="G11" s="64"/>
+      <c r="H11" s="64"/>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
       <c r="A12" s="1" t="s">
@@ -5660,7 +5659,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
@@ -5676,24 +5675,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="63" t="s">
         <v>258</v>
       </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63"/>
-      <c r="F1" s="63"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1">
-      <c r="A3" s="71" t="s">
+      <c r="A3" s="72" t="s">
         <v>259</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
+      <c r="B3" s="64"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1">
       <c r="A4" s="5" t="s">
@@ -5776,10 +5775,10 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A8" s="75" t="s">
+      <c r="A8" s="76" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="67"/>
+      <c r="B8" s="68"/>
       <c r="C8" s="35">
         <v>500</v>
       </c>
@@ -5814,18 +5813,18 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1">
-      <c r="A10" s="74"/>
-      <c r="B10" s="66"/>
-      <c r="C10" s="66"/>
-      <c r="D10" s="66"/>
-      <c r="E10" s="66"/>
-      <c r="F10" s="67"/>
+      <c r="A10" s="75"/>
+      <c r="B10" s="67"/>
+      <c r="C10" s="67"/>
+      <c r="D10" s="67"/>
+      <c r="E10" s="67"/>
+      <c r="F10" s="68"/>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1">
-      <c r="A11" s="73" t="s">
+      <c r="A11" s="74" t="s">
         <v>205</v>
       </c>
-      <c r="B11" s="67"/>
+      <c r="B11" s="68"/>
       <c r="C11" s="34">
         <f>SUM(C5:C9)</f>
         <v>4180</v>
@@ -5886,14 +5885,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="15" customHeight="1">
-      <c r="A17" s="72" t="s">
+      <c r="A17" s="73" t="s">
         <v>273</v>
       </c>
-      <c r="B17" s="66"/>
-      <c r="C17" s="66"/>
-      <c r="D17" s="66"/>
-      <c r="E17" s="66"/>
-      <c r="F17" s="67"/>
+      <c r="B17" s="67"/>
+      <c r="C17" s="67"/>
+      <c r="D17" s="67"/>
+      <c r="E17" s="67"/>
+      <c r="F17" s="68"/>
     </row>
     <row r="18" spans="1:6" ht="15" customHeight="1">
       <c r="A18" s="11" t="s">
@@ -5944,14 +5943,14 @@
       </c>
     </row>
     <row r="23" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A23" s="72" t="s">
+      <c r="A23" s="73" t="s">
         <v>171</v>
       </c>
-      <c r="B23" s="66"/>
-      <c r="C23" s="66"/>
-      <c r="D23" s="66"/>
-      <c r="E23" s="66"/>
-      <c r="F23" s="67"/>
+      <c r="B23" s="67"/>
+      <c r="C23" s="67"/>
+      <c r="D23" s="67"/>
+      <c r="E23" s="67"/>
+      <c r="F23" s="68"/>
     </row>
     <row r="24" spans="1:6" ht="16.5" customHeight="1">
       <c r="A24" s="8" t="s">
@@ -6108,7 +6107,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
@@ -6123,28 +6122,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="63" t="s">
         <v>289</v>
       </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63"/>
-      <c r="F1" s="63"/>
-      <c r="G1" s="63"/>
-      <c r="H1" s="63"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="65" t="s">
         <v>290</v>
       </c>
-      <c r="B2" s="63"/>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
-      <c r="H2" s="63"/>
+      <c r="B2" s="64"/>
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
+      <c r="E2" s="64"/>
+      <c r="F2" s="64"/>
+      <c r="G2" s="64"/>
+      <c r="H2" s="64"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -6505,7 +6504,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
@@ -6521,14 +6520,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="76" t="s">
+      <c r="A1" s="77" t="s">
         <v>303</v>
       </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63"/>
-      <c r="F1" s="63"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
     </row>
     <row r="2" spans="1:6" ht="24.95" customHeight="1">
       <c r="A2" s="9" t="s">

</xml_diff>

<commit_message>
credit card 0-bill cycle finalized: adjust statement dates, buffer cash 2.81w -> 1.10w
</commit_message>
<xml_diff>
--- a/01-Projects/family-hub/credit-card-management/信用卡主控表.xlsx
+++ b/01-Projects/family-hub/credit-card-management/信用卡主控表.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="1-卡片信息" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="965" uniqueCount="349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="970" uniqueCount="388">
   <si>
     <t>信用卡卡片总览 — 韩伟</t>
   </si>
@@ -460,9 +460,6 @@
     <t>10月19日</t>
   </si>
   <si>
-    <t>可兑航空里程</t>
-  </si>
-  <si>
     <t>15W</t>
   </si>
   <si>
@@ -511,30 +508,12 @@
     <t>规则：账单日 = 还款日，当天还清 → 征信报告显示0账单 | 操作：手机日历设提醒 → 当天云闪付还款 → Excel打✅</t>
   </si>
   <si>
-    <t>还款金额</t>
-  </si>
-  <si>
-    <t>本月已还</t>
-  </si>
-  <si>
-    <t>⬜</t>
-  </si>
-  <si>
-    <t>实际27号</t>
-  </si>
-  <si>
     <t>注意：部分银行账单日当天还款可能T+1入账，需测试各银行。</t>
   </si>
   <si>
     <t>❀ 爱人 — 还款日历</t>
   </si>
   <si>
-    <t>年费收取日，账单日待确认</t>
-  </si>
-  <si>
-    <t>账单日待确认</t>
-  </si>
-  <si>
     <t>待确认</t>
   </si>
   <si>
@@ -1016,14 +995,6 @@
   </si>
   <si>
     <t>没有申请按钮，需要分期？</t>
-  </si>
-  <si>
-    <t>18日</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>17日</t>
-    <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
     <t>消费15笔免</t>
@@ -1031,18 +1002,6 @@
   </si>
   <si>
     <t>年费：15笔/1W抵；权益待确认</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>年费：15笔抵</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>可不刷</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>可不刷；  实际16号</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
@@ -1078,10 +1037,6 @@
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
-    <t>兑换里程</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
     <t>银行APP直接搜索年费查询
 6月-9月可兑换</t>
     <phoneticPr fontId="7" type="noConversion"/>
@@ -1164,34 +1119,254 @@
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
+    <t>20日</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>21日</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>24日</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>年消费12W 免年费</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>年消费18W 免年费</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>兴业
+（注销）</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>实际还款</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>理论还款</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>满12W</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>满18W</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>30笔数</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>固定年费</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>满8W</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>10W积分</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>12笔数</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>20W积分</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>6笔数</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>【好卡】</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>40W积分</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>48笔数</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>15笔数</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>5笔数</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>合计</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>可兑航空里程50:1  年5W</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>里程15:1</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>里程50:1</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
     <r>
-      <t>年费收取日，账单日待确认；实际1</t>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>【好卡】年费：15笔抵；</t>
     </r>
     <r>
       <rPr>
-        <sz val="10"/>
-        <rFont val="微软雅黑"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
         <family val="2"/>
-        <charset val="134"/>
+        <scheme val="minor"/>
       </rPr>
-      <t>6日</t>
+      <t xml:space="preserve">
+</t>
     </r>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
-    <t>20日</t>
+    <t>日常微信小额多笔消费</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
-    <t>21日</t>
+    <t>有多少额度刷多少，没有里程兑换上限</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
-    <t>24日</t>
+    <t>每年5W 对应金额250W</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
-    <t>-</t>
+    <t>南航卡（重点刷）</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>兑换里程  只能一倍积分积累</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>10日</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>2日</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>实际16日
+1-26日都可以调整</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>10日</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>爱人-中信</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>鼎致白</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>农行（不刷）</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>爱人-农行</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>工商（不刷）</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>爱人-建行</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>爱人-交通</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>工商银行</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>最大可以兑换10W消费</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>光大-微信刷</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>普通白金卡</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>中信</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>27日</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>27号最优了</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>1日</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>7日</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>后续没有必要修改账单日</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>19日</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>26年无法修改</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>4日</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>账单日</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
@@ -1199,7 +1374,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="20">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1342,8 +1517,31 @@
       <name val="宋体"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF00B0F0"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1446,8 +1644,32 @@
         <bgColor rgb="FFFFCC99"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -1552,11 +1774,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1710,9 +1941,6 @@
     <xf numFmtId="0" fontId="3" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1726,6 +1954,13 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1755,11 +1990,69 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="21" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="20" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="20" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="20">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1797,6 +2090,70 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFFFC7CE"/>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2169,15 +2526,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
     </row>
     <row r="2" spans="1:8" ht="24.95" customHeight="1">
       <c r="A2" s="1" t="s">
@@ -2225,10 +2582,10 @@
         <v>0</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>343</v>
+        <v>330</v>
       </c>
       <c r="H3" s="53" t="s">
-        <v>341</v>
+        <v>328</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="16.5" customHeight="1">
@@ -2253,7 +2610,9 @@
       <c r="G4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="H4" s="26"/>
+      <c r="H4" s="26" t="s">
+        <v>334</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="16.5" customHeight="1">
       <c r="A5" s="8">
@@ -2277,7 +2636,9 @@
       <c r="G5" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="26"/>
+      <c r="H5" s="26" t="s">
+        <v>335</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="16.5" customHeight="1">
       <c r="A6" s="8">
@@ -2373,7 +2734,7 @@
         <v>50000</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>332</v>
+        <v>320</v>
       </c>
       <c r="H9" s="26"/>
     </row>
@@ -2390,10 +2751,10 @@
       <c r="D10" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="62">
+      <c r="E10" s="61">
         <v>80000</v>
       </c>
-      <c r="F10" s="62">
+      <c r="F10" s="61">
         <v>72000</v>
       </c>
       <c r="G10" s="8" t="s">
@@ -2423,7 +2784,7 @@
         <v>26000</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
       <c r="H11" s="26"/>
     </row>
@@ -2497,7 +2858,9 @@
       <c r="G14" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="H14" s="26"/>
+      <c r="H14" s="26" t="s">
+        <v>348</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="16.5" customHeight="1">
       <c r="A15" s="8">
@@ -2593,15 +2956,17 @@
       <c r="G18" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="H18" s="26"/>
+      <c r="H18" s="26" t="s">
+        <v>348</v>
+      </c>
     </row>
     <row r="19" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A19" s="69" t="s">
+      <c r="A19" s="71" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="67"/>
-      <c r="C19" s="67"/>
-      <c r="D19" s="68"/>
+      <c r="B19" s="69"/>
+      <c r="C19" s="69"/>
+      <c r="D19" s="70"/>
       <c r="E19" s="3">
         <f>SUM(E3:E18)</f>
         <v>831000</v>
@@ -2614,26 +2979,26 @@
       <c r="H19" s="26"/>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A21" s="65" t="s">
+      <c r="A21" s="67" t="s">
         <v>56</v>
       </c>
-      <c r="B21" s="64"/>
-      <c r="C21" s="64"/>
-      <c r="D21" s="64"/>
-      <c r="E21" s="64"/>
-      <c r="F21" s="64"/>
-      <c r="G21" s="64"/>
+      <c r="B21" s="66"/>
+      <c r="C21" s="66"/>
+      <c r="D21" s="66"/>
+      <c r="E21" s="66"/>
+      <c r="F21" s="66"/>
+      <c r="G21" s="66"/>
     </row>
     <row r="24" spans="1:8" ht="21" customHeight="1">
-      <c r="A24" s="63" t="s">
+      <c r="A24" s="65" t="s">
         <v>57</v>
       </c>
-      <c r="B24" s="64"/>
-      <c r="C24" s="64"/>
-      <c r="D24" s="64"/>
-      <c r="E24" s="64"/>
-      <c r="F24" s="64"/>
-      <c r="G24" s="64"/>
+      <c r="B24" s="66"/>
+      <c r="C24" s="66"/>
+      <c r="D24" s="66"/>
+      <c r="E24" s="66"/>
+      <c r="F24" s="66"/>
+      <c r="G24" s="66"/>
     </row>
     <row r="25" spans="1:8" ht="21" customHeight="1">
       <c r="A25" s="38" t="s">
@@ -2669,7 +3034,7 @@
         <v>28</v>
       </c>
       <c r="C26" s="50" t="s">
-        <v>338</v>
+        <v>325</v>
       </c>
       <c r="D26" s="35" t="s">
         <v>11</v>
@@ -2681,10 +3046,10 @@
         <v>11000</v>
       </c>
       <c r="G26" s="50" t="s">
-        <v>336</v>
+        <v>323</v>
       </c>
       <c r="H26" s="53" t="s">
-        <v>337</v>
+        <v>324</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="31.5" customHeight="1">
@@ -2750,7 +3115,7 @@
         <v>11</v>
       </c>
       <c r="H29" s="53" t="s">
-        <v>327</v>
+        <v>318</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="16.5" customHeight="1">
@@ -2788,13 +3153,17 @@
       <c r="D31" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="E31" s="39"/>
-      <c r="F31" s="39"/>
+      <c r="E31" s="39">
+        <v>33000</v>
+      </c>
+      <c r="F31" s="39">
+        <v>33000</v>
+      </c>
       <c r="G31" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="H31" s="53" t="s">
-        <v>328</v>
+      <c r="H31" s="90" t="s">
+        <v>357</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="30.75" customHeight="1">
@@ -2916,19 +3285,19 @@
       <c r="H37" s="53"/>
     </row>
     <row r="38" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A38" s="66" t="s">
+      <c r="A38" s="68" t="s">
         <v>73</v>
       </c>
-      <c r="B38" s="67"/>
-      <c r="C38" s="67"/>
-      <c r="D38" s="68"/>
+      <c r="B38" s="69"/>
+      <c r="C38" s="69"/>
+      <c r="D38" s="70"/>
       <c r="E38" s="41">
         <f>SUM(E26:E37)</f>
-        <v>11000</v>
+        <v>44000</v>
       </c>
       <c r="F38" s="41">
         <f>SUM(F26:F37)</f>
-        <v>11000</v>
+        <v>44000</v>
       </c>
       <c r="G38" s="40"/>
       <c r="H38" s="53"/>
@@ -2968,28 +3337,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="65" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1">
-      <c r="A3" s="71" t="s">
+      <c r="A3" s="73" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="67"/>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="68"/>
+      <c r="B3" s="69"/>
+      <c r="C3" s="69"/>
+      <c r="D3" s="69"/>
+      <c r="E3" s="69"/>
+      <c r="F3" s="69"/>
+      <c r="G3" s="69"/>
+      <c r="H3" s="70"/>
       <c r="I3" s="24"/>
     </row>
     <row r="4" spans="1:9" ht="33" customHeight="1">
@@ -3105,7 +3474,7 @@
         <v>90</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>335</v>
+        <v>322</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="26.25" customHeight="1">
@@ -3149,16 +3518,16 @@
       <c r="I9" s="13"/>
     </row>
     <row r="10" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A10" s="71" t="s">
+      <c r="A10" s="73" t="s">
         <v>94</v>
       </c>
-      <c r="B10" s="67"/>
-      <c r="C10" s="67"/>
-      <c r="D10" s="67"/>
-      <c r="E10" s="67"/>
-      <c r="F10" s="67"/>
-      <c r="G10" s="67"/>
-      <c r="H10" s="68"/>
+      <c r="B10" s="69"/>
+      <c r="C10" s="69"/>
+      <c r="D10" s="69"/>
+      <c r="E10" s="69"/>
+      <c r="F10" s="69"/>
+      <c r="G10" s="69"/>
+      <c r="H10" s="70"/>
       <c r="I10" s="24"/>
     </row>
     <row r="11" spans="1:9" ht="16.5" customHeight="1">
@@ -3366,16 +3735,16 @@
       <c r="I18" s="13"/>
     </row>
     <row r="19" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A19" s="71" t="s">
+      <c r="A19" s="73" t="s">
         <v>109</v>
       </c>
-      <c r="B19" s="67"/>
-      <c r="C19" s="67"/>
-      <c r="D19" s="67"/>
-      <c r="E19" s="67"/>
-      <c r="F19" s="67"/>
-      <c r="G19" s="67"/>
-      <c r="H19" s="68"/>
+      <c r="B19" s="69"/>
+      <c r="C19" s="69"/>
+      <c r="D19" s="69"/>
+      <c r="E19" s="69"/>
+      <c r="F19" s="69"/>
+      <c r="G19" s="69"/>
+      <c r="H19" s="70"/>
       <c r="I19" s="24"/>
     </row>
     <row r="20" spans="1:9" ht="16.5" customHeight="1">
@@ -3500,16 +3869,16 @@
       <c r="I24" s="13"/>
     </row>
     <row r="25" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A25" s="71" t="s">
+      <c r="A25" s="73" t="s">
         <v>117</v>
       </c>
-      <c r="B25" s="67"/>
-      <c r="C25" s="67"/>
-      <c r="D25" s="67"/>
-      <c r="E25" s="67"/>
-      <c r="F25" s="67"/>
-      <c r="G25" s="67"/>
-      <c r="H25" s="68"/>
+      <c r="B25" s="69"/>
+      <c r="C25" s="69"/>
+      <c r="D25" s="69"/>
+      <c r="E25" s="69"/>
+      <c r="F25" s="69"/>
+      <c r="G25" s="69"/>
+      <c r="H25" s="70"/>
       <c r="I25" s="24"/>
     </row>
     <row r="26" spans="1:9" ht="16.5" customHeight="1">
@@ -3565,7 +3934,7 @@
         <v>11</v>
       </c>
       <c r="I27" s="14" t="s">
-        <v>339</v>
+        <v>326</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="33" customHeight="1">
@@ -3596,45 +3965,45 @@
       </c>
     </row>
     <row r="29" spans="1:9" ht="33" customHeight="1">
-      <c r="A29" s="58" t="s">
+      <c r="A29" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="B29" s="58" t="s">
+      <c r="B29" s="57" t="s">
         <v>10</v>
       </c>
-      <c r="C29" s="58">
+      <c r="C29" s="57">
         <v>900</v>
       </c>
-      <c r="D29" s="58" t="s">
+      <c r="D29" s="57" t="s">
         <v>129</v>
       </c>
-      <c r="E29" s="58" t="s">
+      <c r="E29" s="57" t="s">
         <v>130</v>
       </c>
-      <c r="F29" s="59" t="s">
-        <v>342</v>
-      </c>
-      <c r="G29" s="58" t="s">
+      <c r="F29" s="58" t="s">
+        <v>329</v>
+      </c>
+      <c r="G29" s="57" t="s">
         <v>131</v>
       </c>
-      <c r="H29" s="60" t="s">
+      <c r="H29" s="59" t="s">
         <v>90</v>
       </c>
-      <c r="I29" s="61" t="s">
+      <c r="I29" s="60" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A32" s="70" t="s">
+      <c r="A32" s="72" t="s">
         <v>133</v>
       </c>
-      <c r="B32" s="64"/>
-      <c r="C32" s="64"/>
-      <c r="D32" s="64"/>
-      <c r="E32" s="64"/>
-      <c r="F32" s="64"/>
-      <c r="G32" s="64"/>
-      <c r="H32" s="64"/>
+      <c r="B32" s="66"/>
+      <c r="C32" s="66"/>
+      <c r="D32" s="66"/>
+      <c r="E32" s="66"/>
+      <c r="F32" s="66"/>
+      <c r="G32" s="66"/>
+      <c r="H32" s="66"/>
     </row>
     <row r="35" spans="1:9" ht="14.25" customHeight="1">
       <c r="A35" s="36" t="s">
@@ -3701,7 +4070,7 @@
         <v>85</v>
       </c>
       <c r="I38" s="52" t="s">
-        <v>138</v>
+        <v>354</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="16.5">
@@ -3712,25 +4081,25 @@
         <v>60</v>
       </c>
       <c r="C39" s="35" t="s">
+        <v>138</v>
+      </c>
+      <c r="D39" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="E39" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="F39" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="D39" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E39" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="F39" s="35" t="s">
+      <c r="G39" s="35" t="s">
         <v>140</v>
-      </c>
-      <c r="G39" s="35" t="s">
-        <v>141</v>
       </c>
       <c r="H39" s="42" t="s">
         <v>85</v>
       </c>
       <c r="I39" s="43" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="16.5">
@@ -3741,19 +4110,19 @@
         <v>62</v>
       </c>
       <c r="C40" s="35" t="s">
+        <v>142</v>
+      </c>
+      <c r="D40" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="E40" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="F40" s="35" t="s">
         <v>143</v>
       </c>
-      <c r="D40" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E40" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="F40" s="35" t="s">
+      <c r="G40" s="35" t="s">
         <v>144</v>
-      </c>
-      <c r="G40" s="35" t="s">
-        <v>145</v>
       </c>
       <c r="H40" s="44" t="s">
         <v>85</v>
@@ -3802,7 +4171,7 @@
         <v>11</v>
       </c>
       <c r="C44" s="35" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D44" s="35" t="s">
         <v>11</v>
@@ -3836,14 +4205,14 @@
         <v>11</v>
       </c>
       <c r="F45" s="35" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G45" s="35"/>
       <c r="H45" s="42" t="s">
         <v>90</v>
       </c>
       <c r="I45" s="43" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="46" spans="1:9" ht="16.5">
@@ -3854,7 +4223,7 @@
         <v>69</v>
       </c>
       <c r="C46" s="49" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
       <c r="D46" s="35" t="s">
         <v>11</v>
@@ -3872,12 +4241,12 @@
         <v>90</v>
       </c>
       <c r="I46" s="45" t="s">
-        <v>334</v>
+        <v>362</v>
       </c>
     </row>
     <row r="48" spans="1:9">
       <c r="A48" s="37" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="49" spans="1:9" ht="16.5">
@@ -3932,7 +4301,7 @@
         <v>11</v>
       </c>
       <c r="H50" s="42" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I50" s="43"/>
     </row>
@@ -3957,10 +4326,10 @@
       </c>
       <c r="G51" s="35"/>
       <c r="H51" s="42" t="s">
+        <v>148</v>
+      </c>
+      <c r="I51" s="43" t="s">
         <v>149</v>
-      </c>
-      <c r="I51" s="43" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="52" spans="1:9" ht="16.5">
@@ -3984,7 +4353,7 @@
       </c>
       <c r="G52" s="35"/>
       <c r="H52" s="42" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I52" s="43"/>
     </row>
@@ -3999,26 +4368,26 @@
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <conditionalFormatting sqref="H4:H9 H11:H13 H15:H16 H18 H20:H24 H26:H28">
-    <cfRule type="cellIs" dxfId="11" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="15" operator="equal">
       <formula>"✅"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="16" operator="equal">
       <formula>"⚠️"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H14">
-    <cfRule type="cellIs" dxfId="9" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="3" operator="equal">
       <formula>"✅"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="4" operator="equal">
       <formula>"⚠️"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H17">
-    <cfRule type="cellIs" dxfId="7" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="1" operator="equal">
       <formula>"✅"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="2" operator="equal">
       <formula>"⚠️"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4031,39 +4400,40 @@
   <sheetPr>
     <tabColor rgb="FF70AD47"/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="8" style="30" customWidth="1"/>
-    <col min="2" max="2" width="10" style="30" customWidth="1"/>
+    <col min="2" max="2" width="10.625" style="30" customWidth="1"/>
     <col min="3" max="3" width="14" style="30" customWidth="1"/>
     <col min="4" max="5" width="10" style="30" customWidth="1"/>
     <col min="6" max="6" width="18" style="30" customWidth="1"/>
+    <col min="8" max="8" width="23.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="63" t="s">
+    <row r="1" spans="1:8" ht="30" customHeight="1">
+      <c r="A1" s="65" t="s">
+        <v>152</v>
+      </c>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+    </row>
+    <row r="2" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A2" s="67" t="s">
         <v>153</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-    </row>
-    <row r="2" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A2" s="65" t="s">
-        <v>154</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-    </row>
-    <row r="3" spans="1:6" ht="15" customHeight="1">
+      <c r="B2" s="66"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
+    </row>
+    <row r="3" spans="1:8" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>387</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>2</v>
@@ -4072,38 +4442,38 @@
         <v>3</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>155</v>
+        <v>338</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>156</v>
+        <v>337</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A4" s="8" t="s">
-        <v>343</v>
-      </c>
-      <c r="B4" s="8" t="s">
+    <row r="4" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A4" s="57" t="s">
+        <v>330</v>
+      </c>
+      <c r="B4" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="57" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="8">
-        <v>50000</v>
-      </c>
-      <c r="E4" s="16" t="s">
-        <v>348</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="16.5" customHeight="1">
+      <c r="D4" s="57">
+        <v>0</v>
+      </c>
+      <c r="E4" s="82">
+        <v>0</v>
+      </c>
+      <c r="F4" s="57" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="16.5" customHeight="1">
       <c r="A5" s="8" t="s">
-        <v>14</v>
+        <v>381</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>12</v>
@@ -4111,498 +4481,755 @@
       <c r="C5" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="85">
+        <v>10000</v>
+      </c>
+      <c r="E5" s="85">
+        <v>10000</v>
+      </c>
+      <c r="F5" s="86" t="s">
+        <v>339</v>
+      </c>
+      <c r="H5" s="62" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A6" s="85" t="s">
+        <v>381</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="D6" s="85">
+        <v>20100</v>
+      </c>
+      <c r="E6" s="85">
+        <v>20100</v>
+      </c>
+      <c r="F6" s="86" t="s">
+        <v>342</v>
+      </c>
+      <c r="H6" s="62" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A7" s="85" t="s">
+        <v>364</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="87">
+        <v>16000</v>
+      </c>
+      <c r="E7" s="8">
+        <v>27000</v>
+      </c>
+      <c r="F7" s="86" t="s">
+        <v>340</v>
+      </c>
+      <c r="H7" s="62" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="62" customFormat="1" ht="16.5">
+      <c r="A8" s="95" t="s">
+        <v>386</v>
+      </c>
+      <c r="B8" s="95" t="s">
+        <v>372</v>
+      </c>
+      <c r="C8" s="98" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" s="98">
+        <v>20000</v>
+      </c>
+      <c r="E8" s="98">
+        <v>20000</v>
+      </c>
+      <c r="F8" s="95"/>
+    </row>
+    <row r="9" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A9" s="85" t="s">
+        <v>382</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" s="85">
+        <v>71000</v>
+      </c>
+      <c r="E9" s="85">
+        <v>71000</v>
+      </c>
+      <c r="F9" s="86" t="s">
+        <v>350</v>
+      </c>
+      <c r="H9" s="62" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" s="62" customFormat="1" ht="16.5" customHeight="1">
+      <c r="A10" s="95"/>
+      <c r="B10" s="63"/>
+      <c r="C10" s="63"/>
+      <c r="D10" s="95"/>
+      <c r="E10" s="63"/>
+      <c r="F10" s="86"/>
+      <c r="H10" s="84"/>
+    </row>
+    <row r="11" spans="1:8" s="62" customFormat="1" ht="16.5" customHeight="1">
+      <c r="A11" s="95"/>
+      <c r="B11" s="63"/>
+      <c r="C11" s="63"/>
+      <c r="D11" s="95"/>
+      <c r="E11" s="63"/>
+      <c r="F11" s="86"/>
+      <c r="H11" s="84"/>
+    </row>
+    <row r="12" spans="1:8" ht="32.25" customHeight="1">
+      <c r="A12" s="57" t="s">
+        <v>363</v>
+      </c>
+      <c r="B12" s="57" t="s">
+        <v>369</v>
+      </c>
+      <c r="C12" s="57" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="57">
         <v>0</v>
       </c>
-      <c r="E5" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F5" s="8"/>
-    </row>
-    <row r="6" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A6" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="8">
-        <v>27000</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F6" s="8"/>
-    </row>
-    <row r="7" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A7" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="8">
+      <c r="E12" s="57">
+        <v>46000</v>
+      </c>
+      <c r="F12" s="94" t="s">
+        <v>341</v>
+      </c>
+      <c r="H12" s="84"/>
+    </row>
+    <row r="13" spans="1:8" ht="33">
+      <c r="A13" s="95" t="s">
+        <v>366</v>
+      </c>
+      <c r="B13" s="63" t="s">
+        <v>367</v>
+      </c>
+      <c r="C13" s="63" t="s">
+        <v>377</v>
+      </c>
+      <c r="D13" s="35">
+        <v>46000</v>
+      </c>
+      <c r="E13" s="89">
+        <v>110000</v>
+      </c>
+      <c r="F13" s="51" t="s">
+        <v>365</v>
+      </c>
+      <c r="G13" s="83" t="s">
+        <v>356</v>
+      </c>
+      <c r="H13" s="92" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="101"/>
+      <c r="B14" s="101"/>
+      <c r="C14" s="101"/>
+      <c r="D14" s="101"/>
+      <c r="E14" s="101"/>
+      <c r="F14" s="101"/>
+    </row>
+    <row r="15" spans="1:8" s="62" customFormat="1" ht="16.5">
+      <c r="A15" s="95"/>
+      <c r="B15" s="95"/>
+      <c r="C15" s="95"/>
+      <c r="D15" s="98"/>
+      <c r="E15" s="100"/>
+      <c r="F15" s="95"/>
+      <c r="G15" s="91"/>
+      <c r="H15" s="92"/>
+    </row>
+    <row r="16" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A16" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="D16" s="87">
+        <v>60000</v>
+      </c>
+      <c r="E16" s="87">
+        <v>60000</v>
+      </c>
+      <c r="F16" s="86" t="s">
+        <v>342</v>
+      </c>
+      <c r="G16" s="83"/>
+      <c r="H16" s="97" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" s="62" customFormat="1" ht="16.5" customHeight="1">
+      <c r="A17" s="95"/>
+      <c r="B17" s="95"/>
+      <c r="C17" s="95"/>
+      <c r="D17" s="95"/>
+      <c r="E17" s="95"/>
+      <c r="F17" s="95"/>
+      <c r="G17" s="91"/>
+      <c r="H17" s="97"/>
+    </row>
+    <row r="18" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A18" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D18" s="8">
+        <v>7000</v>
+      </c>
+      <c r="E18" s="8">
+        <v>7000</v>
+      </c>
+      <c r="F18" s="86" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A19" s="81" t="s">
+        <v>320</v>
+      </c>
+      <c r="B19" s="81" t="s">
+        <v>376</v>
+      </c>
+      <c r="C19" s="81" t="s">
+        <v>48</v>
+      </c>
+      <c r="D19" s="81">
+        <v>0</v>
+      </c>
+      <c r="E19" s="81">
+        <v>5100</v>
+      </c>
+      <c r="F19" s="96" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="33">
+      <c r="A20" s="48" t="s">
+        <v>320</v>
+      </c>
+      <c r="B20" s="63" t="s">
+        <v>370</v>
+      </c>
+      <c r="C20" s="89" t="s">
+        <v>361</v>
+      </c>
+      <c r="D20" s="93">
+        <v>33000</v>
+      </c>
+      <c r="E20" s="93">
+        <v>33000</v>
+      </c>
+      <c r="F20" s="48" t="s">
+        <v>317</v>
+      </c>
+      <c r="G20" s="83" t="s">
+        <v>355</v>
+      </c>
+      <c r="H20" s="92" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" s="62" customFormat="1" ht="16.5">
+      <c r="A21" s="95"/>
+      <c r="B21" s="95"/>
+      <c r="C21" s="100"/>
+      <c r="D21" s="98"/>
+      <c r="E21" s="98"/>
+      <c r="F21" s="95"/>
+      <c r="G21" s="91"/>
+      <c r="H21" s="92"/>
+    </row>
+    <row r="22" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A22" s="8" t="s">
+        <v>319</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D22" s="87">
+        <v>26000</v>
+      </c>
+      <c r="E22" s="87">
+        <v>26000</v>
+      </c>
+      <c r="F22" s="86" t="s">
+        <v>345</v>
+      </c>
+      <c r="H22" s="62" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A23" s="8" t="s">
+        <v>384</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D23" s="85">
+        <v>19000</v>
+      </c>
+      <c r="E23" s="85">
+        <v>19000</v>
+      </c>
+      <c r="F23" s="63" t="s">
+        <v>346</v>
+      </c>
+      <c r="H23" s="62" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A24" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>368</v>
+      </c>
+      <c r="D24" s="8">
+        <v>16000</v>
+      </c>
+      <c r="E24" s="8">
+        <v>35000</v>
+      </c>
+      <c r="F24" s="63" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" s="62" customFormat="1" ht="16.5">
+      <c r="A25" s="63" t="s">
+        <v>331</v>
+      </c>
+      <c r="B25" s="63" t="s">
+        <v>373</v>
+      </c>
+      <c r="C25" s="64" t="s">
+        <v>60</v>
+      </c>
+      <c r="D25" s="93">
+        <v>13000</v>
+      </c>
+      <c r="E25" s="93">
+        <v>13000</v>
+      </c>
+      <c r="F25" s="64"/>
+    </row>
+    <row r="26" spans="1:8" s="62" customFormat="1" ht="16.5">
+      <c r="A26" s="63"/>
+      <c r="B26" s="63"/>
+      <c r="C26" s="64"/>
+      <c r="D26" s="98"/>
+      <c r="E26" s="98"/>
+      <c r="F26" s="64"/>
+    </row>
+    <row r="27" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A27" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="D27" s="87">
+        <v>50000</v>
+      </c>
+      <c r="E27" s="87">
+        <v>50000</v>
+      </c>
+      <c r="F27" s="86" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A28" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D28" s="87">
         <v>20000</v>
       </c>
-      <c r="E7" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A8" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="D8" s="8">
+      <c r="E28" s="87">
+        <v>20000</v>
+      </c>
+      <c r="F28" s="63" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" s="62" customFormat="1" ht="16.5" customHeight="1">
+      <c r="A29" s="63"/>
+      <c r="B29" s="63"/>
+      <c r="C29" s="63"/>
+      <c r="D29" s="95"/>
+      <c r="E29" s="95"/>
+      <c r="F29" s="95"/>
+    </row>
+    <row r="30" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A30" s="57" t="s">
+        <v>51</v>
+      </c>
+      <c r="B30" s="57" t="s">
+        <v>371</v>
+      </c>
+      <c r="C30" s="57" t="s">
+        <v>50</v>
+      </c>
+      <c r="D30" s="57">
+        <v>0</v>
+      </c>
+      <c r="E30" s="57">
+        <v>0</v>
+      </c>
+      <c r="F30" s="94" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="18" customHeight="1">
+      <c r="A31" s="99" t="s">
+        <v>379</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D31" s="87">
         <v>60000</v>
       </c>
-      <c r="E8" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F8" s="8"/>
-    </row>
-    <row r="9" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A9" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="8">
+      <c r="E31" s="87">
+        <v>60000</v>
+      </c>
+      <c r="F31" s="86" t="s">
+        <v>352</v>
+      </c>
+      <c r="H31" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="16.5">
+      <c r="A32" s="88"/>
+      <c r="B32" s="86" t="s">
+        <v>353</v>
+      </c>
+      <c r="C32" s="88"/>
+      <c r="D32" s="88">
+        <f>SUM(D4:D31)</f>
+        <v>487100</v>
+      </c>
+      <c r="E32" s="88">
+        <f>SUM(E4:E31)</f>
+        <v>632200</v>
+      </c>
+      <c r="F32" s="88"/>
+    </row>
+    <row r="33" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A33" s="67" t="s">
+        <v>154</v>
+      </c>
+      <c r="B33" s="66"/>
+      <c r="C33" s="66"/>
+      <c r="D33" s="66"/>
+      <c r="E33" s="66"/>
+      <c r="F33" s="66"/>
+    </row>
+    <row r="36" spans="1:8" ht="14.25">
+      <c r="A36" s="36" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="15">
+      <c r="A37" s="38" t="s">
+        <v>7</v>
+      </c>
+      <c r="B37" s="38" t="s">
+        <v>2</v>
+      </c>
+      <c r="C37" s="38" t="s">
+        <v>3</v>
+      </c>
+      <c r="D37" s="15" t="s">
+        <v>338</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="F37" s="38" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="16.5">
+      <c r="A38" s="95" t="s">
+        <v>386</v>
+      </c>
+      <c r="B38" s="95" t="s">
+        <v>372</v>
+      </c>
+      <c r="C38" s="35" t="s">
+        <v>62</v>
+      </c>
+      <c r="D38" s="93">
         <v>20000</v>
       </c>
-      <c r="E9" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A10" s="8" t="s">
+      <c r="E38" s="93">
+        <v>20000</v>
+      </c>
+      <c r="F38" s="63"/>
+    </row>
+    <row r="39" spans="1:8" s="62" customFormat="1" ht="33">
+      <c r="A39" s="95" t="s">
+        <v>366</v>
+      </c>
+      <c r="B39" s="63" t="s">
+        <v>367</v>
+      </c>
+      <c r="C39" s="64" t="s">
+        <v>58</v>
+      </c>
+      <c r="D39" s="64">
+        <v>46000</v>
+      </c>
+      <c r="E39" s="89">
+        <v>110000</v>
+      </c>
+      <c r="F39" s="63" t="s">
+        <v>365</v>
+      </c>
+      <c r="G39" s="83" t="s">
+        <v>356</v>
+      </c>
+      <c r="H39" s="92" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" s="62" customFormat="1" ht="33">
+      <c r="A40" s="63" t="s">
+        <v>320</v>
+      </c>
+      <c r="B40" s="63" t="s">
+        <v>370</v>
+      </c>
+      <c r="C40" s="89" t="s">
+        <v>361</v>
+      </c>
+      <c r="D40" s="93">
+        <v>33000</v>
+      </c>
+      <c r="E40" s="93">
+        <v>33000</v>
+      </c>
+      <c r="F40" s="63" t="s">
+        <v>317</v>
+      </c>
+      <c r="G40" s="83" t="s">
+        <v>355</v>
+      </c>
+      <c r="H40" s="92" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="16.5">
+      <c r="A41" s="51" t="s">
+        <v>331</v>
+      </c>
+      <c r="B41" s="63" t="s">
+        <v>373</v>
+      </c>
+      <c r="C41" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="D41" s="93">
+        <v>13000</v>
+      </c>
+      <c r="E41" s="93">
+        <v>13000</v>
+      </c>
+      <c r="F41" s="35"/>
+    </row>
+    <row r="42" spans="1:8" ht="16.5">
+      <c r="A42" s="51" t="s">
+        <v>333</v>
+      </c>
+      <c r="B42" s="63" t="s">
+        <v>374</v>
+      </c>
+      <c r="C42" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="D42" s="35"/>
+      <c r="E42" s="35"/>
+      <c r="F42" s="63" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="16.5">
+      <c r="A43" s="51" t="s">
         <v>332</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="D10" s="8">
-        <v>30000</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F10" s="8"/>
-    </row>
-    <row r="11" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A11" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="D11" s="8">
-        <v>20000</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F11" s="8"/>
-    </row>
-    <row r="12" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A12" s="8" t="s">
-        <v>331</v>
-      </c>
-      <c r="B12" s="8" t="s">
+      <c r="B43" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D12" s="8">
-        <v>30000</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F12" s="8"/>
-    </row>
-    <row r="13" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A13" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="D13" s="8">
-        <v>19000</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F13" s="8"/>
-    </row>
-    <row r="14" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A14" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14" s="8">
-        <v>0</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A15" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B15" s="8" t="s">
+      <c r="C43" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="D43" s="35"/>
+      <c r="E43" s="35"/>
+      <c r="F43" s="63" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="16.5">
+      <c r="A44" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="B44" s="35" t="s">
+        <v>44</v>
+      </c>
+      <c r="C44" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="D44" s="35"/>
+      <c r="E44" s="35"/>
+      <c r="F44" s="35"/>
+    </row>
+    <row r="45" spans="1:8" ht="16.5">
+      <c r="A45" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="B45" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="C45" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="D45" s="35"/>
+      <c r="E45" s="35"/>
+      <c r="F45" s="35"/>
+    </row>
+    <row r="46" spans="1:8" ht="16.5">
+      <c r="A46" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="B46" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="D15" s="8">
-        <v>50000</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F15" s="8"/>
-    </row>
-    <row r="16" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A16" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D16" s="8">
-        <v>20000</v>
-      </c>
-      <c r="E16" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F16" s="8"/>
-    </row>
-    <row r="17" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A17" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="D17" s="8">
-        <v>71000</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F17" s="8"/>
-    </row>
-    <row r="18" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A18" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="D18" s="8">
-        <v>0</v>
-      </c>
-      <c r="E18" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A19" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="D19" s="8">
-        <v>60000</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="F19" s="8"/>
-    </row>
-    <row r="21" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A21" s="65" t="s">
-        <v>159</v>
-      </c>
-      <c r="B21" s="64"/>
-      <c r="C21" s="64"/>
-      <c r="D21" s="64"/>
-      <c r="E21" s="64"/>
-      <c r="F21" s="64"/>
-    </row>
-    <row r="24" spans="1:6" ht="14.25">
-      <c r="A24" s="36" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="15">
-      <c r="A25" s="38" t="s">
-        <v>7</v>
-      </c>
-      <c r="B25" s="38" t="s">
-        <v>2</v>
-      </c>
-      <c r="C25" s="38" t="s">
-        <v>3</v>
-      </c>
-      <c r="D25" s="38" t="s">
-        <v>155</v>
-      </c>
-      <c r="E25" s="38" t="s">
-        <v>156</v>
-      </c>
-      <c r="F25" s="38" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="33">
-      <c r="A26" s="48" t="s">
-        <v>332</v>
-      </c>
-      <c r="B26" s="35" t="s">
-        <v>28</v>
-      </c>
-      <c r="C26" s="35" t="s">
-        <v>58</v>
-      </c>
-      <c r="D26" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E26" s="57" t="s">
-        <v>157</v>
-      </c>
-      <c r="F26" s="51" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="16.5">
-      <c r="A27" s="51" t="s">
-        <v>345</v>
-      </c>
-      <c r="B27" s="35" t="s">
-        <v>59</v>
-      </c>
-      <c r="C27" s="35" t="s">
-        <v>60</v>
-      </c>
-      <c r="D27" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E27" s="35" t="s">
-        <v>157</v>
-      </c>
-      <c r="F27" s="35" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="33">
-      <c r="A28" s="48" t="s">
-        <v>324</v>
-      </c>
-      <c r="B28" s="35" t="s">
-        <v>41</v>
-      </c>
-      <c r="C28" s="35" t="s">
-        <v>62</v>
-      </c>
-      <c r="D28" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E28" s="35" t="s">
-        <v>157</v>
-      </c>
-      <c r="F28" s="35" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="16.5">
-      <c r="A29" s="48" t="s">
-        <v>325</v>
-      </c>
-      <c r="B29" s="35" t="s">
-        <v>18</v>
-      </c>
-      <c r="C29" s="35" t="s">
-        <v>69</v>
-      </c>
-      <c r="D29" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E29" s="35" t="s">
-        <v>157</v>
-      </c>
-      <c r="F29" s="48" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="16.5">
-      <c r="A30" s="51" t="s">
-        <v>347</v>
-      </c>
-      <c r="B30" s="35" t="s">
-        <v>64</v>
-      </c>
-      <c r="C30" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="D30" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E30" s="35" t="s">
-        <v>157</v>
-      </c>
-      <c r="F30" s="35" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="16.5">
-      <c r="A31" s="51" t="s">
-        <v>346</v>
-      </c>
-      <c r="B31" s="35" t="s">
-        <v>40</v>
-      </c>
-      <c r="C31" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="D31" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E31" s="35" t="s">
-        <v>157</v>
-      </c>
-      <c r="F31" s="35" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="16.5">
-      <c r="A32" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="B32" s="35" t="s">
-        <v>44</v>
-      </c>
-      <c r="C32" s="35" t="s">
-        <v>45</v>
-      </c>
-      <c r="D32" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E32" s="35" t="s">
-        <v>157</v>
-      </c>
-      <c r="F32" s="35" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="16.5">
-      <c r="A33" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="B33" s="35" t="s">
-        <v>67</v>
-      </c>
-      <c r="C33" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="D33" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E33" s="35" t="s">
-        <v>157</v>
-      </c>
-      <c r="F33" s="35" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="16.5">
-      <c r="A34" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="B34" s="35" t="s">
-        <v>38</v>
-      </c>
-      <c r="C34" s="35" t="s">
+      <c r="C46" s="35" t="s">
         <v>71</v>
       </c>
-      <c r="D34" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E34" s="35" t="s">
-        <v>157</v>
-      </c>
-      <c r="F34" s="35" t="s">
-        <v>152</v>
-      </c>
+      <c r="D46" s="35"/>
+      <c r="E46" s="35"/>
+      <c r="F46" s="35"/>
+    </row>
+    <row r="47" spans="1:8" ht="16.5">
+      <c r="A47" s="88"/>
+      <c r="B47" s="86" t="s">
+        <v>353</v>
+      </c>
+      <c r="C47" s="88"/>
+      <c r="D47" s="88">
+        <f>SUM(D13:D46)</f>
+        <v>949100</v>
+      </c>
+      <c r="E47" s="88">
+        <f>SUM(E13:E46)</f>
+        <v>1246300</v>
+      </c>
+      <c r="F47" s="88"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A33:F33"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
-  <conditionalFormatting sqref="D4:D19">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+  <conditionalFormatting sqref="D4 D12 D18:D19 D10:E11 D27:D31 D22:E22 D5:E7 D9 D23:D24">
+    <cfRule type="cellIs" dxfId="13" priority="9" operator="equal">
+      <formula>"✅"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E18">
+    <cfRule type="cellIs" dxfId="12" priority="7" operator="equal">
+      <formula>"✅"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E19">
+    <cfRule type="cellIs" dxfId="11" priority="6" operator="equal">
+      <formula>"✅"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E23">
+    <cfRule type="cellIs" dxfId="10" priority="5" operator="equal">
+      <formula>"✅"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E27">
+    <cfRule type="cellIs" dxfId="9" priority="4" operator="equal">
+      <formula>"✅"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E28:E29">
+    <cfRule type="cellIs" dxfId="8" priority="3" operator="equal">
+      <formula>"✅"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E9">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+      <formula>"✅"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E31">
+    <cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
       <formula>"✅"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4616,7 +5243,7 @@
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="10" style="30" customWidth="1"/>
@@ -4628,53 +5255,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="63" t="s">
-        <v>164</v>
-      </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
+      <c r="A1" s="65" t="s">
+        <v>157</v>
+      </c>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
-      <c r="A3" s="72" t="s">
-        <v>165</v>
-      </c>
-      <c r="B3" s="64"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
+      <c r="A3" s="74" t="s">
+        <v>158</v>
+      </c>
+      <c r="B3" s="66"/>
+      <c r="C3" s="66"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="66"/>
+      <c r="F3" s="66"/>
+      <c r="G3" s="66"/>
+      <c r="H3" s="66"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="16.5" customHeight="1">
@@ -4682,7 +5309,7 @@
         <v>41</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="C5" s="8">
         <v>3</v>
@@ -4694,13 +5321,13 @@
         <v>3</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="33" customHeight="1">
@@ -4708,7 +5335,7 @@
         <v>41</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="C6" s="8">
         <v>5</v>
@@ -4720,13 +5347,13 @@
         <v>5</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="16.5" customHeight="1">
@@ -4734,7 +5361,7 @@
         <v>35</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="C7" s="8">
         <v>6</v>
@@ -4746,13 +5373,13 @@
         <v>6</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="16.5" customHeight="1">
@@ -4760,7 +5387,7 @@
         <v>35</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="C8" s="8">
         <v>2</v>
@@ -4772,13 +5399,13 @@
         <v>2</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="33" customHeight="1">
@@ -4786,7 +5413,7 @@
         <v>35</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="C9" s="8">
         <v>4</v>
@@ -4798,13 +5425,13 @@
         <v>4</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="33" customHeight="1">
@@ -4812,7 +5439,7 @@
         <v>35</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="C10" s="35">
         <v>6</v>
@@ -4824,13 +5451,13 @@
         <v>6</v>
       </c>
       <c r="F10" s="35" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="G10" s="35" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="H10" s="35" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="16.5" customHeight="1">
@@ -4838,7 +5465,7 @@
         <v>49</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="C11" s="8">
         <v>6</v>
@@ -4850,13 +5477,13 @@
         <v>6</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="33" customHeight="1">
@@ -4864,7 +5491,7 @@
         <v>49</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="C12" s="8">
         <v>1</v>
@@ -4876,10 +5503,10 @@
         <v>1</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>11</v>
@@ -4887,28 +5514,28 @@
     </row>
     <row r="13" spans="1:8" ht="33" customHeight="1">
       <c r="A13" s="8" t="s">
-        <v>9</v>
+        <v>336</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="C13" s="8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D13" s="8">
         <v>0</v>
       </c>
       <c r="E13" s="8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="16.5" customHeight="1">
@@ -4916,7 +5543,7 @@
         <v>9</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="C14" s="8">
         <v>2</v>
@@ -4928,13 +5555,13 @@
         <v>2</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="16.5" customHeight="1">
@@ -4942,104 +5569,98 @@
         <v>32</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="D15" s="8">
         <v>0</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="G15" s="8" t="s">
         <v>11</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A16" s="73" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16" s="67"/>
-      <c r="C16" s="67"/>
-      <c r="D16" s="67"/>
-      <c r="E16" s="68"/>
-      <c r="F16" s="73" t="s">
-        <v>178</v>
-      </c>
-      <c r="G16" s="68"/>
-      <c r="H16" s="8" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A17" s="74" t="s">
-        <v>205</v>
-      </c>
-      <c r="B17" s="68"/>
-      <c r="C17">
+      <c r="A16" s="76" t="s">
+        <v>198</v>
+      </c>
+      <c r="B16" s="80"/>
+      <c r="C16" s="8">
         <f>SUM(C5:C15)</f>
-        <v>39</v>
-      </c>
-      <c r="D17">
+        <v>35</v>
+      </c>
+      <c r="D16" s="8">
         <f>SUM(D5:D15)</f>
         <v>0</v>
       </c>
-      <c r="E17">
+      <c r="E16" s="8">
         <f>SUM(E5:E15)</f>
-        <v>39</v>
-      </c>
-      <c r="F17" s="74" t="s">
-        <v>206</v>
-      </c>
-      <c r="G17" s="68"/>
-      <c r="H17" s="21"/>
+        <v>35</v>
+      </c>
+      <c r="F16" s="76" t="s">
+        <v>199</v>
+      </c>
+      <c r="G16" s="80"/>
+      <c r="H16" s="21"/>
+    </row>
+    <row r="17" spans="1:8" ht="15" customHeight="1">
+      <c r="A17" s="66"/>
+      <c r="B17" s="66"/>
+      <c r="C17" s="66"/>
+      <c r="D17" s="66"/>
+      <c r="E17" s="66"/>
+      <c r="F17" s="66"/>
+      <c r="G17" s="66"/>
+      <c r="H17" s="66"/>
     </row>
     <row r="18" spans="1:8" ht="15" customHeight="1">
-      <c r="A18" s="64"/>
-      <c r="B18" s="64"/>
-      <c r="C18" s="64"/>
-      <c r="D18" s="64"/>
-      <c r="E18" s="64"/>
-      <c r="F18" s="64"/>
-      <c r="G18" s="64"/>
-      <c r="H18" s="64"/>
-    </row>
-    <row r="19" spans="1:8" ht="15" customHeight="1">
-      <c r="A19" s="33" t="s">
-        <v>207</v>
-      </c>
+      <c r="A18" s="33" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A19" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="H19" s="1"/>
     </row>
     <row r="20" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A20" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="H20" s="1"/>
+      <c r="A20" s="8"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
     </row>
     <row r="21" spans="1:8" ht="16.5" customHeight="1">
       <c r="A21" s="8"/>
@@ -5131,48 +5752,67 @@
       <c r="G29" s="8"/>
       <c r="H29" s="8"/>
     </row>
-    <row r="30" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A30" s="8"/>
-      <c r="B30" s="8"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
-      <c r="F30" s="8"/>
-      <c r="G30" s="8"/>
-      <c r="H30" s="8"/>
-    </row>
-    <row r="33" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A33" s="29" t="s">
+    <row r="32" spans="1:8" ht="14.25" customHeight="1">
+      <c r="A32" s="29" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="15">
+      <c r="A33" s="38" t="s">
+        <v>2</v>
+      </c>
+      <c r="B33" s="38" t="s">
+        <v>3</v>
+      </c>
+      <c r="C33" s="38" t="s">
+        <v>206</v>
+      </c>
+      <c r="D33" s="38" t="s">
+        <v>207</v>
+      </c>
+      <c r="E33" s="38" t="s">
+        <v>208</v>
+      </c>
+      <c r="F33" s="38" t="s">
+        <v>162</v>
+      </c>
+      <c r="G33" s="38" t="s">
+        <v>209</v>
+      </c>
+      <c r="H33" s="38" t="s">
+        <v>210</v>
+      </c>
+      <c r="I33" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="33">
+      <c r="A34" s="35" t="s">
+        <v>28</v>
+      </c>
+      <c r="B34" s="35" t="s">
+        <v>58</v>
+      </c>
+      <c r="C34" s="35" t="s">
+        <v>211</v>
+      </c>
+      <c r="D34" s="35">
+        <v>4</v>
+      </c>
+      <c r="E34" s="35">
+        <v>0</v>
+      </c>
+      <c r="F34" s="35">
+        <v>4</v>
+      </c>
+      <c r="G34" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="H34" s="35" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" ht="15">
-      <c r="A34" s="38" t="s">
-        <v>2</v>
-      </c>
-      <c r="B34" s="38" t="s">
-        <v>3</v>
-      </c>
-      <c r="C34" s="38" t="s">
+      <c r="I34" t="s">
         <v>213</v>
-      </c>
-      <c r="D34" s="38" t="s">
-        <v>214</v>
-      </c>
-      <c r="E34" s="38" t="s">
-        <v>215</v>
-      </c>
-      <c r="F34" s="38" t="s">
-        <v>169</v>
-      </c>
-      <c r="G34" s="38" t="s">
-        <v>216</v>
-      </c>
-      <c r="H34" s="38" t="s">
-        <v>217</v>
-      </c>
-      <c r="I34" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="33">
@@ -5183,54 +5823,51 @@
         <v>58</v>
       </c>
       <c r="C35" s="35" t="s">
-        <v>218</v>
-      </c>
-      <c r="D35" s="35">
-        <v>4</v>
-      </c>
-      <c r="E35" s="35">
+        <v>214</v>
+      </c>
+      <c r="D35" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="E35" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="F35" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="G35" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="H35" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="I35" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="16.5">
+      <c r="A36" s="35" t="s">
+        <v>59</v>
+      </c>
+      <c r="B36" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="C36" s="35" t="s">
+        <v>174</v>
+      </c>
+      <c r="D36" s="35">
+        <v>6</v>
+      </c>
+      <c r="E36" s="35">
         <v>0</v>
       </c>
-      <c r="F35" s="35">
-        <v>4</v>
-      </c>
-      <c r="G35" s="35" t="s">
-        <v>178</v>
-      </c>
-      <c r="H35" s="35" t="s">
-        <v>219</v>
-      </c>
-      <c r="I35" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" ht="33">
-      <c r="A36" s="35" t="s">
-        <v>28</v>
-      </c>
-      <c r="B36" s="35" t="s">
-        <v>58</v>
-      </c>
-      <c r="C36" s="35" t="s">
-        <v>221</v>
-      </c>
-      <c r="D36" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E36" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="F36" s="35" t="s">
-        <v>11</v>
+      <c r="F36" s="35">
+        <v>6</v>
       </c>
       <c r="G36" s="35" t="s">
-        <v>11</v>
+        <v>171</v>
       </c>
       <c r="H36" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="I36" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="16.5">
@@ -5241,51 +5878,51 @@
         <v>60</v>
       </c>
       <c r="C37" s="35" t="s">
-        <v>181</v>
+        <v>217</v>
       </c>
       <c r="D37" s="35">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E37" s="35">
         <v>0</v>
       </c>
       <c r="F37" s="35">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G37" s="35" t="s">
-        <v>178</v>
+        <v>11</v>
       </c>
       <c r="H37" s="35" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" ht="16.5">
+        <v>218</v>
+      </c>
+      <c r="I37" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="33">
       <c r="A38" s="35" t="s">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="B38" s="35" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C38" s="35" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="D38" s="35">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E38" s="35">
         <v>0</v>
       </c>
       <c r="F38" s="35">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="G38" s="35" t="s">
-        <v>11</v>
+        <v>186</v>
       </c>
       <c r="H38" s="35" t="s">
-        <v>225</v>
-      </c>
-      <c r="I38" t="s">
-        <v>226</v>
+        <v>85</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="33">
@@ -5296,22 +5933,25 @@
         <v>62</v>
       </c>
       <c r="C39" s="35" t="s">
-        <v>227</v>
+        <v>174</v>
       </c>
       <c r="D39" s="35">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E39" s="35">
         <v>0</v>
       </c>
       <c r="F39" s="35">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G39" s="35" t="s">
-        <v>193</v>
+        <v>171</v>
       </c>
       <c r="H39" s="35" t="s">
-        <v>85</v>
+        <v>216</v>
+      </c>
+      <c r="I39" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="33">
@@ -5322,65 +5962,39 @@
         <v>62</v>
       </c>
       <c r="C40" s="35" t="s">
-        <v>181</v>
+        <v>222</v>
       </c>
       <c r="D40" s="35">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E40" s="35">
         <v>0</v>
       </c>
       <c r="F40" s="35">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G40" s="35" t="s">
-        <v>178</v>
+        <v>11</v>
       </c>
       <c r="H40" s="35" t="s">
-        <v>223</v>
-      </c>
-      <c r="I40" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" ht="33">
-      <c r="A41" s="35" t="s">
-        <v>41</v>
-      </c>
-      <c r="B41" s="35" t="s">
-        <v>62</v>
-      </c>
-      <c r="C41" s="35" t="s">
-        <v>229</v>
-      </c>
-      <c r="D41" s="35">
-        <v>6</v>
-      </c>
-      <c r="E41" s="35">
-        <v>0</v>
-      </c>
-      <c r="F41" s="35">
-        <v>6</v>
-      </c>
-      <c r="G41" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="H41" s="35" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A18:H18"/>
+  <mergeCells count="5">
+    <mergeCell ref="A17:H17"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A16:B16"/>
     <mergeCell ref="F16:G16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="F17:G17"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <conditionalFormatting sqref="E5:E15">
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
+      <formula>"0"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E16">
     <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
       <formula>"0"</formula>
     </cfRule>
@@ -5404,147 +6018,147 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="63" t="s">
-        <v>230</v>
-      </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
+      <c r="A1" s="65" t="s">
+        <v>223</v>
+      </c>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
-      <c r="A3" s="72" t="s">
-        <v>231</v>
-      </c>
-      <c r="B3" s="64"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
+      <c r="A3" s="74" t="s">
+        <v>224</v>
+      </c>
+      <c r="B3" s="66"/>
+      <c r="C3" s="66"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="66"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="49.5" customHeight="1">
       <c r="A5" s="8" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>47</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="33" customHeight="1">
       <c r="A6" s="8" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="B6" s="8" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="33" customHeight="1">
       <c r="A7" s="8" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>25</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="33" customHeight="1">
       <c r="A8" s="8" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
-      <c r="A11" s="72" t="s">
-        <v>251</v>
-      </c>
-      <c r="B11" s="64"/>
-      <c r="C11" s="64"/>
-      <c r="D11" s="64"/>
-      <c r="E11" s="64"/>
-      <c r="F11" s="64"/>
-      <c r="G11" s="64"/>
-      <c r="H11" s="64"/>
+      <c r="A11" s="74" t="s">
+        <v>244</v>
+      </c>
+      <c r="B11" s="66"/>
+      <c r="C11" s="66"/>
+      <c r="D11" s="66"/>
+      <c r="E11" s="66"/>
+      <c r="F11" s="66"/>
+      <c r="G11" s="66"/>
+      <c r="H11" s="66"/>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="16.5" customHeight="1">
@@ -5675,24 +6289,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="63" t="s">
-        <v>258</v>
-      </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
+      <c r="A1" s="65" t="s">
+        <v>251</v>
+      </c>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1">
-      <c r="A3" s="72" t="s">
-        <v>259</v>
-      </c>
-      <c r="B3" s="64"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
+      <c r="A3" s="74" t="s">
+        <v>252</v>
+      </c>
+      <c r="B3" s="66"/>
+      <c r="C3" s="66"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="66"/>
+      <c r="F3" s="66"/>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1">
       <c r="A4" s="5" t="s">
@@ -5702,13 +6316,13 @@
         <v>3</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>82</v>
@@ -5725,7 +6339,7 @@
         <v>480</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="E5" s="8">
         <v>480</v>
@@ -5745,7 +6359,7 @@
         <v>500</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="E6" s="8">
         <v>500</v>
@@ -5765,7 +6379,7 @@
         <v>900</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="E7" s="8">
         <v>900</v>
@@ -5775,21 +6389,21 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A8" s="76" t="s">
+      <c r="A8" s="78" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="68"/>
+      <c r="B8" s="70"/>
       <c r="C8" s="35">
         <v>500</v>
       </c>
       <c r="D8" s="35" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="E8" s="35" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="35" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="16.5" customHeight="1">
@@ -5803,7 +6417,7 @@
         <v>1800</v>
       </c>
       <c r="D9" s="35" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="E9" s="35" t="s">
         <v>11</v>
@@ -5813,18 +6427,18 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1">
-      <c r="A10" s="75"/>
-      <c r="B10" s="67"/>
-      <c r="C10" s="67"/>
-      <c r="D10" s="67"/>
-      <c r="E10" s="67"/>
-      <c r="F10" s="68"/>
+      <c r="A10" s="77"/>
+      <c r="B10" s="69"/>
+      <c r="C10" s="69"/>
+      <c r="D10" s="69"/>
+      <c r="E10" s="69"/>
+      <c r="F10" s="70"/>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1">
-      <c r="A11" s="74" t="s">
-        <v>205</v>
-      </c>
-      <c r="B11" s="68"/>
+      <c r="A11" s="76" t="s">
+        <v>198</v>
+      </c>
+      <c r="B11" s="70"/>
       <c r="C11" s="34">
         <f>SUM(C5:C9)</f>
         <v>4180</v>
@@ -5839,18 +6453,18 @@
     <row r="12" spans="1:6" ht="16.5" customHeight="1"/>
     <row r="13" spans="1:6" ht="16.5" customHeight="1">
       <c r="A13" s="33" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16.5" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>11</v>
@@ -5864,10 +6478,10 @@
     </row>
     <row r="15" spans="1:6" ht="16.5" customHeight="1">
       <c r="A15" s="8" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="C15" s="8">
         <v>0</v>
@@ -5875,7 +6489,7 @@
     </row>
     <row r="16" spans="1:6" ht="16.5" customHeight="1">
       <c r="A16" s="8" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="B16" s="8" t="s">
         <v>11</v>
@@ -5885,21 +6499,21 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="15" customHeight="1">
-      <c r="A17" s="73" t="s">
-        <v>273</v>
-      </c>
-      <c r="B17" s="67"/>
-      <c r="C17" s="67"/>
-      <c r="D17" s="67"/>
-      <c r="E17" s="67"/>
-      <c r="F17" s="68"/>
+      <c r="A17" s="75" t="s">
+        <v>266</v>
+      </c>
+      <c r="B17" s="69"/>
+      <c r="C17" s="69"/>
+      <c r="D17" s="69"/>
+      <c r="E17" s="69"/>
+      <c r="F17" s="70"/>
     </row>
     <row r="18" spans="1:6" ht="15" customHeight="1">
       <c r="A18" s="11" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="C18" s="11">
         <v>0</v>
@@ -5911,15 +6525,15 @@
     <row r="19" spans="1:6" ht="16.5" customHeight="1"/>
     <row r="20" spans="1:6" ht="16.5" customHeight="1">
       <c r="A20" s="33" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="16.5" customHeight="1">
       <c r="A21" s="1" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>11</v>
@@ -5936,38 +6550,38 @@
     </row>
     <row r="22" spans="1:6" ht="16.5" customHeight="1">
       <c r="A22" s="22" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A23" s="73" t="s">
-        <v>171</v>
-      </c>
-      <c r="B23" s="67"/>
-      <c r="C23" s="67"/>
-      <c r="D23" s="67"/>
-      <c r="E23" s="67"/>
-      <c r="F23" s="68"/>
+      <c r="A23" s="75" t="s">
+        <v>164</v>
+      </c>
+      <c r="B23" s="69"/>
+      <c r="C23" s="69"/>
+      <c r="D23" s="69"/>
+      <c r="E23" s="69"/>
+      <c r="F23" s="70"/>
     </row>
     <row r="24" spans="1:6" ht="16.5" customHeight="1">
       <c r="A24" s="8" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="15.75" customHeight="1">
       <c r="A26" s="31" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="14.25" customHeight="1">
       <c r="A29" s="29" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="15">
@@ -5978,13 +6592,13 @@
         <v>3</v>
       </c>
       <c r="C30" s="46" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="D30" s="46" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="E30" s="46" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="F30" s="46" t="s">
         <v>82</v>
@@ -6001,13 +6615,13 @@
         <v>980</v>
       </c>
       <c r="D31" s="35" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="E31" s="35" t="s">
         <v>11</v>
       </c>
       <c r="F31" s="35" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="16.5">
@@ -6021,13 +6635,13 @@
         <v>500</v>
       </c>
       <c r="D32" s="35" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="E32" s="35" t="s">
         <v>11</v>
       </c>
       <c r="F32" s="35" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="16.5">
@@ -6041,13 +6655,13 @@
         <v>580</v>
       </c>
       <c r="D33" s="35" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="E33" s="35" t="s">
         <v>11</v>
       </c>
       <c r="F33" s="35" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="16.5">
@@ -6061,13 +6675,13 @@
         <v>11</v>
       </c>
       <c r="D34" s="35" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="E34" s="35" t="s">
         <v>11</v>
       </c>
       <c r="F34" s="35" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="16.5">
@@ -6081,7 +6695,7 @@
         <v>11</v>
       </c>
       <c r="D35" s="35" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="E35" s="35" t="s">
         <v>11</v>
@@ -6122,28 +6736,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="63" t="s">
-        <v>289</v>
-      </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
+      <c r="A1" s="65" t="s">
+        <v>282</v>
+      </c>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" s="65" t="s">
-        <v>290</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
+      <c r="A2" s="67" t="s">
+        <v>283</v>
+      </c>
+      <c r="B2" s="66"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -6153,22 +6767,22 @@
         <v>3</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>78</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="16.5" customHeight="1">
@@ -6179,7 +6793,7 @@
         <v>42</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>11</v>
@@ -6205,7 +6819,7 @@
         <v>36</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>11</v>
@@ -6231,7 +6845,7 @@
         <v>48</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>11</v>
@@ -6257,7 +6871,7 @@
         <v>33</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>11</v>
@@ -6283,7 +6897,7 @@
         <v>19</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>11</v>
@@ -6295,7 +6909,7 @@
         <v>11</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="H8" s="8" t="s">
         <v>11</v>
@@ -6309,7 +6923,7 @@
         <v>45</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>11</v>
@@ -6321,7 +6935,7 @@
         <v>11</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="H9" s="8" t="s">
         <v>11</v>
@@ -6335,7 +6949,7 @@
         <v>53</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>11</v>
@@ -6347,7 +6961,7 @@
         <v>11</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="H10" s="8" t="s">
         <v>11</v>
@@ -6355,7 +6969,7 @@
     </row>
     <row r="13" spans="1:8" ht="14.25" customHeight="1">
       <c r="A13" s="29" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15">
@@ -6366,22 +6980,22 @@
         <v>3</v>
       </c>
       <c r="C14" s="38" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="D14" s="38" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="E14" s="38" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="F14" s="38" t="s">
         <v>78</v>
       </c>
       <c r="G14" s="38" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="H14" s="38" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="16.5">
@@ -6392,13 +7006,13 @@
         <v>58</v>
       </c>
       <c r="C15" s="35" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>11</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="F15" s="35" t="s">
         <v>11</v>
@@ -6418,13 +7032,13 @@
         <v>60</v>
       </c>
       <c r="C16" s="35" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="D16" s="35" t="s">
         <v>11</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="F16" s="35" t="s">
         <v>11</v>
@@ -6444,13 +7058,13 @@
         <v>62</v>
       </c>
       <c r="C17" s="35" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="D17" s="35" t="s">
         <v>11</v>
       </c>
       <c r="E17" s="35" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="F17" s="35" t="s">
         <v>11</v>
@@ -6470,7 +7084,7 @@
         <v>53</v>
       </c>
       <c r="C18" s="35" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="D18" s="35" t="s">
         <v>11</v>
@@ -6482,10 +7096,10 @@
         <v>11</v>
       </c>
       <c r="G18" s="35" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="H18" s="35" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -6520,30 +7134,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="77" t="s">
-        <v>303</v>
-      </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
+      <c r="A1" s="79" t="s">
+        <v>296</v>
+      </c>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
     </row>
     <row r="2" spans="1:6" ht="24.95" customHeight="1">
       <c r="A2" s="9" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>82</v>
@@ -6551,59 +7165,59 @@
     </row>
     <row r="3" spans="1:6" ht="21.95" customHeight="1">
       <c r="A3" s="10" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>49</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="21.95" customHeight="1">
       <c r="A4" s="10" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>44</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="21.95" customHeight="1">
       <c r="A5" s="10" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>41</v>
       </c>
       <c r="C5" s="10" t="s">
+        <v>301</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>301</v>
+      </c>
+      <c r="E5" s="19" t="s">
         <v>308</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>308</v>
-      </c>
-      <c r="E5" s="19" t="s">
-        <v>315</v>
       </c>
       <c r="F5" s="10" t="s">
         <v>11</v>
@@ -6617,13 +7231,13 @@
         <v>25</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="F6" s="10" t="s">
         <v>11</v>
@@ -6637,16 +7251,16 @@
         <v>28</v>
       </c>
       <c r="C7" s="54" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="D7" s="54" t="s">
         <v>11</v>
       </c>
       <c r="E7" s="55" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="F7" s="56" t="s">
-        <v>340</v>
+        <v>327</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="21.95" customHeight="1">
@@ -6657,13 +7271,13 @@
         <v>18</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="F8" s="10" t="s">
         <v>11</v>
@@ -6677,13 +7291,13 @@
         <v>18</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="F9" s="10" t="s">
         <v>11</v>
@@ -6691,19 +7305,19 @@
     </row>
     <row r="10" spans="1:6" ht="21.95" customHeight="1">
       <c r="A10" s="10" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>18</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="F10" s="10" t="s">
         <v>11</v>
@@ -6717,13 +7331,13 @@
         <v>47</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="F11" s="10" t="s">
         <v>11</v>
@@ -6737,13 +7351,13 @@
         <v>35</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="E12" s="20" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="F12" s="10" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
auto: add 02-Knowledge (2), modify 01-Projects (2)
</commit_message>
<xml_diff>
--- a/01-Projects/family-hub/credit-card-management/信用卡主控表.xlsx
+++ b/01-Projects/family-hub/credit-card-management/信用卡主控表.xlsx
@@ -1963,6 +1963,63 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="21" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="20" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="20" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1979,75 +2036,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="21" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="20" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="20" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -2526,15 +2526,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="87"/>
+      <c r="G1" s="87"/>
     </row>
     <row r="2" spans="1:8" ht="24.95" customHeight="1">
       <c r="A2" s="1" t="s">
@@ -2961,12 +2961,12 @@
       </c>
     </row>
     <row r="19" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A19" s="71" t="s">
+      <c r="A19" s="92" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="69"/>
-      <c r="C19" s="69"/>
-      <c r="D19" s="70"/>
+      <c r="B19" s="90"/>
+      <c r="C19" s="90"/>
+      <c r="D19" s="91"/>
       <c r="E19" s="3">
         <f>SUM(E3:E18)</f>
         <v>831000</v>
@@ -2979,26 +2979,26 @@
       <c r="H19" s="26"/>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A21" s="67" t="s">
+      <c r="A21" s="88" t="s">
         <v>56</v>
       </c>
-      <c r="B21" s="66"/>
-      <c r="C21" s="66"/>
-      <c r="D21" s="66"/>
-      <c r="E21" s="66"/>
-      <c r="F21" s="66"/>
-      <c r="G21" s="66"/>
+      <c r="B21" s="87"/>
+      <c r="C21" s="87"/>
+      <c r="D21" s="87"/>
+      <c r="E21" s="87"/>
+      <c r="F21" s="87"/>
+      <c r="G21" s="87"/>
     </row>
     <row r="24" spans="1:8" ht="21" customHeight="1">
-      <c r="A24" s="65" t="s">
+      <c r="A24" s="86" t="s">
         <v>57</v>
       </c>
-      <c r="B24" s="66"/>
-      <c r="C24" s="66"/>
-      <c r="D24" s="66"/>
-      <c r="E24" s="66"/>
-      <c r="F24" s="66"/>
-      <c r="G24" s="66"/>
+      <c r="B24" s="87"/>
+      <c r="C24" s="87"/>
+      <c r="D24" s="87"/>
+      <c r="E24" s="87"/>
+      <c r="F24" s="87"/>
+      <c r="G24" s="87"/>
     </row>
     <row r="25" spans="1:8" ht="21" customHeight="1">
       <c r="A25" s="38" t="s">
@@ -3162,7 +3162,7 @@
       <c r="G31" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="H31" s="90" t="s">
+      <c r="H31" s="74" t="s">
         <v>357</v>
       </c>
     </row>
@@ -3285,12 +3285,12 @@
       <c r="H37" s="53"/>
     </row>
     <row r="38" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A38" s="68" t="s">
+      <c r="A38" s="89" t="s">
         <v>73</v>
       </c>
-      <c r="B38" s="69"/>
-      <c r="C38" s="69"/>
-      <c r="D38" s="70"/>
+      <c r="B38" s="90"/>
+      <c r="C38" s="90"/>
+      <c r="D38" s="91"/>
       <c r="E38" s="41">
         <f>SUM(E26:E37)</f>
         <v>44000</v>
@@ -3337,28 +3337,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="86" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="87"/>
+      <c r="G1" s="87"/>
+      <c r="H1" s="87"/>
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1">
-      <c r="A3" s="73" t="s">
+      <c r="A3" s="94" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="69"/>
-      <c r="C3" s="69"/>
-      <c r="D3" s="69"/>
-      <c r="E3" s="69"/>
-      <c r="F3" s="69"/>
-      <c r="G3" s="69"/>
-      <c r="H3" s="70"/>
+      <c r="B3" s="90"/>
+      <c r="C3" s="90"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="91"/>
       <c r="I3" s="24"/>
     </row>
     <row r="4" spans="1:9" ht="33" customHeight="1">
@@ -3518,16 +3518,16 @@
       <c r="I9" s="13"/>
     </row>
     <row r="10" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A10" s="73" t="s">
+      <c r="A10" s="94" t="s">
         <v>94</v>
       </c>
-      <c r="B10" s="69"/>
-      <c r="C10" s="69"/>
-      <c r="D10" s="69"/>
-      <c r="E10" s="69"/>
-      <c r="F10" s="69"/>
-      <c r="G10" s="69"/>
-      <c r="H10" s="70"/>
+      <c r="B10" s="90"/>
+      <c r="C10" s="90"/>
+      <c r="D10" s="90"/>
+      <c r="E10" s="90"/>
+      <c r="F10" s="90"/>
+      <c r="G10" s="90"/>
+      <c r="H10" s="91"/>
       <c r="I10" s="24"/>
     </row>
     <row r="11" spans="1:9" ht="16.5" customHeight="1">
@@ -3735,16 +3735,16 @@
       <c r="I18" s="13"/>
     </row>
     <row r="19" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A19" s="73" t="s">
+      <c r="A19" s="94" t="s">
         <v>109</v>
       </c>
-      <c r="B19" s="69"/>
-      <c r="C19" s="69"/>
-      <c r="D19" s="69"/>
-      <c r="E19" s="69"/>
-      <c r="F19" s="69"/>
-      <c r="G19" s="69"/>
-      <c r="H19" s="70"/>
+      <c r="B19" s="90"/>
+      <c r="C19" s="90"/>
+      <c r="D19" s="90"/>
+      <c r="E19" s="90"/>
+      <c r="F19" s="90"/>
+      <c r="G19" s="90"/>
+      <c r="H19" s="91"/>
       <c r="I19" s="24"/>
     </row>
     <row r="20" spans="1:9" ht="16.5" customHeight="1">
@@ -3869,16 +3869,16 @@
       <c r="I24" s="13"/>
     </row>
     <row r="25" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A25" s="73" t="s">
+      <c r="A25" s="94" t="s">
         <v>117</v>
       </c>
-      <c r="B25" s="69"/>
-      <c r="C25" s="69"/>
-      <c r="D25" s="69"/>
-      <c r="E25" s="69"/>
-      <c r="F25" s="69"/>
-      <c r="G25" s="69"/>
-      <c r="H25" s="70"/>
+      <c r="B25" s="90"/>
+      <c r="C25" s="90"/>
+      <c r="D25" s="90"/>
+      <c r="E25" s="90"/>
+      <c r="F25" s="90"/>
+      <c r="G25" s="90"/>
+      <c r="H25" s="91"/>
       <c r="I25" s="24"/>
     </row>
     <row r="26" spans="1:9" ht="16.5" customHeight="1">
@@ -3994,16 +3994,16 @@
       </c>
     </row>
     <row r="32" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A32" s="72" t="s">
+      <c r="A32" s="93" t="s">
         <v>133</v>
       </c>
-      <c r="B32" s="66"/>
-      <c r="C32" s="66"/>
-      <c r="D32" s="66"/>
-      <c r="E32" s="66"/>
-      <c r="F32" s="66"/>
-      <c r="G32" s="66"/>
-      <c r="H32" s="66"/>
+      <c r="B32" s="87"/>
+      <c r="C32" s="87"/>
+      <c r="D32" s="87"/>
+      <c r="E32" s="87"/>
+      <c r="F32" s="87"/>
+      <c r="G32" s="87"/>
+      <c r="H32" s="87"/>
     </row>
     <row r="35" spans="1:9" ht="14.25" customHeight="1">
       <c r="A35" s="36" t="s">
@@ -4412,24 +4412,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="86" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="87"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" s="67" t="s">
+      <c r="A2" s="88" t="s">
         <v>153</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
+      <c r="B2" s="87"/>
+      <c r="C2" s="87"/>
+      <c r="D2" s="87"/>
+      <c r="E2" s="87"/>
+      <c r="F2" s="87"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -4464,7 +4464,7 @@
       <c r="D4" s="57">
         <v>0</v>
       </c>
-      <c r="E4" s="82">
+      <c r="E4" s="66">
         <v>0</v>
       </c>
       <c r="F4" s="57" t="s">
@@ -4481,13 +4481,13 @@
       <c r="C5" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="85">
+      <c r="D5" s="69">
         <v>10000</v>
       </c>
-      <c r="E5" s="85">
+      <c r="E5" s="69">
         <v>10000</v>
       </c>
-      <c r="F5" s="86" t="s">
+      <c r="F5" s="70" t="s">
         <v>339</v>
       </c>
       <c r="H5" s="62" t="s">
@@ -4495,7 +4495,7 @@
       </c>
     </row>
     <row r="6" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A6" s="85" t="s">
+      <c r="A6" s="69" t="s">
         <v>381</v>
       </c>
       <c r="B6" s="8" t="s">
@@ -4504,13 +4504,13 @@
       <c r="C6" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="D6" s="85">
+      <c r="D6" s="69">
         <v>20100</v>
       </c>
-      <c r="E6" s="85">
+      <c r="E6" s="69">
         <v>20100</v>
       </c>
-      <c r="F6" s="86" t="s">
+      <c r="F6" s="70" t="s">
         <v>342</v>
       </c>
       <c r="H6" s="62" t="s">
@@ -4518,7 +4518,7 @@
       </c>
     </row>
     <row r="7" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A7" s="85" t="s">
+      <c r="A7" s="69" t="s">
         <v>364</v>
       </c>
       <c r="B7" s="8" t="s">
@@ -4527,13 +4527,13 @@
       <c r="C7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="87">
+      <c r="D7" s="71">
         <v>16000</v>
       </c>
       <c r="E7" s="8">
         <v>27000</v>
       </c>
-      <c r="F7" s="86" t="s">
+      <c r="F7" s="70" t="s">
         <v>340</v>
       </c>
       <c r="H7" s="62" t="s">
@@ -4541,25 +4541,25 @@
       </c>
     </row>
     <row r="8" spans="1:8" s="62" customFormat="1" ht="16.5">
-      <c r="A8" s="95" t="s">
+      <c r="A8" s="79" t="s">
         <v>386</v>
       </c>
-      <c r="B8" s="95" t="s">
+      <c r="B8" s="79" t="s">
         <v>372</v>
       </c>
-      <c r="C8" s="98" t="s">
+      <c r="C8" s="82" t="s">
         <v>62</v>
       </c>
-      <c r="D8" s="98">
+      <c r="D8" s="82">
         <v>20000</v>
       </c>
-      <c r="E8" s="98">
+      <c r="E8" s="82">
         <v>20000</v>
       </c>
-      <c r="F8" s="95"/>
+      <c r="F8" s="79"/>
     </row>
     <row r="9" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A9" s="85" t="s">
+      <c r="A9" s="69" t="s">
         <v>382</v>
       </c>
       <c r="B9" s="8" t="s">
@@ -4568,13 +4568,13 @@
       <c r="C9" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D9" s="85">
+      <c r="D9" s="69">
         <v>71000</v>
       </c>
-      <c r="E9" s="85">
+      <c r="E9" s="69">
         <v>71000</v>
       </c>
-      <c r="F9" s="86" t="s">
+      <c r="F9" s="70" t="s">
         <v>350</v>
       </c>
       <c r="H9" s="62" t="s">
@@ -4582,22 +4582,22 @@
       </c>
     </row>
     <row r="10" spans="1:8" s="62" customFormat="1" ht="16.5" customHeight="1">
-      <c r="A10" s="95"/>
+      <c r="A10" s="79"/>
       <c r="B10" s="63"/>
       <c r="C10" s="63"/>
-      <c r="D10" s="95"/>
+      <c r="D10" s="79"/>
       <c r="E10" s="63"/>
-      <c r="F10" s="86"/>
-      <c r="H10" s="84"/>
+      <c r="F10" s="70"/>
+      <c r="H10" s="68"/>
     </row>
     <row r="11" spans="1:8" s="62" customFormat="1" ht="16.5" customHeight="1">
-      <c r="A11" s="95"/>
+      <c r="A11" s="79"/>
       <c r="B11" s="63"/>
       <c r="C11" s="63"/>
-      <c r="D11" s="95"/>
+      <c r="D11" s="79"/>
       <c r="E11" s="63"/>
-      <c r="F11" s="86"/>
-      <c r="H11" s="84"/>
+      <c r="F11" s="70"/>
+      <c r="H11" s="68"/>
     </row>
     <row r="12" spans="1:8" ht="32.25" customHeight="1">
       <c r="A12" s="57" t="s">
@@ -4615,13 +4615,13 @@
       <c r="E12" s="57">
         <v>46000</v>
       </c>
-      <c r="F12" s="94" t="s">
+      <c r="F12" s="78" t="s">
         <v>341</v>
       </c>
-      <c r="H12" s="84"/>
+      <c r="H12" s="68"/>
     </row>
     <row r="13" spans="1:8" ht="33">
-      <c r="A13" s="95" t="s">
+      <c r="A13" s="79" t="s">
         <v>366</v>
       </c>
       <c r="B13" s="63" t="s">
@@ -4633,36 +4633,36 @@
       <c r="D13" s="35">
         <v>46000</v>
       </c>
-      <c r="E13" s="89">
+      <c r="E13" s="73">
         <v>110000</v>
       </c>
       <c r="F13" s="51" t="s">
         <v>365</v>
       </c>
-      <c r="G13" s="83" t="s">
+      <c r="G13" s="67" t="s">
         <v>356</v>
       </c>
-      <c r="H13" s="92" t="s">
+      <c r="H13" s="76" t="s">
         <v>360</v>
       </c>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="101"/>
-      <c r="B14" s="101"/>
-      <c r="C14" s="101"/>
-      <c r="D14" s="101"/>
-      <c r="E14" s="101"/>
-      <c r="F14" s="101"/>
+      <c r="A14" s="85"/>
+      <c r="B14" s="85"/>
+      <c r="C14" s="85"/>
+      <c r="D14" s="85"/>
+      <c r="E14" s="85"/>
+      <c r="F14" s="85"/>
     </row>
     <row r="15" spans="1:8" s="62" customFormat="1" ht="16.5">
-      <c r="A15" s="95"/>
-      <c r="B15" s="95"/>
-      <c r="C15" s="95"/>
-      <c r="D15" s="98"/>
-      <c r="E15" s="100"/>
-      <c r="F15" s="95"/>
-      <c r="G15" s="91"/>
-      <c r="H15" s="92"/>
+      <c r="A15" s="79"/>
+      <c r="B15" s="79"/>
+      <c r="C15" s="79"/>
+      <c r="D15" s="82"/>
+      <c r="E15" s="84"/>
+      <c r="F15" s="79"/>
+      <c r="G15" s="75"/>
+      <c r="H15" s="76"/>
     </row>
     <row r="16" spans="1:8" ht="16.5" customHeight="1">
       <c r="A16" s="8" t="s">
@@ -4674,29 +4674,29 @@
       <c r="C16" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="D16" s="87">
+      <c r="D16" s="71">
         <v>60000</v>
       </c>
-      <c r="E16" s="87">
+      <c r="E16" s="71">
         <v>60000</v>
       </c>
-      <c r="F16" s="86" t="s">
+      <c r="F16" s="70" t="s">
         <v>342</v>
       </c>
-      <c r="G16" s="83"/>
-      <c r="H16" s="97" t="s">
+      <c r="G16" s="67"/>
+      <c r="H16" s="81" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="17" spans="1:8" s="62" customFormat="1" ht="16.5" customHeight="1">
-      <c r="A17" s="95"/>
-      <c r="B17" s="95"/>
-      <c r="C17" s="95"/>
-      <c r="D17" s="95"/>
-      <c r="E17" s="95"/>
-      <c r="F17" s="95"/>
-      <c r="G17" s="91"/>
-      <c r="H17" s="97"/>
+      <c r="A17" s="79"/>
+      <c r="B17" s="79"/>
+      <c r="C17" s="79"/>
+      <c r="D17" s="79"/>
+      <c r="E17" s="79"/>
+      <c r="F17" s="79"/>
+      <c r="G17" s="75"/>
+      <c r="H17" s="81"/>
     </row>
     <row r="18" spans="1:8" ht="16.5" customHeight="1">
       <c r="A18" s="8" t="s">
@@ -4714,27 +4714,27 @@
       <c r="E18" s="8">
         <v>7000</v>
       </c>
-      <c r="F18" s="86" t="s">
+      <c r="F18" s="70" t="s">
         <v>343</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A19" s="81" t="s">
+      <c r="A19" s="65" t="s">
         <v>320</v>
       </c>
-      <c r="B19" s="81" t="s">
+      <c r="B19" s="65" t="s">
         <v>376</v>
       </c>
-      <c r="C19" s="81" t="s">
+      <c r="C19" s="65" t="s">
         <v>48</v>
       </c>
-      <c r="D19" s="81">
+      <c r="D19" s="65">
         <v>0</v>
       </c>
-      <c r="E19" s="81">
+      <c r="E19" s="65">
         <v>5100</v>
       </c>
-      <c r="F19" s="96" t="s">
+      <c r="F19" s="80" t="s">
         <v>344</v>
       </c>
     </row>
@@ -4745,34 +4745,34 @@
       <c r="B20" s="63" t="s">
         <v>370</v>
       </c>
-      <c r="C20" s="89" t="s">
+      <c r="C20" s="73" t="s">
         <v>361</v>
       </c>
-      <c r="D20" s="93">
+      <c r="D20" s="77">
         <v>33000</v>
       </c>
-      <c r="E20" s="93">
+      <c r="E20" s="77">
         <v>33000</v>
       </c>
       <c r="F20" s="48" t="s">
         <v>317</v>
       </c>
-      <c r="G20" s="83" t="s">
+      <c r="G20" s="67" t="s">
         <v>355</v>
       </c>
-      <c r="H20" s="92" t="s">
+      <c r="H20" s="76" t="s">
         <v>359</v>
       </c>
     </row>
     <row r="21" spans="1:8" s="62" customFormat="1" ht="16.5">
-      <c r="A21" s="95"/>
-      <c r="B21" s="95"/>
-      <c r="C21" s="100"/>
-      <c r="D21" s="98"/>
-      <c r="E21" s="98"/>
-      <c r="F21" s="95"/>
-      <c r="G21" s="91"/>
-      <c r="H21" s="92"/>
+      <c r="A21" s="79"/>
+      <c r="B21" s="79"/>
+      <c r="C21" s="84"/>
+      <c r="D21" s="82"/>
+      <c r="E21" s="82"/>
+      <c r="F21" s="79"/>
+      <c r="G21" s="75"/>
+      <c r="H21" s="76"/>
     </row>
     <row r="22" spans="1:8" ht="16.5" customHeight="1">
       <c r="A22" s="8" t="s">
@@ -4784,13 +4784,13 @@
       <c r="C22" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="D22" s="87">
+      <c r="D22" s="71">
         <v>26000</v>
       </c>
-      <c r="E22" s="87">
+      <c r="E22" s="71">
         <v>26000</v>
       </c>
-      <c r="F22" s="86" t="s">
+      <c r="F22" s="70" t="s">
         <v>345</v>
       </c>
       <c r="H22" s="62" t="s">
@@ -4807,10 +4807,10 @@
       <c r="C23" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="D23" s="85">
+      <c r="D23" s="69">
         <v>19000</v>
       </c>
-      <c r="E23" s="85">
+      <c r="E23" s="69">
         <v>19000</v>
       </c>
       <c r="F23" s="63" t="s">
@@ -4850,10 +4850,10 @@
       <c r="C25" s="64" t="s">
         <v>60</v>
       </c>
-      <c r="D25" s="93">
+      <c r="D25" s="77">
         <v>13000</v>
       </c>
-      <c r="E25" s="93">
+      <c r="E25" s="77">
         <v>13000</v>
       </c>
       <c r="F25" s="64"/>
@@ -4862,8 +4862,8 @@
       <c r="A26" s="63"/>
       <c r="B26" s="63"/>
       <c r="C26" s="64"/>
-      <c r="D26" s="98"/>
-      <c r="E26" s="98"/>
+      <c r="D26" s="82"/>
+      <c r="E26" s="82"/>
       <c r="F26" s="64"/>
     </row>
     <row r="27" spans="1:8" ht="16.5" customHeight="1">
@@ -4876,13 +4876,13 @@
       <c r="C27" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="D27" s="87">
+      <c r="D27" s="71">
         <v>50000</v>
       </c>
-      <c r="E27" s="87">
+      <c r="E27" s="71">
         <v>50000</v>
       </c>
-      <c r="F27" s="86" t="s">
+      <c r="F27" s="70" t="s">
         <v>347</v>
       </c>
     </row>
@@ -4896,10 +4896,10 @@
       <c r="C28" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D28" s="87">
+      <c r="D28" s="71">
         <v>20000</v>
       </c>
-      <c r="E28" s="87">
+      <c r="E28" s="71">
         <v>20000</v>
       </c>
       <c r="F28" s="63" t="s">
@@ -4910,9 +4910,9 @@
       <c r="A29" s="63"/>
       <c r="B29" s="63"/>
       <c r="C29" s="63"/>
-      <c r="D29" s="95"/>
-      <c r="E29" s="95"/>
-      <c r="F29" s="95"/>
+      <c r="D29" s="79"/>
+      <c r="E29" s="79"/>
+      <c r="F29" s="79"/>
     </row>
     <row r="30" spans="1:8" ht="16.5" customHeight="1">
       <c r="A30" s="57" t="s">
@@ -4930,12 +4930,12 @@
       <c r="E30" s="57">
         <v>0</v>
       </c>
-      <c r="F30" s="94" t="s">
+      <c r="F30" s="78" t="s">
         <v>351</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="18" customHeight="1">
-      <c r="A31" s="99" t="s">
+      <c r="A31" s="83" t="s">
         <v>379</v>
       </c>
       <c r="B31" s="8" t="s">
@@ -4944,13 +4944,13 @@
       <c r="C31" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="D31" s="87">
+      <c r="D31" s="71">
         <v>60000</v>
       </c>
-      <c r="E31" s="87">
+      <c r="E31" s="71">
         <v>60000</v>
       </c>
-      <c r="F31" s="86" t="s">
+      <c r="F31" s="70" t="s">
         <v>352</v>
       </c>
       <c r="H31" t="s">
@@ -4958,30 +4958,30 @@
       </c>
     </row>
     <row r="32" spans="1:8" ht="16.5">
-      <c r="A32" s="88"/>
-      <c r="B32" s="86" t="s">
+      <c r="A32" s="72"/>
+      <c r="B32" s="70" t="s">
         <v>353</v>
       </c>
-      <c r="C32" s="88"/>
-      <c r="D32" s="88">
+      <c r="C32" s="72"/>
+      <c r="D32" s="72">
         <f>SUM(D4:D31)</f>
         <v>487100</v>
       </c>
-      <c r="E32" s="88">
+      <c r="E32" s="72">
         <f>SUM(E4:E31)</f>
         <v>632200</v>
       </c>
-      <c r="F32" s="88"/>
+      <c r="F32" s="72"/>
     </row>
     <row r="33" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A33" s="67" t="s">
+      <c r="A33" s="88" t="s">
         <v>154</v>
       </c>
-      <c r="B33" s="66"/>
-      <c r="C33" s="66"/>
-      <c r="D33" s="66"/>
-      <c r="E33" s="66"/>
-      <c r="F33" s="66"/>
+      <c r="B33" s="87"/>
+      <c r="C33" s="87"/>
+      <c r="D33" s="87"/>
+      <c r="E33" s="87"/>
+      <c r="F33" s="87"/>
     </row>
     <row r="36" spans="1:8" ht="14.25">
       <c r="A36" s="36" t="s">
@@ -5009,25 +5009,25 @@
       </c>
     </row>
     <row r="38" spans="1:8" ht="16.5">
-      <c r="A38" s="95" t="s">
+      <c r="A38" s="79" t="s">
         <v>386</v>
       </c>
-      <c r="B38" s="95" t="s">
+      <c r="B38" s="79" t="s">
         <v>372</v>
       </c>
       <c r="C38" s="35" t="s">
         <v>62</v>
       </c>
-      <c r="D38" s="93">
+      <c r="D38" s="77">
         <v>20000</v>
       </c>
-      <c r="E38" s="93">
+      <c r="E38" s="77">
         <v>20000</v>
       </c>
       <c r="F38" s="63"/>
     </row>
     <row r="39" spans="1:8" s="62" customFormat="1" ht="33">
-      <c r="A39" s="95" t="s">
+      <c r="A39" s="79" t="s">
         <v>366</v>
       </c>
       <c r="B39" s="63" t="s">
@@ -5039,16 +5039,16 @@
       <c r="D39" s="64">
         <v>46000</v>
       </c>
-      <c r="E39" s="89">
+      <c r="E39" s="73">
         <v>110000</v>
       </c>
       <c r="F39" s="63" t="s">
         <v>365</v>
       </c>
-      <c r="G39" s="83" t="s">
+      <c r="G39" s="67" t="s">
         <v>356</v>
       </c>
-      <c r="H39" s="92" t="s">
+      <c r="H39" s="76" t="s">
         <v>360</v>
       </c>
     </row>
@@ -5059,22 +5059,22 @@
       <c r="B40" s="63" t="s">
         <v>370</v>
       </c>
-      <c r="C40" s="89" t="s">
+      <c r="C40" s="73" t="s">
         <v>361</v>
       </c>
-      <c r="D40" s="93">
+      <c r="D40" s="77">
         <v>33000</v>
       </c>
-      <c r="E40" s="93">
+      <c r="E40" s="77">
         <v>33000</v>
       </c>
       <c r="F40" s="63" t="s">
         <v>317</v>
       </c>
-      <c r="G40" s="83" t="s">
+      <c r="G40" s="67" t="s">
         <v>355</v>
       </c>
-      <c r="H40" s="92" t="s">
+      <c r="H40" s="76" t="s">
         <v>359</v>
       </c>
     </row>
@@ -5088,20 +5088,20 @@
       <c r="C41" s="35" t="s">
         <v>60</v>
       </c>
-      <c r="D41" s="93">
+      <c r="D41" s="77">
         <v>13000</v>
       </c>
-      <c r="E41" s="93">
+      <c r="E41" s="77">
         <v>13000</v>
       </c>
       <c r="F41" s="35"/>
     </row>
     <row r="42" spans="1:8" ht="16.5">
       <c r="A42" s="51" t="s">
-        <v>333</v>
-      </c>
-      <c r="B42" s="63" t="s">
-        <v>374</v>
+        <v>332</v>
+      </c>
+      <c r="B42" s="35" t="s">
+        <v>40</v>
       </c>
       <c r="C42" s="35" t="s">
         <v>11</v>
@@ -5114,10 +5114,10 @@
     </row>
     <row r="43" spans="1:8" ht="16.5">
       <c r="A43" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="B43" s="35" t="s">
-        <v>40</v>
+        <v>333</v>
+      </c>
+      <c r="B43" s="63" t="s">
+        <v>374</v>
       </c>
       <c r="C43" s="35" t="s">
         <v>11</v>
@@ -5171,20 +5171,20 @@
       <c r="F46" s="35"/>
     </row>
     <row r="47" spans="1:8" ht="16.5">
-      <c r="A47" s="88"/>
-      <c r="B47" s="86" t="s">
+      <c r="A47" s="72"/>
+      <c r="B47" s="70" t="s">
         <v>353</v>
       </c>
-      <c r="C47" s="88"/>
-      <c r="D47" s="88">
+      <c r="C47" s="72"/>
+      <c r="D47" s="72">
         <f>SUM(D13:D46)</f>
         <v>949100</v>
       </c>
-      <c r="E47" s="88">
+      <c r="E47" s="72">
         <f>SUM(E13:E46)</f>
         <v>1246300</v>
       </c>
-      <c r="F47" s="88"/>
+      <c r="F47" s="72"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -5255,28 +5255,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="86" t="s">
         <v>157</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="87"/>
+      <c r="G1" s="87"/>
+      <c r="H1" s="87"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
-      <c r="A3" s="74" t="s">
+      <c r="A3" s="95" t="s">
         <v>158</v>
       </c>
-      <c r="B3" s="66"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
+      <c r="B3" s="87"/>
+      <c r="C3" s="87"/>
+      <c r="D3" s="87"/>
+      <c r="E3" s="87"/>
+      <c r="F3" s="87"/>
+      <c r="G3" s="87"/>
+      <c r="H3" s="87"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -5591,10 +5591,10 @@
       </c>
     </row>
     <row r="16" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A16" s="76" t="s">
+      <c r="A16" s="96" t="s">
         <v>198</v>
       </c>
-      <c r="B16" s="80"/>
+      <c r="B16" s="97"/>
       <c r="C16" s="8">
         <f>SUM(C5:C15)</f>
         <v>35</v>
@@ -5607,21 +5607,21 @@
         <f>SUM(E5:E15)</f>
         <v>35</v>
       </c>
-      <c r="F16" s="76" t="s">
+      <c r="F16" s="96" t="s">
         <v>199</v>
       </c>
-      <c r="G16" s="80"/>
+      <c r="G16" s="97"/>
       <c r="H16" s="21"/>
     </row>
     <row r="17" spans="1:8" ht="15" customHeight="1">
-      <c r="A17" s="66"/>
-      <c r="B17" s="66"/>
-      <c r="C17" s="66"/>
-      <c r="D17" s="66"/>
-      <c r="E17" s="66"/>
-      <c r="F17" s="66"/>
-      <c r="G17" s="66"/>
-      <c r="H17" s="66"/>
+      <c r="A17" s="87"/>
+      <c r="B17" s="87"/>
+      <c r="C17" s="87"/>
+      <c r="D17" s="87"/>
+      <c r="E17" s="87"/>
+      <c r="F17" s="87"/>
+      <c r="G17" s="87"/>
+      <c r="H17" s="87"/>
     </row>
     <row r="18" spans="1:8" ht="15" customHeight="1">
       <c r="A18" s="33" t="s">
@@ -6018,25 +6018,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="86" t="s">
         <v>223</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="87"/>
+      <c r="G1" s="87"/>
+      <c r="H1" s="87"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
-      <c r="A3" s="74" t="s">
+      <c r="A3" s="95" t="s">
         <v>224</v>
       </c>
-      <c r="B3" s="66"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
+      <c r="B3" s="87"/>
+      <c r="C3" s="87"/>
+      <c r="D3" s="87"/>
+      <c r="E3" s="87"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -6124,16 +6124,16 @@
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
-      <c r="A11" s="74" t="s">
+      <c r="A11" s="95" t="s">
         <v>244</v>
       </c>
-      <c r="B11" s="66"/>
-      <c r="C11" s="66"/>
-      <c r="D11" s="66"/>
-      <c r="E11" s="66"/>
-      <c r="F11" s="66"/>
-      <c r="G11" s="66"/>
-      <c r="H11" s="66"/>
+      <c r="B11" s="87"/>
+      <c r="C11" s="87"/>
+      <c r="D11" s="87"/>
+      <c r="E11" s="87"/>
+      <c r="F11" s="87"/>
+      <c r="G11" s="87"/>
+      <c r="H11" s="87"/>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
       <c r="A12" s="1" t="s">
@@ -6289,24 +6289,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="86" t="s">
         <v>251</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="87"/>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1">
-      <c r="A3" s="74" t="s">
+      <c r="A3" s="95" t="s">
         <v>252</v>
       </c>
-      <c r="B3" s="66"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
+      <c r="B3" s="87"/>
+      <c r="C3" s="87"/>
+      <c r="D3" s="87"/>
+      <c r="E3" s="87"/>
+      <c r="F3" s="87"/>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1">
       <c r="A4" s="5" t="s">
@@ -6389,10 +6389,10 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A8" s="78" t="s">
+      <c r="A8" s="100" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="70"/>
+      <c r="B8" s="91"/>
       <c r="C8" s="35">
         <v>500</v>
       </c>
@@ -6427,18 +6427,18 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1">
-      <c r="A10" s="77"/>
-      <c r="B10" s="69"/>
-      <c r="C10" s="69"/>
-      <c r="D10" s="69"/>
-      <c r="E10" s="69"/>
-      <c r="F10" s="70"/>
+      <c r="A10" s="98"/>
+      <c r="B10" s="90"/>
+      <c r="C10" s="90"/>
+      <c r="D10" s="90"/>
+      <c r="E10" s="90"/>
+      <c r="F10" s="91"/>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1">
-      <c r="A11" s="76" t="s">
+      <c r="A11" s="96" t="s">
         <v>198</v>
       </c>
-      <c r="B11" s="70"/>
+      <c r="B11" s="91"/>
       <c r="C11" s="34">
         <f>SUM(C5:C9)</f>
         <v>4180</v>
@@ -6499,14 +6499,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="15" customHeight="1">
-      <c r="A17" s="75" t="s">
+      <c r="A17" s="99" t="s">
         <v>266</v>
       </c>
-      <c r="B17" s="69"/>
-      <c r="C17" s="69"/>
-      <c r="D17" s="69"/>
-      <c r="E17" s="69"/>
-      <c r="F17" s="70"/>
+      <c r="B17" s="90"/>
+      <c r="C17" s="90"/>
+      <c r="D17" s="90"/>
+      <c r="E17" s="90"/>
+      <c r="F17" s="91"/>
     </row>
     <row r="18" spans="1:6" ht="15" customHeight="1">
       <c r="A18" s="11" t="s">
@@ -6557,14 +6557,14 @@
       </c>
     </row>
     <row r="23" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A23" s="75" t="s">
+      <c r="A23" s="99" t="s">
         <v>164</v>
       </c>
-      <c r="B23" s="69"/>
-      <c r="C23" s="69"/>
-      <c r="D23" s="69"/>
-      <c r="E23" s="69"/>
-      <c r="F23" s="70"/>
+      <c r="B23" s="90"/>
+      <c r="C23" s="90"/>
+      <c r="D23" s="90"/>
+      <c r="E23" s="90"/>
+      <c r="F23" s="91"/>
     </row>
     <row r="24" spans="1:6" ht="16.5" customHeight="1">
       <c r="A24" s="8" t="s">
@@ -6736,28 +6736,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="86" t="s">
         <v>282</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="87"/>
+      <c r="G1" s="87"/>
+      <c r="H1" s="87"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" s="67" t="s">
+      <c r="A2" s="88" t="s">
         <v>283</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="66"/>
-      <c r="H2" s="66"/>
+      <c r="B2" s="87"/>
+      <c r="C2" s="87"/>
+      <c r="D2" s="87"/>
+      <c r="E2" s="87"/>
+      <c r="F2" s="87"/>
+      <c r="G2" s="87"/>
+      <c r="H2" s="87"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -7134,14 +7134,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="79" t="s">
+      <c r="A1" s="101" t="s">
         <v>296</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="87"/>
     </row>
     <row r="2" spans="1:6" ht="24.95" customHeight="1">
       <c r="A2" s="9" t="s">

</xml_diff>

<commit_message>
auto: add 02-Knowledge (1), delete 01-Projects (2), modify 01-Projects (4)
</commit_message>
<xml_diff>
--- a/01-Projects/family-hub/credit-card-management/信用卡主控表.xlsx
+++ b/01-Projects/family-hub/credit-card-management/信用卡主控表.xlsx
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="971" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="980" uniqueCount="394">
   <si>
     <t>信用卡卡片总览 — 韩伟</t>
   </si>
@@ -1367,6 +1367,30 @@
   </si>
   <si>
     <t>农行</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>积分兑换里程</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>APP可以领取 30元券</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>交通-2</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>白金</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>6笔</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>刷6笔数抵扣</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
@@ -1787,7 +1811,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2021,6 +2045,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2049,6 +2077,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="58" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -2527,15 +2558,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="87" t="s">
+      <c r="A1" s="89" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
     </row>
     <row r="2" spans="1:8" ht="24.95" customHeight="1">
       <c r="A2" s="1" t="s">
@@ -2962,12 +2993,12 @@
       </c>
     </row>
     <row r="19" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A19" s="93" t="s">
+      <c r="A19" s="95" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="91"/>
-      <c r="C19" s="91"/>
-      <c r="D19" s="92"/>
+      <c r="B19" s="93"/>
+      <c r="C19" s="93"/>
+      <c r="D19" s="94"/>
       <c r="E19" s="3">
         <f>SUM(E3:E18)</f>
         <v>831000</v>
@@ -2980,26 +3011,26 @@
       <c r="H19" s="26"/>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A21" s="89" t="s">
+      <c r="A21" s="91" t="s">
         <v>56</v>
       </c>
-      <c r="B21" s="88"/>
-      <c r="C21" s="88"/>
-      <c r="D21" s="88"/>
-      <c r="E21" s="88"/>
-      <c r="F21" s="88"/>
-      <c r="G21" s="88"/>
+      <c r="B21" s="90"/>
+      <c r="C21" s="90"/>
+      <c r="D21" s="90"/>
+      <c r="E21" s="90"/>
+      <c r="F21" s="90"/>
+      <c r="G21" s="90"/>
     </row>
     <row r="24" spans="1:8" ht="21" customHeight="1">
-      <c r="A24" s="87" t="s">
+      <c r="A24" s="89" t="s">
         <v>57</v>
       </c>
-      <c r="B24" s="88"/>
-      <c r="C24" s="88"/>
-      <c r="D24" s="88"/>
-      <c r="E24" s="88"/>
-      <c r="F24" s="88"/>
-      <c r="G24" s="88"/>
+      <c r="B24" s="90"/>
+      <c r="C24" s="90"/>
+      <c r="D24" s="90"/>
+      <c r="E24" s="90"/>
+      <c r="F24" s="90"/>
+      <c r="G24" s="90"/>
     </row>
     <row r="25" spans="1:8" ht="21" customHeight="1">
       <c r="A25" s="38" t="s">
@@ -3286,12 +3317,12 @@
       <c r="H37" s="53"/>
     </row>
     <row r="38" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A38" s="90" t="s">
+      <c r="A38" s="92" t="s">
         <v>73</v>
       </c>
-      <c r="B38" s="91"/>
-      <c r="C38" s="91"/>
-      <c r="D38" s="92"/>
+      <c r="B38" s="93"/>
+      <c r="C38" s="93"/>
+      <c r="D38" s="94"/>
       <c r="E38" s="41">
         <f>SUM(E26:E37)</f>
         <v>44000</v>
@@ -3323,7 +3354,7 @@
   <sheetPr>
     <tabColor rgb="FFED7D31"/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="10" style="30" customWidth="1"/>
@@ -3338,28 +3369,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1">
-      <c r="A1" s="87" t="s">
+      <c r="A1" s="89" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1">
-      <c r="A3" s="95" t="s">
+      <c r="A3" s="97" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="91"/>
-      <c r="C3" s="91"/>
-      <c r="D3" s="91"/>
-      <c r="E3" s="91"/>
-      <c r="F3" s="91"/>
-      <c r="G3" s="91"/>
-      <c r="H3" s="92"/>
+      <c r="B3" s="93"/>
+      <c r="C3" s="93"/>
+      <c r="D3" s="93"/>
+      <c r="E3" s="93"/>
+      <c r="F3" s="93"/>
+      <c r="G3" s="93"/>
+      <c r="H3" s="94"/>
       <c r="I3" s="24"/>
     </row>
     <row r="4" spans="1:9" ht="33" customHeight="1">
@@ -3519,16 +3550,16 @@
       <c r="I9" s="13"/>
     </row>
     <row r="10" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A10" s="95" t="s">
+      <c r="A10" s="97" t="s">
         <v>94</v>
       </c>
-      <c r="B10" s="91"/>
-      <c r="C10" s="91"/>
-      <c r="D10" s="91"/>
-      <c r="E10" s="91"/>
-      <c r="F10" s="91"/>
-      <c r="G10" s="91"/>
-      <c r="H10" s="92"/>
+      <c r="B10" s="93"/>
+      <c r="C10" s="93"/>
+      <c r="D10" s="93"/>
+      <c r="E10" s="93"/>
+      <c r="F10" s="93"/>
+      <c r="G10" s="93"/>
+      <c r="H10" s="94"/>
       <c r="I10" s="24"/>
     </row>
     <row r="11" spans="1:9" ht="16.5" customHeight="1">
@@ -3589,42 +3620,40 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A13" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" s="8">
+    <row r="13" spans="1:9" s="87" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A13" s="88" t="s">
+        <v>390</v>
+      </c>
+      <c r="B13" s="88" t="s">
+        <v>391</v>
+      </c>
+      <c r="C13" s="88" t="s">
+        <v>392</v>
+      </c>
+      <c r="D13" s="88">
+        <v>6</v>
+      </c>
+      <c r="E13" s="88">
         <v>0</v>
       </c>
-      <c r="F13" s="12">
-        <v>46234</v>
-      </c>
-      <c r="G13" s="8"/>
+      <c r="F13" s="105">
+        <v>46265</v>
+      </c>
+      <c r="G13" s="88"/>
       <c r="H13" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="I13" s="13" t="s">
-        <v>86</v>
-      </c>
+      <c r="I13" s="43"/>
     </row>
     <row r="14" spans="1:9" ht="16.5" customHeight="1">
       <c r="A14" s="8" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>11</v>
@@ -3633,7 +3662,7 @@
         <v>0</v>
       </c>
       <c r="F14" s="12">
-        <v>46317</v>
+        <v>46234</v>
       </c>
       <c r="G14" s="8"/>
       <c r="H14" s="16" t="s">
@@ -3643,316 +3672,316 @@
         <v>86</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="30.75" customHeight="1">
+    <row r="15" spans="1:9" ht="16.5" customHeight="1">
       <c r="A15" s="8" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="D15" s="8">
-        <v>5</v>
+        <v>102</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>11</v>
       </c>
       <c r="E15" s="8">
         <v>0</v>
       </c>
       <c r="F15" s="12">
-        <v>46080</v>
+        <v>46317</v>
       </c>
       <c r="G15" s="8"/>
       <c r="H15" s="16" t="s">
         <v>85</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="16.5" customHeight="1">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="30.75" customHeight="1">
       <c r="A16" s="8" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D16" s="8">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E16" s="8">
         <v>0</v>
       </c>
-      <c r="F16" s="8" t="s">
-        <v>11</v>
+      <c r="F16" s="12">
+        <v>46080</v>
       </c>
       <c r="G16" s="8"/>
       <c r="H16" s="16" t="s">
         <v>85</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="16.5" customHeight="1">
       <c r="A17" s="8" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D17" s="8">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E17" s="8">
         <v>0</v>
       </c>
-      <c r="F17" s="12">
-        <v>46044</v>
+      <c r="F17" s="8" t="s">
+        <v>11</v>
       </c>
       <c r="G17" s="8"/>
       <c r="H17" s="16" t="s">
         <v>85</v>
       </c>
       <c r="I17" s="13" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="16.5" customHeight="1">
+      <c r="A18" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D18" s="8">
+        <v>6</v>
+      </c>
+      <c r="E18" s="8">
+        <v>0</v>
+      </c>
+      <c r="F18" s="12">
+        <v>46044</v>
+      </c>
+      <c r="G18" s="8"/>
+      <c r="H18" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="I18" s="13" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A18" s="8"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="13"/>
-    </row>
     <row r="19" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A19" s="95" t="s">
+      <c r="A19" s="8"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="13"/>
+    </row>
+    <row r="20" spans="1:9" ht="16.5" customHeight="1">
+      <c r="A20" s="97" t="s">
         <v>109</v>
       </c>
-      <c r="B19" s="91"/>
-      <c r="C19" s="91"/>
-      <c r="D19" s="91"/>
-      <c r="E19" s="91"/>
-      <c r="F19" s="91"/>
-      <c r="G19" s="91"/>
-      <c r="H19" s="92"/>
-      <c r="I19" s="24"/>
-    </row>
-    <row r="20" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A20" s="4" t="s">
+      <c r="B20" s="93"/>
+      <c r="C20" s="93"/>
+      <c r="D20" s="93"/>
+      <c r="E20" s="93"/>
+      <c r="F20" s="93"/>
+      <c r="G20" s="93"/>
+      <c r="H20" s="94"/>
+      <c r="I20" s="24"/>
+    </row>
+    <row r="21" spans="1:9" ht="16.5" customHeight="1">
+      <c r="A21" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B21" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C21" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D21" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E21" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F21" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="G20" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="H20" s="4" t="s">
+      <c r="G21" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H21" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="I20" s="4" t="s">
+      <c r="I21" s="4" t="s">
         <v>82</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A21" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="D21" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="E21" s="8">
-        <v>0</v>
-      </c>
-      <c r="F21" s="12">
-        <v>46233</v>
-      </c>
-      <c r="G21" s="8"/>
-      <c r="H21" s="16" t="s">
-        <v>85</v>
-      </c>
-      <c r="I21" s="14" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="16.5" customHeight="1">
       <c r="A22" s="8" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E22" s="8">
         <v>0</v>
       </c>
-      <c r="F22" s="8" t="s">
-        <v>114</v>
+      <c r="F22" s="12">
+        <v>46233</v>
       </c>
       <c r="G22" s="8"/>
       <c r="H22" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="I22" s="13" t="s">
+      <c r="I22" s="14" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="16.5" customHeight="1">
+      <c r="A23" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="E23" s="8">
+        <v>0</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="G23" s="8"/>
+      <c r="H23" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="I23" s="13" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="30.75" customHeight="1">
-      <c r="A23" s="8" t="s">
+    <row r="24" spans="1:9" ht="30.75" customHeight="1">
+      <c r="A24" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B24" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C24" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="D23" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E23" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="F23" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="G23" s="8"/>
-      <c r="H23" s="17" t="s">
+      <c r="D24" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G24" s="8"/>
+      <c r="H24" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="I23" s="14" t="s">
+      <c r="I24" s="14" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A24" s="8"/>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="8"/>
-      <c r="I24" s="13"/>
-    </row>
     <row r="25" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A25" s="95" t="s">
+      <c r="A25" s="8"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="13"/>
+    </row>
+    <row r="26" spans="1:9" ht="16.5" customHeight="1">
+      <c r="A26" s="97" t="s">
         <v>117</v>
       </c>
-      <c r="B25" s="91"/>
-      <c r="C25" s="91"/>
-      <c r="D25" s="91"/>
-      <c r="E25" s="91"/>
-      <c r="F25" s="91"/>
-      <c r="G25" s="91"/>
-      <c r="H25" s="92"/>
-      <c r="I25" s="24"/>
-    </row>
-    <row r="26" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A26" s="4" t="s">
+      <c r="B26" s="93"/>
+      <c r="C26" s="93"/>
+      <c r="D26" s="93"/>
+      <c r="E26" s="93"/>
+      <c r="F26" s="93"/>
+      <c r="G26" s="93"/>
+      <c r="H26" s="94"/>
+      <c r="I26" s="24"/>
+    </row>
+    <row r="27" spans="1:9" ht="16.5" customHeight="1">
+      <c r="A27" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B27" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C27" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D27" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E27" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F27" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="G26" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="H26" s="4" t="s">
+      <c r="G27" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H27" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="I26" s="4" t="s">
+      <c r="I27" s="4" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A27" s="8" t="s">
+    <row r="28" spans="1:9" ht="16.5" customHeight="1">
+      <c r="A28" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B28" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C28" s="8">
         <v>480</v>
       </c>
-      <c r="D27" s="8" t="s">
+      <c r="D28" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="E27" s="8" t="s">
+      <c r="E28" s="8" t="s">
         <v>123</v>
-      </c>
-      <c r="F27" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="G27" s="8"/>
-      <c r="H27" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="I27" s="14" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" ht="33" customHeight="1">
-      <c r="A28" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="C28" s="8">
-        <v>500</v>
-      </c>
-      <c r="D28" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>127</v>
       </c>
       <c r="F28" s="8" t="s">
         <v>124</v>
@@ -3961,128 +3990,126 @@
       <c r="H28" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="I28" s="13" t="s">
+      <c r="I28" s="14" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="33" customHeight="1">
+      <c r="A29" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C29" s="8">
+        <v>500</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="G29" s="8"/>
+      <c r="H29" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="I29" s="13" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="33" customHeight="1">
-      <c r="A29" s="57" t="s">
+    <row r="30" spans="1:9" ht="33" customHeight="1">
+      <c r="A30" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="B29" s="57" t="s">
+      <c r="B30" s="57" t="s">
         <v>10</v>
       </c>
-      <c r="C29" s="57">
+      <c r="C30" s="57">
         <v>900</v>
       </c>
-      <c r="D29" s="57" t="s">
+      <c r="D30" s="57" t="s">
         <v>129</v>
       </c>
-      <c r="E29" s="57" t="s">
+      <c r="E30" s="57" t="s">
         <v>130</v>
       </c>
-      <c r="F29" s="58" t="s">
+      <c r="F30" s="58" t="s">
         <v>329</v>
       </c>
-      <c r="G29" s="57" t="s">
+      <c r="G30" s="57" t="s">
         <v>131</v>
       </c>
-      <c r="H29" s="59" t="s">
+      <c r="H30" s="59" t="s">
         <v>90</v>
       </c>
-      <c r="I29" s="60" t="s">
+      <c r="I30" s="60" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A32" s="94" t="s">
+    <row r="33" spans="1:9" ht="15.75" customHeight="1">
+      <c r="A33" s="96" t="s">
         <v>133</v>
       </c>
-      <c r="B32" s="88"/>
-      <c r="C32" s="88"/>
-      <c r="D32" s="88"/>
-      <c r="E32" s="88"/>
-      <c r="F32" s="88"/>
-      <c r="G32" s="88"/>
-      <c r="H32" s="88"/>
-    </row>
-    <row r="35" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A35" s="36" t="s">
+      <c r="B33" s="90"/>
+      <c r="C33" s="90"/>
+      <c r="D33" s="90"/>
+      <c r="E33" s="90"/>
+      <c r="F33" s="90"/>
+      <c r="G33" s="90"/>
+      <c r="H33" s="90"/>
+    </row>
+    <row r="36" spans="1:9" ht="14.25" customHeight="1">
+      <c r="A36" s="36" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="36" spans="1:9">
-      <c r="A36" s="37" t="s">
+    <row r="37" spans="1:9">
+      <c r="A37" s="37" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="16.5">
-      <c r="A37" s="47" t="s">
+    <row r="38" spans="1:9" ht="16.5">
+      <c r="A38" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="B37" s="47" t="s">
+      <c r="B38" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="C37" s="47" t="s">
+      <c r="C38" s="47" t="s">
         <v>76</v>
       </c>
-      <c r="D37" s="47" t="s">
+      <c r="D38" s="47" t="s">
         <v>77</v>
       </c>
-      <c r="E37" s="47" t="s">
+      <c r="E38" s="47" t="s">
         <v>78</v>
       </c>
-      <c r="F37" s="47" t="s">
+      <c r="F38" s="47" t="s">
         <v>79</v>
       </c>
-      <c r="G37" s="47" t="s">
+      <c r="G38" s="47" t="s">
         <v>80</v>
       </c>
-      <c r="H37" s="47" t="s">
+      <c r="H38" s="47" t="s">
         <v>81</v>
       </c>
-      <c r="I37" s="47" t="s">
+      <c r="I38" s="47" t="s">
         <v>82</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" ht="16.5">
-      <c r="A38" s="35" t="s">
-        <v>28</v>
-      </c>
-      <c r="B38" s="35" t="s">
-        <v>58</v>
-      </c>
-      <c r="C38" s="35" t="s">
-        <v>135</v>
-      </c>
-      <c r="D38" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E38" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="F38" s="35" t="s">
-        <v>136</v>
-      </c>
-      <c r="G38" s="35" t="s">
-        <v>137</v>
-      </c>
-      <c r="H38" s="42" t="s">
-        <v>85</v>
-      </c>
-      <c r="I38" s="52" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="16.5">
       <c r="A39" s="35" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="B39" s="35" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C39" s="35" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D39" s="35" t="s">
         <v>11</v>
@@ -4091,113 +4118,117 @@
         <v>11</v>
       </c>
       <c r="F39" s="35" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="G39" s="35" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H39" s="42" t="s">
         <v>85</v>
       </c>
-      <c r="I39" s="43" t="s">
-        <v>141</v>
+      <c r="I39" s="52" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="16.5">
       <c r="A40" s="35" t="s">
+        <v>59</v>
+      </c>
+      <c r="B40" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="C40" s="35" t="s">
+        <v>138</v>
+      </c>
+      <c r="D40" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="E40" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="F40" s="35" t="s">
+        <v>139</v>
+      </c>
+      <c r="G40" s="35" t="s">
+        <v>140</v>
+      </c>
+      <c r="H40" s="42" t="s">
+        <v>85</v>
+      </c>
+      <c r="I40" s="43" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="16.5">
+      <c r="A41" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="B40" s="35" t="s">
+      <c r="B41" s="35" t="s">
         <v>62</v>
       </c>
-      <c r="C40" s="35" t="s">
+      <c r="C41" s="35" t="s">
         <v>142</v>
       </c>
-      <c r="D40" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E40" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="F40" s="35" t="s">
+      <c r="D41" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="E41" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="F41" s="35" t="s">
         <v>143</v>
       </c>
-      <c r="G40" s="35" t="s">
+      <c r="G41" s="35" t="s">
         <v>144</v>
       </c>
-      <c r="H40" s="44" t="s">
+      <c r="H41" s="44" t="s">
         <v>85</v>
       </c>
-      <c r="I40" s="43"/>
-    </row>
-    <row r="42" spans="1:9">
-      <c r="A42" s="37" t="s">
+      <c r="I41" s="43"/>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="A43" s="37" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="16.5">
-      <c r="A43" s="47" t="s">
+    <row r="44" spans="1:9" ht="16.5">
+      <c r="A44" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="B43" s="47" t="s">
+      <c r="B44" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="C43" s="47" t="s">
+      <c r="C44" s="47" t="s">
         <v>95</v>
       </c>
-      <c r="D43" s="47" t="s">
+      <c r="D44" s="47" t="s">
         <v>96</v>
       </c>
-      <c r="E43" s="47" t="s">
+      <c r="E44" s="47" t="s">
         <v>78</v>
       </c>
-      <c r="F43" s="47" t="s">
+      <c r="F44" s="47" t="s">
         <v>97</v>
       </c>
-      <c r="G43" s="47" t="s">
-        <v>11</v>
-      </c>
-      <c r="H43" s="47" t="s">
+      <c r="G44" s="47" t="s">
+        <v>11</v>
+      </c>
+      <c r="H44" s="47" t="s">
         <v>81</v>
       </c>
-      <c r="I43" s="47" t="s">
+      <c r="I44" s="47" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" ht="16.5">
-      <c r="A44" s="35" t="s">
-        <v>64</v>
-      </c>
-      <c r="B44" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="C44" s="35" t="s">
-        <v>145</v>
-      </c>
-      <c r="D44" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E44" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="F44" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="G44" s="35"/>
-      <c r="H44" s="42" t="s">
-        <v>90</v>
-      </c>
-      <c r="I44" s="43"/>
     </row>
     <row r="45" spans="1:9" ht="16.5">
       <c r="A45" s="35" t="s">
-        <v>40</v>
+        <v>64</v>
       </c>
       <c r="B45" s="35" t="s">
         <v>11</v>
       </c>
       <c r="C45" s="35" t="s">
-        <v>102</v>
+        <v>145</v>
       </c>
       <c r="D45" s="35" t="s">
         <v>11</v>
@@ -4206,25 +4237,23 @@
         <v>11</v>
       </c>
       <c r="F45" s="35" t="s">
-        <v>146</v>
+        <v>11</v>
       </c>
       <c r="G45" s="35"/>
       <c r="H45" s="42" t="s">
         <v>90</v>
       </c>
-      <c r="I45" s="43" t="s">
-        <v>147</v>
-      </c>
+      <c r="I45" s="43"/>
     </row>
     <row r="46" spans="1:9" ht="16.5">
       <c r="A46" s="35" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="B46" s="35" t="s">
-        <v>69</v>
-      </c>
-      <c r="C46" s="49" t="s">
-        <v>321</v>
+        <v>11</v>
+      </c>
+      <c r="C46" s="35" t="s">
+        <v>102</v>
       </c>
       <c r="D46" s="35" t="s">
         <v>11</v>
@@ -4233,88 +4262,88 @@
         <v>11</v>
       </c>
       <c r="F46" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="G46" s="35" t="s">
-        <v>11</v>
-      </c>
+        <v>146</v>
+      </c>
+      <c r="G46" s="35"/>
       <c r="H46" s="42" t="s">
         <v>90</v>
       </c>
-      <c r="I46" s="45" t="s">
+      <c r="I46" s="43" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="16.5">
+      <c r="A47" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="B47" s="35" t="s">
+        <v>69</v>
+      </c>
+      <c r="C47" s="49" t="s">
+        <v>321</v>
+      </c>
+      <c r="D47" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="F47" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="G47" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="H47" s="42" t="s">
+        <v>90</v>
+      </c>
+      <c r="I47" s="45" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="48" spans="1:9">
-      <c r="A48" s="37" t="s">
+    <row r="49" spans="1:9">
+      <c r="A49" s="37" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="49" spans="1:9" ht="16.5">
-      <c r="A49" s="47" t="s">
+    <row r="50" spans="1:9" ht="16.5">
+      <c r="A50" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="B49" s="47" t="s">
+      <c r="B50" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="C49" s="47" t="s">
-        <v>11</v>
-      </c>
-      <c r="D49" s="47" t="s">
-        <v>11</v>
-      </c>
-      <c r="E49" s="47" t="s">
-        <v>11</v>
-      </c>
-      <c r="F49" s="47" t="s">
-        <v>11</v>
-      </c>
-      <c r="G49" s="47" t="s">
-        <v>11</v>
-      </c>
-      <c r="H49" s="47" t="s">
+      <c r="C50" s="47" t="s">
+        <v>11</v>
+      </c>
+      <c r="D50" s="47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E50" s="47" t="s">
+        <v>11</v>
+      </c>
+      <c r="F50" s="47" t="s">
+        <v>11</v>
+      </c>
+      <c r="G50" s="47" t="s">
+        <v>11</v>
+      </c>
+      <c r="H50" s="47" t="s">
         <v>81</v>
       </c>
-      <c r="I49" s="47" t="s">
+      <c r="I50" s="47" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" ht="16.5">
-      <c r="A50" s="35" t="s">
-        <v>38</v>
-      </c>
-      <c r="B50" s="35" t="s">
-        <v>71</v>
-      </c>
-      <c r="C50" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="D50" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E50" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="F50" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="G50" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="H50" s="42" t="s">
-        <v>151</v>
-      </c>
-      <c r="I50" s="43"/>
     </row>
     <row r="51" spans="1:9" ht="16.5">
       <c r="A51" s="35" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B51" s="35" t="s">
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="C51" s="35" t="s">
-        <v>101</v>
+        <v>11</v>
       </c>
       <c r="D51" s="35" t="s">
         <v>11</v>
@@ -4325,23 +4354,23 @@
       <c r="F51" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="G51" s="35"/>
+      <c r="G51" s="35" t="s">
+        <v>11</v>
+      </c>
       <c r="H51" s="42" t="s">
-        <v>148</v>
-      </c>
-      <c r="I51" s="43" t="s">
-        <v>149</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="I51" s="43"/>
     </row>
     <row r="52" spans="1:9" ht="16.5">
       <c r="A52" s="35" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B52" s="35" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="C52" s="35" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D52" s="35" t="s">
         <v>11</v>
@@ -4356,19 +4385,46 @@
       <c r="H52" s="42" t="s">
         <v>148</v>
       </c>
-      <c r="I52" s="43"/>
+      <c r="I52" s="43" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" ht="16.5">
+      <c r="A53" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="B53" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="C53" s="35" t="s">
+        <v>103</v>
+      </c>
+      <c r="D53" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="E53" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="F53" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="G53" s="35"/>
+      <c r="H53" s="42" t="s">
+        <v>148</v>
+      </c>
+      <c r="I53" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A33:H33"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A26:H26"/>
     <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A20:H20"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
-  <conditionalFormatting sqref="H4:H9 H11:H13 H15:H16 H18 H20:H24 H26:H28">
+  <conditionalFormatting sqref="H4:H9 H16:H17 H19 H21:H25 H27:H29 H11:H14">
     <cfRule type="cellIs" dxfId="19" priority="15" operator="equal">
       <formula>"✅"</formula>
     </cfRule>
@@ -4376,7 +4432,7 @@
       <formula>"⚠️"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H14">
+  <conditionalFormatting sqref="H15">
     <cfRule type="cellIs" dxfId="17" priority="3" operator="equal">
       <formula>"✅"</formula>
     </cfRule>
@@ -4384,7 +4440,7 @@
       <formula>"⚠️"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H17">
+  <conditionalFormatting sqref="H18">
     <cfRule type="cellIs" dxfId="15" priority="1" operator="equal">
       <formula>"✅"</formula>
     </cfRule>
@@ -4413,24 +4469,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="87" t="s">
+      <c r="A1" s="89" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" s="89" t="s">
+      <c r="A2" s="91" t="s">
         <v>153</v>
       </c>
-      <c r="B2" s="88"/>
-      <c r="C2" s="88"/>
-      <c r="D2" s="88"/>
-      <c r="E2" s="88"/>
-      <c r="F2" s="88"/>
+      <c r="B2" s="90"/>
+      <c r="C2" s="90"/>
+      <c r="D2" s="90"/>
+      <c r="E2" s="90"/>
+      <c r="F2" s="90"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -4635,14 +4691,30 @@
       <c r="F13" s="85"/>
     </row>
     <row r="14" spans="1:8" s="62" customFormat="1" ht="16.5">
-      <c r="A14" s="79"/>
-      <c r="B14" s="79"/>
-      <c r="C14" s="79"/>
-      <c r="D14" s="82"/>
-      <c r="E14" s="84"/>
-      <c r="F14" s="79"/>
+      <c r="A14" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>388</v>
+      </c>
+      <c r="D14" s="71">
+        <f>109000-D15</f>
+        <v>49000</v>
+      </c>
+      <c r="E14" s="71">
+        <f>D14</f>
+        <v>49000</v>
+      </c>
+      <c r="F14" s="70" t="s">
+        <v>393</v>
+      </c>
       <c r="G14" s="75"/>
-      <c r="H14" s="76"/>
+      <c r="H14" s="76" t="s">
+        <v>389</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="16.5" customHeight="1">
       <c r="A15" s="8" t="s">
@@ -4960,23 +5032,23 @@
       <c r="C31" s="72"/>
       <c r="D31" s="72">
         <f>SUM(D4:D30)</f>
-        <v>534100</v>
+        <v>583100</v>
       </c>
       <c r="E31" s="72">
         <f>SUM(E4:E30)</f>
-        <v>633200</v>
+        <v>682200</v>
       </c>
       <c r="F31" s="72"/>
     </row>
     <row r="32" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A32" s="89" t="s">
+      <c r="A32" s="91" t="s">
         <v>154</v>
       </c>
-      <c r="B32" s="88"/>
-      <c r="C32" s="88"/>
-      <c r="D32" s="88"/>
-      <c r="E32" s="88"/>
-      <c r="F32" s="88"/>
+      <c r="B32" s="90"/>
+      <c r="C32" s="90"/>
+      <c r="D32" s="90"/>
+      <c r="E32" s="90"/>
+      <c r="F32" s="90"/>
     </row>
     <row r="35" spans="1:8" ht="14.25">
       <c r="A35" s="36" t="s">
@@ -5173,11 +5245,11 @@
       <c r="C46" s="72"/>
       <c r="D46" s="72">
         <f>SUM(D12:D45)</f>
-        <v>1043100</v>
+        <v>1141100</v>
       </c>
       <c r="E46" s="72">
         <f>SUM(E12:E45)</f>
-        <v>1294300</v>
+        <v>1392300</v>
       </c>
       <c r="F46" s="72"/>
     </row>
@@ -5250,28 +5322,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="87" t="s">
+      <c r="A1" s="89" t="s">
         <v>157</v>
       </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
-      <c r="A3" s="96" t="s">
+      <c r="A3" s="98" t="s">
         <v>158</v>
       </c>
-      <c r="B3" s="88"/>
-      <c r="C3" s="88"/>
-      <c r="D3" s="88"/>
-      <c r="E3" s="88"/>
-      <c r="F3" s="88"/>
-      <c r="G3" s="88"/>
-      <c r="H3" s="88"/>
+      <c r="B3" s="90"/>
+      <c r="C3" s="90"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="90"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -5586,10 +5658,10 @@
       </c>
     </row>
     <row r="16" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A16" s="97" t="s">
+      <c r="A16" s="99" t="s">
         <v>198</v>
       </c>
-      <c r="B16" s="98"/>
+      <c r="B16" s="100"/>
       <c r="C16" s="8">
         <f>SUM(C5:C15)</f>
         <v>35</v>
@@ -5602,21 +5674,21 @@
         <f>SUM(E5:E15)</f>
         <v>35</v>
       </c>
-      <c r="F16" s="97" t="s">
+      <c r="F16" s="99" t="s">
         <v>199</v>
       </c>
-      <c r="G16" s="98"/>
+      <c r="G16" s="100"/>
       <c r="H16" s="21"/>
     </row>
     <row r="17" spans="1:8" ht="15" customHeight="1">
-      <c r="A17" s="88"/>
-      <c r="B17" s="88"/>
-      <c r="C17" s="88"/>
-      <c r="D17" s="88"/>
-      <c r="E17" s="88"/>
-      <c r="F17" s="88"/>
-      <c r="G17" s="88"/>
-      <c r="H17" s="88"/>
+      <c r="A17" s="90"/>
+      <c r="B17" s="90"/>
+      <c r="C17" s="90"/>
+      <c r="D17" s="90"/>
+      <c r="E17" s="90"/>
+      <c r="F17" s="90"/>
+      <c r="G17" s="90"/>
+      <c r="H17" s="90"/>
     </row>
     <row r="18" spans="1:8" ht="15" customHeight="1">
       <c r="A18" s="33" t="s">
@@ -6013,25 +6085,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="87" t="s">
+      <c r="A1" s="89" t="s">
         <v>223</v>
       </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
-      <c r="A3" s="96" t="s">
+      <c r="A3" s="98" t="s">
         <v>224</v>
       </c>
-      <c r="B3" s="88"/>
-      <c r="C3" s="88"/>
-      <c r="D3" s="88"/>
-      <c r="E3" s="88"/>
+      <c r="B3" s="90"/>
+      <c r="C3" s="90"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -6119,16 +6191,16 @@
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
-      <c r="A11" s="96" t="s">
+      <c r="A11" s="98" t="s">
         <v>244</v>
       </c>
-      <c r="B11" s="88"/>
-      <c r="C11" s="88"/>
-      <c r="D11" s="88"/>
-      <c r="E11" s="88"/>
-      <c r="F11" s="88"/>
-      <c r="G11" s="88"/>
-      <c r="H11" s="88"/>
+      <c r="B11" s="90"/>
+      <c r="C11" s="90"/>
+      <c r="D11" s="90"/>
+      <c r="E11" s="90"/>
+      <c r="F11" s="90"/>
+      <c r="G11" s="90"/>
+      <c r="H11" s="90"/>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
       <c r="A12" s="1" t="s">
@@ -6284,24 +6356,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="87" t="s">
+      <c r="A1" s="89" t="s">
         <v>251</v>
       </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1">
-      <c r="A3" s="96" t="s">
+      <c r="A3" s="98" t="s">
         <v>252</v>
       </c>
-      <c r="B3" s="88"/>
-      <c r="C3" s="88"/>
-      <c r="D3" s="88"/>
-      <c r="E3" s="88"/>
-      <c r="F3" s="88"/>
+      <c r="B3" s="90"/>
+      <c r="C3" s="90"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1">
       <c r="A4" s="5" t="s">
@@ -6384,10 +6456,10 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A8" s="101" t="s">
+      <c r="A8" s="103" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="92"/>
+      <c r="B8" s="94"/>
       <c r="C8" s="35">
         <v>500</v>
       </c>
@@ -6422,18 +6494,18 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1">
-      <c r="A10" s="99"/>
-      <c r="B10" s="91"/>
-      <c r="C10" s="91"/>
-      <c r="D10" s="91"/>
-      <c r="E10" s="91"/>
-      <c r="F10" s="92"/>
+      <c r="A10" s="101"/>
+      <c r="B10" s="93"/>
+      <c r="C10" s="93"/>
+      <c r="D10" s="93"/>
+      <c r="E10" s="93"/>
+      <c r="F10" s="94"/>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1">
-      <c r="A11" s="97" t="s">
+      <c r="A11" s="99" t="s">
         <v>198</v>
       </c>
-      <c r="B11" s="92"/>
+      <c r="B11" s="94"/>
       <c r="C11" s="34">
         <f>SUM(C5:C9)</f>
         <v>4180</v>
@@ -6494,14 +6566,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="15" customHeight="1">
-      <c r="A17" s="100" t="s">
+      <c r="A17" s="102" t="s">
         <v>266</v>
       </c>
-      <c r="B17" s="91"/>
-      <c r="C17" s="91"/>
-      <c r="D17" s="91"/>
-      <c r="E17" s="91"/>
-      <c r="F17" s="92"/>
+      <c r="B17" s="93"/>
+      <c r="C17" s="93"/>
+      <c r="D17" s="93"/>
+      <c r="E17" s="93"/>
+      <c r="F17" s="94"/>
     </row>
     <row r="18" spans="1:6" ht="15" customHeight="1">
       <c r="A18" s="11" t="s">
@@ -6552,14 +6624,14 @@
       </c>
     </row>
     <row r="23" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A23" s="100" t="s">
+      <c r="A23" s="102" t="s">
         <v>164</v>
       </c>
-      <c r="B23" s="91"/>
-      <c r="C23" s="91"/>
-      <c r="D23" s="91"/>
-      <c r="E23" s="91"/>
-      <c r="F23" s="92"/>
+      <c r="B23" s="93"/>
+      <c r="C23" s="93"/>
+      <c r="D23" s="93"/>
+      <c r="E23" s="93"/>
+      <c r="F23" s="94"/>
     </row>
     <row r="24" spans="1:6" ht="16.5" customHeight="1">
       <c r="A24" s="8" t="s">
@@ -6731,28 +6803,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="87" t="s">
+      <c r="A1" s="89" t="s">
         <v>282</v>
       </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" s="89" t="s">
+      <c r="A2" s="91" t="s">
         <v>283</v>
       </c>
-      <c r="B2" s="88"/>
-      <c r="C2" s="88"/>
-      <c r="D2" s="88"/>
-      <c r="E2" s="88"/>
-      <c r="F2" s="88"/>
-      <c r="G2" s="88"/>
-      <c r="H2" s="88"/>
+      <c r="B2" s="90"/>
+      <c r="C2" s="90"/>
+      <c r="D2" s="90"/>
+      <c r="E2" s="90"/>
+      <c r="F2" s="90"/>
+      <c r="G2" s="90"/>
+      <c r="H2" s="90"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -7129,14 +7201,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="104" t="s">
         <v>296</v>
       </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
     </row>
     <row r="2" spans="1:6" ht="24.95" customHeight="1">
       <c r="A2" s="9" t="s">

</xml_diff>

<commit_message>
auto: add 03-Memory (1), delete 01-Projects (1), modify 01-Projects (1), modify 03-Memory (2)
</commit_message>
<xml_diff>
--- a/01-Projects/family-hub/credit-card-management/信用卡主控表.xlsx
+++ b/01-Projects/family-hub/credit-card-management/信用卡主控表.xlsx
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="980" uniqueCount="394">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="995" uniqueCount="402">
   <si>
     <t>信用卡卡片总览 — 韩伟</t>
   </si>
@@ -500,9 +500,6 @@
   </si>
   <si>
     <t>📋待办</t>
-  </si>
-  <si>
-    <t>0账单还款日历 — 账单日=还款日，当天还清</t>
   </si>
   <si>
     <t>规则：账单日 = 还款日，当天还清 → 征信报告显示0账单 | 操作：手机日历设提醒 → 当天云闪付还款 → Excel打✅</t>
@@ -1374,10 +1371,6 @@
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
-    <t>APP可以领取 30元券</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
     <t>交通-2</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
@@ -1391,6 +1384,47 @@
   </si>
   <si>
     <t>刷6笔数抵扣</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>0账单还款日历1 — 账单日=还款日，当天还清</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>0账单还款日历2 — 账单日=还款日，当天还清</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>交通2</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>工商2</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>南航卡</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>不支持修改账单日！</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>APP可以领取 30元券
+账单日 根据1卡走</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>自动兑换里程</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>农行</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>南航 体检了申请</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
@@ -1811,7 +1845,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2049,6 +2083,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="58" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2077,14 +2115,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="58" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="21">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2130,6 +2166,14 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFFFC7CE"/>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2558,15 +2602,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="91" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
+      <c r="B1" s="92"/>
+      <c r="C1" s="92"/>
+      <c r="D1" s="92"/>
+      <c r="E1" s="92"/>
+      <c r="F1" s="92"/>
+      <c r="G1" s="92"/>
     </row>
     <row r="2" spans="1:8" ht="24.95" customHeight="1">
       <c r="A2" s="1" t="s">
@@ -2614,10 +2658,10 @@
         <v>0</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="H3" s="53" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="16.5" customHeight="1">
@@ -2643,7 +2687,7 @@
         <v>14</v>
       </c>
       <c r="H4" s="26" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="16.5" customHeight="1">
@@ -2669,7 +2713,7 @@
         <v>17</v>
       </c>
       <c r="H5" s="26" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="16.5" customHeight="1">
@@ -2766,7 +2810,7 @@
         <v>50000</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H9" s="26"/>
     </row>
@@ -2816,7 +2860,7 @@
         <v>26000</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="H11" s="26"/>
     </row>
@@ -2891,7 +2935,7 @@
         <v>39</v>
       </c>
       <c r="H14" s="26" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="16.5" customHeight="1">
@@ -2989,16 +3033,16 @@
         <v>54</v>
       </c>
       <c r="H18" s="26" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A19" s="95" t="s">
+      <c r="A19" s="97" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="93"/>
-      <c r="C19" s="93"/>
-      <c r="D19" s="94"/>
+      <c r="B19" s="95"/>
+      <c r="C19" s="95"/>
+      <c r="D19" s="96"/>
       <c r="E19" s="3">
         <f>SUM(E3:E18)</f>
         <v>831000</v>
@@ -3011,26 +3055,26 @@
       <c r="H19" s="26"/>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A21" s="91" t="s">
+      <c r="A21" s="93" t="s">
         <v>56</v>
       </c>
-      <c r="B21" s="90"/>
-      <c r="C21" s="90"/>
-      <c r="D21" s="90"/>
-      <c r="E21" s="90"/>
-      <c r="F21" s="90"/>
-      <c r="G21" s="90"/>
+      <c r="B21" s="92"/>
+      <c r="C21" s="92"/>
+      <c r="D21" s="92"/>
+      <c r="E21" s="92"/>
+      <c r="F21" s="92"/>
+      <c r="G21" s="92"/>
     </row>
     <row r="24" spans="1:8" ht="21" customHeight="1">
-      <c r="A24" s="89" t="s">
+      <c r="A24" s="91" t="s">
         <v>57</v>
       </c>
-      <c r="B24" s="90"/>
-      <c r="C24" s="90"/>
-      <c r="D24" s="90"/>
-      <c r="E24" s="90"/>
-      <c r="F24" s="90"/>
-      <c r="G24" s="90"/>
+      <c r="B24" s="92"/>
+      <c r="C24" s="92"/>
+      <c r="D24" s="92"/>
+      <c r="E24" s="92"/>
+      <c r="F24" s="92"/>
+      <c r="G24" s="92"/>
     </row>
     <row r="25" spans="1:8" ht="21" customHeight="1">
       <c r="A25" s="38" t="s">
@@ -3066,7 +3110,7 @@
         <v>28</v>
       </c>
       <c r="C26" s="50" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D26" s="35" t="s">
         <v>11</v>
@@ -3078,10 +3122,10 @@
         <v>11000</v>
       </c>
       <c r="G26" s="50" t="s">
+        <v>322</v>
+      </c>
+      <c r="H26" s="53" t="s">
         <v>323</v>
-      </c>
-      <c r="H26" s="53" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="31.5" customHeight="1">
@@ -3147,7 +3191,7 @@
         <v>11</v>
       </c>
       <c r="H29" s="53" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="16.5" customHeight="1">
@@ -3195,7 +3239,7 @@
         <v>11</v>
       </c>
       <c r="H31" s="74" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="30.75" customHeight="1">
@@ -3317,12 +3361,12 @@
       <c r="H37" s="53"/>
     </row>
     <row r="38" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A38" s="92" t="s">
+      <c r="A38" s="94" t="s">
         <v>73</v>
       </c>
-      <c r="B38" s="93"/>
-      <c r="C38" s="93"/>
-      <c r="D38" s="94"/>
+      <c r="B38" s="95"/>
+      <c r="C38" s="95"/>
+      <c r="D38" s="96"/>
       <c r="E38" s="41">
         <f>SUM(E26:E37)</f>
         <v>44000</v>
@@ -3369,28 +3413,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="91" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
+      <c r="B1" s="92"/>
+      <c r="C1" s="92"/>
+      <c r="D1" s="92"/>
+      <c r="E1" s="92"/>
+      <c r="F1" s="92"/>
+      <c r="G1" s="92"/>
+      <c r="H1" s="92"/>
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1">
-      <c r="A3" s="97" t="s">
+      <c r="A3" s="99" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="93"/>
-      <c r="C3" s="93"/>
-      <c r="D3" s="93"/>
-      <c r="E3" s="93"/>
-      <c r="F3" s="93"/>
-      <c r="G3" s="93"/>
-      <c r="H3" s="94"/>
+      <c r="B3" s="95"/>
+      <c r="C3" s="95"/>
+      <c r="D3" s="95"/>
+      <c r="E3" s="95"/>
+      <c r="F3" s="95"/>
+      <c r="G3" s="95"/>
+      <c r="H3" s="96"/>
       <c r="I3" s="24"/>
     </row>
     <row r="4" spans="1:9" ht="33" customHeight="1">
@@ -3506,7 +3550,7 @@
         <v>90</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="26.25" customHeight="1">
@@ -3550,16 +3594,16 @@
       <c r="I9" s="13"/>
     </row>
     <row r="10" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A10" s="97" t="s">
+      <c r="A10" s="99" t="s">
         <v>94</v>
       </c>
-      <c r="B10" s="93"/>
-      <c r="C10" s="93"/>
-      <c r="D10" s="93"/>
-      <c r="E10" s="93"/>
-      <c r="F10" s="93"/>
-      <c r="G10" s="93"/>
-      <c r="H10" s="94"/>
+      <c r="B10" s="95"/>
+      <c r="C10" s="95"/>
+      <c r="D10" s="95"/>
+      <c r="E10" s="95"/>
+      <c r="F10" s="95"/>
+      <c r="G10" s="95"/>
+      <c r="H10" s="96"/>
       <c r="I10" s="24"/>
     </row>
     <row r="11" spans="1:9" ht="16.5" customHeight="1">
@@ -3622,13 +3666,13 @@
     </row>
     <row r="13" spans="1:9" s="87" customFormat="1" ht="31.5" customHeight="1">
       <c r="A13" s="88" t="s">
+        <v>388</v>
+      </c>
+      <c r="B13" s="88" t="s">
+        <v>389</v>
+      </c>
+      <c r="C13" s="88" t="s">
         <v>390</v>
-      </c>
-      <c r="B13" s="88" t="s">
-        <v>391</v>
-      </c>
-      <c r="C13" s="88" t="s">
-        <v>392</v>
       </c>
       <c r="D13" s="88">
         <v>6</v>
@@ -3636,7 +3680,7 @@
       <c r="E13" s="88">
         <v>0</v>
       </c>
-      <c r="F13" s="105">
+      <c r="F13" s="90">
         <v>46265</v>
       </c>
       <c r="G13" s="88"/>
@@ -3792,16 +3836,16 @@
       <c r="I19" s="13"/>
     </row>
     <row r="20" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A20" s="97" t="s">
+      <c r="A20" s="99" t="s">
         <v>109</v>
       </c>
-      <c r="B20" s="93"/>
-      <c r="C20" s="93"/>
-      <c r="D20" s="93"/>
-      <c r="E20" s="93"/>
-      <c r="F20" s="93"/>
-      <c r="G20" s="93"/>
-      <c r="H20" s="94"/>
+      <c r="B20" s="95"/>
+      <c r="C20" s="95"/>
+      <c r="D20" s="95"/>
+      <c r="E20" s="95"/>
+      <c r="F20" s="95"/>
+      <c r="G20" s="95"/>
+      <c r="H20" s="96"/>
       <c r="I20" s="24"/>
     </row>
     <row r="21" spans="1:9" ht="16.5" customHeight="1">
@@ -3926,16 +3970,16 @@
       <c r="I25" s="13"/>
     </row>
     <row r="26" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A26" s="97" t="s">
+      <c r="A26" s="99" t="s">
         <v>117</v>
       </c>
-      <c r="B26" s="93"/>
-      <c r="C26" s="93"/>
-      <c r="D26" s="93"/>
-      <c r="E26" s="93"/>
-      <c r="F26" s="93"/>
-      <c r="G26" s="93"/>
-      <c r="H26" s="94"/>
+      <c r="B26" s="95"/>
+      <c r="C26" s="95"/>
+      <c r="D26" s="95"/>
+      <c r="E26" s="95"/>
+      <c r="F26" s="95"/>
+      <c r="G26" s="95"/>
+      <c r="H26" s="96"/>
       <c r="I26" s="24"/>
     </row>
     <row r="27" spans="1:9" ht="16.5" customHeight="1">
@@ -3991,7 +4035,7 @@
         <v>11</v>
       </c>
       <c r="I28" s="14" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="33" customHeight="1">
@@ -4038,7 +4082,7 @@
         <v>130</v>
       </c>
       <c r="F30" s="58" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G30" s="57" t="s">
         <v>131</v>
@@ -4051,16 +4095,16 @@
       </c>
     </row>
     <row r="33" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A33" s="96" t="s">
+      <c r="A33" s="98" t="s">
         <v>133</v>
       </c>
-      <c r="B33" s="90"/>
-      <c r="C33" s="90"/>
-      <c r="D33" s="90"/>
-      <c r="E33" s="90"/>
-      <c r="F33" s="90"/>
-      <c r="G33" s="90"/>
-      <c r="H33" s="90"/>
+      <c r="B33" s="92"/>
+      <c r="C33" s="92"/>
+      <c r="D33" s="92"/>
+      <c r="E33" s="92"/>
+      <c r="F33" s="92"/>
+      <c r="G33" s="92"/>
+      <c r="H33" s="92"/>
     </row>
     <row r="36" spans="1:9" ht="14.25" customHeight="1">
       <c r="A36" s="36" t="s">
@@ -4127,7 +4171,7 @@
         <v>85</v>
       </c>
       <c r="I39" s="52" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="16.5">
@@ -4280,7 +4324,7 @@
         <v>69</v>
       </c>
       <c r="C47" s="49" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D47" s="35" t="s">
         <v>11</v>
@@ -4298,7 +4342,7 @@
         <v>90</v>
       </c>
       <c r="I47" s="45" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -4425,26 +4469,26 @@
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <conditionalFormatting sqref="H4:H9 H16:H17 H19 H21:H25 H27:H29 H11:H14">
-    <cfRule type="cellIs" dxfId="19" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="15" operator="equal">
       <formula>"✅"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="16" operator="equal">
       <formula>"⚠️"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H15">
-    <cfRule type="cellIs" dxfId="17" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="3" operator="equal">
       <formula>"✅"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="4" operator="equal">
       <formula>"⚠️"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H18">
-    <cfRule type="cellIs" dxfId="15" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="1" operator="equal">
       <formula>"✅"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="2" operator="equal">
       <formula>"⚠️"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4457,7 +4501,7 @@
   <sheetPr>
     <tabColor rgb="FF70AD47"/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="8" style="30" customWidth="1"/>
@@ -4469,28 +4513,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="91" t="s">
+        <v>392</v>
+      </c>
+      <c r="B1" s="92"/>
+      <c r="C1" s="92"/>
+      <c r="D1" s="92"/>
+      <c r="E1" s="92"/>
+      <c r="F1" s="92"/>
+    </row>
+    <row r="2" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A2" s="93" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-    </row>
-    <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" s="91" t="s">
-        <v>153</v>
-      </c>
-      <c r="B2" s="90"/>
-      <c r="C2" s="90"/>
-      <c r="D2" s="90"/>
-      <c r="E2" s="90"/>
-      <c r="F2" s="90"/>
+      <c r="B2" s="92"/>
+      <c r="C2" s="92"/>
+      <c r="D2" s="92"/>
+      <c r="E2" s="92"/>
+      <c r="F2" s="92"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>2</v>
@@ -4499,10 +4543,10 @@
         <v>3</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>82</v>
@@ -4510,7 +4554,7 @@
     </row>
     <row r="4" spans="1:8" ht="16.5" customHeight="1">
       <c r="A4" s="57" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B4" s="57" t="s">
         <v>9</v>
@@ -4525,12 +4569,12 @@
         <v>0</v>
       </c>
       <c r="F4" s="57" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="16.5" customHeight="1">
       <c r="A5" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>12</v>
@@ -4545,18 +4589,18 @@
         <v>10000</v>
       </c>
       <c r="F5" s="70" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="H5" s="62" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="16.5" customHeight="1">
       <c r="A6" s="69" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>69</v>
@@ -4568,15 +4612,15 @@
         <v>20100</v>
       </c>
       <c r="F6" s="70" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="H6" s="62" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="16.5" customHeight="1">
       <c r="A7" s="69" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>15</v>
@@ -4591,18 +4635,18 @@
         <v>27000</v>
       </c>
       <c r="F7" s="70" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="H7" s="62" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="62" customFormat="1" ht="16.5">
       <c r="A8" s="79" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B8" s="79" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C8" s="82" t="s">
         <v>62</v>
@@ -4617,7 +4661,7 @@
     </row>
     <row r="9" spans="1:8" ht="16.5" customHeight="1">
       <c r="A9" s="69" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B9" s="8" t="s">
         <v>44</v>
@@ -4632,10 +4676,10 @@
         <v>71000</v>
       </c>
       <c r="F9" s="70" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="H9" s="62" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="10" spans="1:8" s="62" customFormat="1" ht="16.5" customHeight="1">
@@ -4658,13 +4702,13 @@
     </row>
     <row r="12" spans="1:8" ht="33">
       <c r="A12" s="79" t="s">
+        <v>364</v>
+      </c>
+      <c r="B12" s="63" t="s">
         <v>365</v>
       </c>
-      <c r="B12" s="63" t="s">
-        <v>366</v>
-      </c>
       <c r="C12" s="63" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="D12" s="35">
         <v>46000</v>
@@ -4673,13 +4717,13 @@
         <v>110000</v>
       </c>
       <c r="F12" s="51" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="G12" s="67" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="H12" s="76" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -4690,7 +4734,7 @@
       <c r="E13" s="85"/>
       <c r="F13" s="85"/>
     </row>
-    <row r="14" spans="1:8" s="62" customFormat="1" ht="16.5">
+    <row r="14" spans="1:8" ht="16.5" customHeight="1">
       <c r="A14" s="8" t="s">
         <v>23</v>
       </c>
@@ -4698,570 +4742,668 @@
         <v>21</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>388</v>
+        <v>125</v>
       </c>
       <c r="D14" s="71">
-        <f>109000-D15</f>
-        <v>49000</v>
+        <v>60000</v>
       </c>
       <c r="E14" s="71">
-        <f>D14</f>
-        <v>49000</v>
+        <v>60000</v>
       </c>
       <c r="F14" s="70" t="s">
-        <v>393</v>
-      </c>
-      <c r="G14" s="75"/>
-      <c r="H14" s="76" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A15" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="D15" s="71">
-        <v>60000</v>
-      </c>
-      <c r="E15" s="71">
-        <v>60000</v>
-      </c>
-      <c r="F15" s="70" t="s">
+        <v>341</v>
+      </c>
+      <c r="G14" s="67"/>
+      <c r="H14" s="81" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" s="62" customFormat="1" ht="16.5" customHeight="1">
+      <c r="A15" s="79"/>
+      <c r="B15" s="79"/>
+      <c r="C15" s="79"/>
+      <c r="D15" s="79"/>
+      <c r="E15" s="79"/>
+      <c r="F15" s="79"/>
+      <c r="G15" s="75"/>
+      <c r="H15" s="81"/>
+    </row>
+    <row r="16" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A16" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="8">
+        <v>7000</v>
+      </c>
+      <c r="E16" s="8">
+        <v>7000</v>
+      </c>
+      <c r="F16" s="70" t="s">
         <v>342</v>
       </c>
-      <c r="G15" s="67"/>
-      <c r="H15" s="81" t="s">
+    </row>
+    <row r="17" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A17" s="65" t="s">
+        <v>319</v>
+      </c>
+      <c r="B17" s="65" t="s">
         <v>373</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" s="62" customFormat="1" ht="16.5" customHeight="1">
-      <c r="A16" s="79"/>
-      <c r="B16" s="79"/>
-      <c r="C16" s="79"/>
-      <c r="D16" s="79"/>
-      <c r="E16" s="79"/>
-      <c r="F16" s="79"/>
-      <c r="G16" s="75"/>
-      <c r="H16" s="81"/>
-    </row>
-    <row r="17" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A17" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="D17" s="8">
-        <v>7000</v>
-      </c>
-      <c r="E17" s="8">
-        <v>7000</v>
-      </c>
-      <c r="F17" s="70" t="s">
+      <c r="C17" s="65" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" s="65">
+        <v>0</v>
+      </c>
+      <c r="E17" s="65">
+        <v>5100</v>
+      </c>
+      <c r="F17" s="80" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A18" s="65" t="s">
-        <v>320</v>
-      </c>
-      <c r="B18" s="65" t="s">
-        <v>374</v>
-      </c>
-      <c r="C18" s="65" t="s">
-        <v>48</v>
-      </c>
-      <c r="D18" s="65">
-        <v>0</v>
-      </c>
-      <c r="E18" s="65">
-        <v>5100</v>
-      </c>
-      <c r="F18" s="80" t="s">
+    <row r="18" spans="1:8" ht="33">
+      <c r="A18" s="48" t="s">
+        <v>319</v>
+      </c>
+      <c r="B18" s="63" t="s">
+        <v>367</v>
+      </c>
+      <c r="C18" s="73" t="s">
+        <v>360</v>
+      </c>
+      <c r="D18" s="77">
+        <v>33000</v>
+      </c>
+      <c r="E18" s="77">
+        <v>33000</v>
+      </c>
+      <c r="F18" s="48" t="s">
+        <v>316</v>
+      </c>
+      <c r="G18" s="67" t="s">
+        <v>354</v>
+      </c>
+      <c r="H18" s="76" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" s="62" customFormat="1" ht="16.5">
+      <c r="A19" s="79"/>
+      <c r="B19" s="79"/>
+      <c r="C19" s="84"/>
+      <c r="D19" s="82"/>
+      <c r="E19" s="82"/>
+      <c r="F19" s="79"/>
+      <c r="G19" s="75"/>
+      <c r="H19" s="76"/>
+    </row>
+    <row r="20" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A20" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20" s="71">
+        <v>26000</v>
+      </c>
+      <c r="E20" s="71">
+        <v>26000</v>
+      </c>
+      <c r="F20" s="70" t="s">
         <v>344</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" ht="33">
-      <c r="A19" s="48" t="s">
-        <v>320</v>
-      </c>
-      <c r="B19" s="63" t="s">
-        <v>368</v>
-      </c>
-      <c r="C19" s="73" t="s">
-        <v>361</v>
-      </c>
-      <c r="D19" s="77">
-        <v>33000</v>
-      </c>
-      <c r="E19" s="77">
-        <v>33000</v>
-      </c>
-      <c r="F19" s="48" t="s">
-        <v>317</v>
-      </c>
-      <c r="G19" s="67" t="s">
-        <v>355</v>
-      </c>
-      <c r="H19" s="76" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" s="62" customFormat="1" ht="16.5">
-      <c r="A20" s="79"/>
-      <c r="B20" s="79"/>
-      <c r="C20" s="84"/>
-      <c r="D20" s="82"/>
-      <c r="E20" s="82"/>
-      <c r="F20" s="79"/>
-      <c r="G20" s="75"/>
-      <c r="H20" s="76"/>
+      <c r="H20" s="62" t="s">
+        <v>382</v>
+      </c>
     </row>
     <row r="21" spans="1:8" ht="16.5" customHeight="1">
       <c r="A21" s="8" t="s">
-        <v>319</v>
+        <v>381</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D21" s="71">
-        <v>26000</v>
-      </c>
-      <c r="E21" s="71">
-        <v>26000</v>
-      </c>
-      <c r="F21" s="70" t="s">
+        <v>33</v>
+      </c>
+      <c r="D21" s="69">
+        <v>19000</v>
+      </c>
+      <c r="E21" s="69">
+        <v>19000</v>
+      </c>
+      <c r="F21" s="63" t="s">
         <v>345</v>
       </c>
       <c r="H21" s="62" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="16.5" customHeight="1">
       <c r="A22" s="8" t="s">
-        <v>382</v>
+        <v>37</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="D22" s="69">
-        <v>19000</v>
-      </c>
-      <c r="E22" s="69">
-        <v>19000</v>
+        <v>366</v>
+      </c>
+      <c r="D22" s="8">
+        <v>16000</v>
+      </c>
+      <c r="E22" s="8">
+        <v>35000</v>
       </c>
       <c r="F22" s="63" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" s="62" customFormat="1" ht="16.5">
+      <c r="A23" s="63" t="s">
+        <v>330</v>
+      </c>
+      <c r="B23" s="63" t="s">
+        <v>370</v>
+      </c>
+      <c r="C23" s="64" t="s">
+        <v>60</v>
+      </c>
+      <c r="D23" s="77">
+        <v>13000</v>
+      </c>
+      <c r="E23" s="77">
+        <v>13000</v>
+      </c>
+      <c r="F23" s="64"/>
+    </row>
+    <row r="24" spans="1:8" s="62" customFormat="1" ht="16.5">
+      <c r="A24" s="63"/>
+      <c r="B24" s="63"/>
+      <c r="C24" s="64"/>
+      <c r="D24" s="82"/>
+      <c r="E24" s="82"/>
+      <c r="F24" s="64"/>
+    </row>
+    <row r="25" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A25" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="D25" s="71">
+        <v>50000</v>
+      </c>
+      <c r="E25" s="71">
+        <v>50000</v>
+      </c>
+      <c r="F25" s="70" t="s">
         <v>346</v>
       </c>
-      <c r="H22" s="62" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A23" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>367</v>
-      </c>
-      <c r="D23" s="8">
-        <v>16000</v>
-      </c>
-      <c r="E23" s="8">
-        <v>35000</v>
-      </c>
-      <c r="F23" s="63" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" s="62" customFormat="1" ht="16.5">
-      <c r="A24" s="63" t="s">
-        <v>331</v>
-      </c>
-      <c r="B24" s="63" t="s">
-        <v>371</v>
-      </c>
-      <c r="C24" s="64" t="s">
-        <v>60</v>
-      </c>
-      <c r="D24" s="77">
-        <v>13000</v>
-      </c>
-      <c r="E24" s="77">
-        <v>13000</v>
-      </c>
-      <c r="F24" s="64"/>
-    </row>
-    <row r="25" spans="1:8" s="62" customFormat="1" ht="16.5">
-      <c r="A25" s="63"/>
-      <c r="B25" s="63"/>
-      <c r="C25" s="64"/>
-      <c r="D25" s="82"/>
-      <c r="E25" s="82"/>
-      <c r="F25" s="64"/>
     </row>
     <row r="26" spans="1:8" ht="16.5" customHeight="1">
       <c r="A26" s="8" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B26" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D26" s="71">
+        <v>20000</v>
+      </c>
+      <c r="E26" s="71">
+        <v>20000</v>
+      </c>
+      <c r="F26" s="63" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="32.25" customHeight="1">
+      <c r="A27" s="69" t="s">
+        <v>385</v>
+      </c>
+      <c r="B27" s="69" t="s">
+        <v>386</v>
+      </c>
+      <c r="C27" s="69" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27" s="69">
+        <v>47000</v>
+      </c>
+      <c r="E27" s="69">
+        <v>47000</v>
+      </c>
+      <c r="F27" s="79" t="s">
+        <v>340</v>
+      </c>
+      <c r="H27" s="86" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A28" s="57" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="57" t="s">
+        <v>368</v>
+      </c>
+      <c r="C28" s="57" t="s">
+        <v>50</v>
+      </c>
+      <c r="D28" s="57">
+        <v>0</v>
+      </c>
+      <c r="E28" s="57">
+        <v>0</v>
+      </c>
+      <c r="F28" s="78" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="18" customHeight="1">
+      <c r="A29" s="83" t="s">
+        <v>376</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D29" s="71">
+        <v>60000</v>
+      </c>
+      <c r="E29" s="71">
+        <v>60000</v>
+      </c>
+      <c r="F29" s="70" t="s">
+        <v>351</v>
+      </c>
+      <c r="H29" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="16.5">
+      <c r="A30" s="72"/>
+      <c r="B30" s="70" t="s">
+        <v>352</v>
+      </c>
+      <c r="C30" s="72"/>
+      <c r="D30" s="72">
+        <f>SUM(D4:D29)</f>
+        <v>534100</v>
+      </c>
+      <c r="E30" s="72">
+        <f>SUM(E4:E29)</f>
+        <v>633200</v>
+      </c>
+      <c r="F30" s="72"/>
+    </row>
+    <row r="31" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A31" s="93" t="s">
+        <v>153</v>
+      </c>
+      <c r="B31" s="92"/>
+      <c r="C31" s="92"/>
+      <c r="D31" s="92"/>
+      <c r="E31" s="92"/>
+      <c r="F31" s="92"/>
+    </row>
+    <row r="32" spans="1:8" s="89" customFormat="1" ht="30" customHeight="1">
+      <c r="A32" s="91" t="s">
+        <v>393</v>
+      </c>
+      <c r="B32" s="92"/>
+      <c r="C32" s="92"/>
+      <c r="D32" s="92"/>
+      <c r="E32" s="92"/>
+      <c r="F32" s="92"/>
+    </row>
+    <row r="33" spans="1:8" s="89" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A33" s="93" t="s">
+        <v>152</v>
+      </c>
+      <c r="B33" s="92"/>
+      <c r="C33" s="92"/>
+      <c r="D33" s="92"/>
+      <c r="E33" s="92"/>
+      <c r="F33" s="92"/>
+    </row>
+    <row r="34" spans="1:8" s="89" customFormat="1" ht="15" customHeight="1">
+      <c r="A34" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>337</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" s="89" customFormat="1" ht="16.5" customHeight="1">
+      <c r="A35" s="65" t="s">
+        <v>378</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>395</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>396</v>
+      </c>
+      <c r="D35" s="69">
+        <v>100000</v>
+      </c>
+      <c r="E35" s="69">
+        <v>100000</v>
+      </c>
+      <c r="F35" s="70" t="s">
+        <v>399</v>
+      </c>
+      <c r="H35" s="107" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" s="89" customFormat="1" ht="16.5" customHeight="1">
+      <c r="A36" s="69"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="69"/>
+      <c r="E36" s="69"/>
+      <c r="F36" s="70"/>
+    </row>
+    <row r="37" spans="1:8" s="89" customFormat="1" ht="16.5" customHeight="1">
+      <c r="A37" s="69"/>
+      <c r="B37" s="8" t="s">
+        <v>400</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>401</v>
+      </c>
+      <c r="D37" s="69"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="70"/>
+    </row>
+    <row r="38" spans="1:8" s="89" customFormat="1" ht="16.5">
+      <c r="A38" s="79"/>
+      <c r="B38" s="79"/>
+      <c r="C38" s="82"/>
+      <c r="D38" s="82"/>
+      <c r="E38" s="82"/>
+      <c r="F38" s="79"/>
+    </row>
+    <row r="39" spans="1:8" s="62" customFormat="1" ht="33">
+      <c r="A39" s="65" t="s">
+        <v>23</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>394</v>
+      </c>
+      <c r="C39" s="8" t="s">
+        <v>387</v>
+      </c>
+      <c r="D39" s="71">
+        <f>109000-D14</f>
+        <v>49000</v>
+      </c>
+      <c r="E39" s="71">
+        <f>D39</f>
+        <v>49000</v>
+      </c>
+      <c r="F39" s="70" t="s">
+        <v>391</v>
+      </c>
+      <c r="G39" s="75"/>
+      <c r="H39" s="76" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="14.25">
+      <c r="A42" s="36" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="15">
+      <c r="A43" s="38" t="s">
+        <v>7</v>
+      </c>
+      <c r="B43" s="38" t="s">
+        <v>2</v>
+      </c>
+      <c r="C43" s="38" t="s">
+        <v>3</v>
+      </c>
+      <c r="D43" s="15" t="s">
+        <v>337</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="F43" s="38" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="16.5">
+      <c r="A44" s="79" t="s">
+        <v>383</v>
+      </c>
+      <c r="B44" s="79" t="s">
+        <v>369</v>
+      </c>
+      <c r="C44" s="35" t="s">
+        <v>62</v>
+      </c>
+      <c r="D44" s="77">
+        <v>20000</v>
+      </c>
+      <c r="E44" s="77">
+        <v>20000</v>
+      </c>
+      <c r="F44" s="63"/>
+    </row>
+    <row r="45" spans="1:8" s="62" customFormat="1" ht="33">
+      <c r="A45" s="79" t="s">
+        <v>364</v>
+      </c>
+      <c r="B45" s="63" t="s">
+        <v>365</v>
+      </c>
+      <c r="C45" s="64" t="s">
+        <v>58</v>
+      </c>
+      <c r="D45" s="64">
+        <v>46000</v>
+      </c>
+      <c r="E45" s="73">
+        <v>110000</v>
+      </c>
+      <c r="F45" s="63" t="s">
+        <v>363</v>
+      </c>
+      <c r="G45" s="67" t="s">
+        <v>355</v>
+      </c>
+      <c r="H45" s="76" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" s="62" customFormat="1" ht="33">
+      <c r="A46" s="63" t="s">
+        <v>319</v>
+      </c>
+      <c r="B46" s="63" t="s">
+        <v>367</v>
+      </c>
+      <c r="C46" s="73" t="s">
+        <v>360</v>
+      </c>
+      <c r="D46" s="77">
+        <v>33000</v>
+      </c>
+      <c r="E46" s="77">
+        <v>33000</v>
+      </c>
+      <c r="F46" s="63" t="s">
+        <v>316</v>
+      </c>
+      <c r="G46" s="67" t="s">
+        <v>354</v>
+      </c>
+      <c r="H46" s="76" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="16.5">
+      <c r="A47" s="51" t="s">
+        <v>330</v>
+      </c>
+      <c r="B47" s="63" t="s">
+        <v>370</v>
+      </c>
+      <c r="C47" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="D47" s="77">
+        <v>13000</v>
+      </c>
+      <c r="E47" s="77">
+        <v>13000</v>
+      </c>
+      <c r="F47" s="35"/>
+    </row>
+    <row r="48" spans="1:8" ht="16.5">
+      <c r="A48" s="51" t="s">
+        <v>331</v>
+      </c>
+      <c r="B48" s="35" t="s">
+        <v>40</v>
+      </c>
+      <c r="C48" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="D48" s="35"/>
+      <c r="E48" s="35"/>
+      <c r="F48" s="63" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="16.5">
+      <c r="A49" s="51" t="s">
+        <v>332</v>
+      </c>
+      <c r="B49" s="63" t="s">
+        <v>371</v>
+      </c>
+      <c r="C49" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="D49" s="35"/>
+      <c r="E49" s="35"/>
+      <c r="F49" s="63" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="16.5">
+      <c r="A50" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="B50" s="35" t="s">
+        <v>44</v>
+      </c>
+      <c r="C50" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="D50" s="35"/>
+      <c r="E50" s="35"/>
+      <c r="F50" s="35"/>
+    </row>
+    <row r="51" spans="1:6" ht="16.5">
+      <c r="A51" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="B51" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="C51" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="D51" s="35"/>
+      <c r="E51" s="35"/>
+      <c r="F51" s="35"/>
+    </row>
+    <row r="52" spans="1:6" ht="16.5">
+      <c r="A52" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="B52" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="C26" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="D26" s="71">
-        <v>50000</v>
-      </c>
-      <c r="E26" s="71">
-        <v>50000</v>
-      </c>
-      <c r="F26" s="70" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A27" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D27" s="71">
-        <v>20000</v>
-      </c>
-      <c r="E27" s="71">
-        <v>20000</v>
-      </c>
-      <c r="F27" s="63" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="32.25" customHeight="1">
-      <c r="A28" s="69" t="s">
-        <v>386</v>
-      </c>
-      <c r="B28" s="69" t="s">
-        <v>387</v>
-      </c>
-      <c r="C28" s="69" t="s">
-        <v>19</v>
-      </c>
-      <c r="D28" s="69">
-        <v>47000</v>
-      </c>
-      <c r="E28" s="69">
-        <v>47000</v>
-      </c>
-      <c r="F28" s="79" t="s">
-        <v>341</v>
-      </c>
-      <c r="H28" s="86" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A29" s="57" t="s">
-        <v>51</v>
-      </c>
-      <c r="B29" s="57" t="s">
-        <v>369</v>
-      </c>
-      <c r="C29" s="57" t="s">
-        <v>50</v>
-      </c>
-      <c r="D29" s="57">
-        <v>0</v>
-      </c>
-      <c r="E29" s="57">
-        <v>0</v>
-      </c>
-      <c r="F29" s="78" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="18" customHeight="1">
-      <c r="A30" s="83" t="s">
-        <v>377</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="D30" s="71">
-        <v>60000</v>
-      </c>
-      <c r="E30" s="71">
-        <v>60000</v>
-      </c>
-      <c r="F30" s="70" t="s">
+      <c r="C52" s="35" t="s">
+        <v>71</v>
+      </c>
+      <c r="D52" s="35"/>
+      <c r="E52" s="35"/>
+      <c r="F52" s="35"/>
+    </row>
+    <row r="53" spans="1:6" ht="16.5">
+      <c r="A53" s="72"/>
+      <c r="B53" s="70" t="s">
         <v>352</v>
       </c>
-      <c r="H30" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="16.5">
-      <c r="A31" s="72"/>
-      <c r="B31" s="70" t="s">
-        <v>353</v>
-      </c>
-      <c r="C31" s="72"/>
-      <c r="D31" s="72">
-        <f>SUM(D4:D30)</f>
-        <v>583100</v>
-      </c>
-      <c r="E31" s="72">
-        <f>SUM(E4:E30)</f>
-        <v>682200</v>
-      </c>
-      <c r="F31" s="72"/>
-    </row>
-    <row r="32" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A32" s="91" t="s">
-        <v>154</v>
-      </c>
-      <c r="B32" s="90"/>
-      <c r="C32" s="90"/>
-      <c r="D32" s="90"/>
-      <c r="E32" s="90"/>
-      <c r="F32" s="90"/>
-    </row>
-    <row r="35" spans="1:8" ht="14.25">
-      <c r="A35" s="36" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" ht="15">
-      <c r="A36" s="38" t="s">
-        <v>7</v>
-      </c>
-      <c r="B36" s="38" t="s">
-        <v>2</v>
-      </c>
-      <c r="C36" s="38" t="s">
-        <v>3</v>
-      </c>
-      <c r="D36" s="15" t="s">
-        <v>338</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>337</v>
-      </c>
-      <c r="F36" s="38" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" ht="16.5">
-      <c r="A37" s="79" t="s">
-        <v>384</v>
-      </c>
-      <c r="B37" s="79" t="s">
-        <v>370</v>
-      </c>
-      <c r="C37" s="35" t="s">
-        <v>62</v>
-      </c>
-      <c r="D37" s="77">
-        <v>20000</v>
-      </c>
-      <c r="E37" s="77">
-        <v>20000</v>
-      </c>
-      <c r="F37" s="63"/>
-    </row>
-    <row r="38" spans="1:8" s="62" customFormat="1" ht="33">
-      <c r="A38" s="79" t="s">
-        <v>365</v>
-      </c>
-      <c r="B38" s="63" t="s">
-        <v>366</v>
-      </c>
-      <c r="C38" s="64" t="s">
-        <v>58</v>
-      </c>
-      <c r="D38" s="64">
-        <v>46000</v>
-      </c>
-      <c r="E38" s="73">
-        <v>110000</v>
-      </c>
-      <c r="F38" s="63" t="s">
-        <v>364</v>
-      </c>
-      <c r="G38" s="67" t="s">
-        <v>356</v>
-      </c>
-      <c r="H38" s="76" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" s="62" customFormat="1" ht="33">
-      <c r="A39" s="63" t="s">
-        <v>320</v>
-      </c>
-      <c r="B39" s="63" t="s">
-        <v>368</v>
-      </c>
-      <c r="C39" s="73" t="s">
-        <v>361</v>
-      </c>
-      <c r="D39" s="77">
-        <v>33000</v>
-      </c>
-      <c r="E39" s="77">
-        <v>33000</v>
-      </c>
-      <c r="F39" s="63" t="s">
-        <v>317</v>
-      </c>
-      <c r="G39" s="67" t="s">
-        <v>355</v>
-      </c>
-      <c r="H39" s="76" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" ht="16.5">
-      <c r="A40" s="51" t="s">
-        <v>331</v>
-      </c>
-      <c r="B40" s="63" t="s">
-        <v>371</v>
-      </c>
-      <c r="C40" s="35" t="s">
-        <v>60</v>
-      </c>
-      <c r="D40" s="77">
-        <v>13000</v>
-      </c>
-      <c r="E40" s="77">
-        <v>13000</v>
-      </c>
-      <c r="F40" s="35"/>
-    </row>
-    <row r="41" spans="1:8" ht="16.5">
-      <c r="A41" s="51" t="s">
-        <v>332</v>
-      </c>
-      <c r="B41" s="35" t="s">
-        <v>40</v>
-      </c>
-      <c r="C41" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="D41" s="35"/>
-      <c r="E41" s="35"/>
-      <c r="F41" s="63" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" ht="16.5">
-      <c r="A42" s="51" t="s">
-        <v>333</v>
-      </c>
-      <c r="B42" s="63" t="s">
-        <v>372</v>
-      </c>
-      <c r="C42" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="D42" s="35"/>
-      <c r="E42" s="35"/>
-      <c r="F42" s="63" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" ht="16.5">
-      <c r="A43" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="B43" s="35" t="s">
-        <v>44</v>
-      </c>
-      <c r="C43" s="35" t="s">
-        <v>45</v>
-      </c>
-      <c r="D43" s="35"/>
-      <c r="E43" s="35"/>
-      <c r="F43" s="35"/>
-    </row>
-    <row r="44" spans="1:8" ht="16.5">
-      <c r="A44" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="B44" s="35" t="s">
-        <v>67</v>
-      </c>
-      <c r="C44" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="D44" s="35"/>
-      <c r="E44" s="35"/>
-      <c r="F44" s="35"/>
-    </row>
-    <row r="45" spans="1:8" ht="16.5">
-      <c r="A45" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="B45" s="35" t="s">
-        <v>38</v>
-      </c>
-      <c r="C45" s="35" t="s">
-        <v>71</v>
-      </c>
-      <c r="D45" s="35"/>
-      <c r="E45" s="35"/>
-      <c r="F45" s="35"/>
-    </row>
-    <row r="46" spans="1:8" ht="16.5">
-      <c r="A46" s="72"/>
-      <c r="B46" s="70" t="s">
-        <v>353</v>
-      </c>
-      <c r="C46" s="72"/>
-      <c r="D46" s="72">
-        <f>SUM(D12:D45)</f>
-        <v>1141100</v>
-      </c>
-      <c r="E46" s="72">
-        <f>SUM(E12:E45)</f>
-        <v>1392300</v>
-      </c>
-      <c r="F46" s="72"/>
+      <c r="C53" s="72"/>
+      <c r="D53" s="72">
+        <f>SUM(D12:D52)</f>
+        <v>1192100</v>
+      </c>
+      <c r="E53" s="72">
+        <f>SUM(E12:E52)</f>
+        <v>1443300</v>
+      </c>
+      <c r="F53" s="72"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A32:F32"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A33:F33"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
-  <conditionalFormatting sqref="D4 D17:D18 D10:E11 D21:E21 D5:E7 D9 D22:D23 D26:D27 D29:D30">
-    <cfRule type="cellIs" dxfId="13" priority="9" operator="equal">
+  <conditionalFormatting sqref="D4 D16:D17 D10:E11 D20:E20 D5:E7 D9 D21:D22 D25:D26 D28:D29">
+    <cfRule type="cellIs" dxfId="14" priority="10" operator="equal">
+      <formula>"✅"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E16">
+    <cfRule type="cellIs" dxfId="13" priority="8" operator="equal">
       <formula>"✅"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5270,12 +5412,12 @@
       <formula>"✅"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E18">
+  <conditionalFormatting sqref="E21">
     <cfRule type="cellIs" dxfId="11" priority="6" operator="equal">
       <formula>"✅"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E22">
+  <conditionalFormatting sqref="E25">
     <cfRule type="cellIs" dxfId="10" priority="5" operator="equal">
       <formula>"✅"</formula>
     </cfRule>
@@ -5285,17 +5427,17 @@
       <formula>"✅"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E27">
+  <conditionalFormatting sqref="E9">
     <cfRule type="cellIs" dxfId="8" priority="3" operator="equal">
       <formula>"✅"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E9">
+  <conditionalFormatting sqref="E29">
     <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
       <formula>"✅"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E30">
+  <conditionalFormatting sqref="D35:E37">
     <cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
       <formula>"✅"</formula>
     </cfRule>
@@ -5322,53 +5464,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="91" t="s">
+        <v>156</v>
+      </c>
+      <c r="B1" s="92"/>
+      <c r="C1" s="92"/>
+      <c r="D1" s="92"/>
+      <c r="E1" s="92"/>
+      <c r="F1" s="92"/>
+      <c r="G1" s="92"/>
+      <c r="H1" s="92"/>
+    </row>
+    <row r="3" spans="1:8" ht="15" customHeight="1">
+      <c r="A3" s="100" t="s">
         <v>157</v>
       </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-    </row>
-    <row r="3" spans="1:8" ht="15" customHeight="1">
-      <c r="A3" s="98" t="s">
-        <v>158</v>
-      </c>
-      <c r="B3" s="90"/>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
+      <c r="B3" s="92"/>
+      <c r="C3" s="92"/>
+      <c r="D3" s="92"/>
+      <c r="E3" s="92"/>
+      <c r="F3" s="92"/>
+      <c r="G3" s="92"/>
+      <c r="H3" s="92"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="16.5" customHeight="1">
@@ -5376,7 +5518,7 @@
         <v>41</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C5" s="8">
         <v>3</v>
@@ -5388,13 +5530,13 @@
         <v>3</v>
       </c>
       <c r="F5" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="G5" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="H5" s="8" t="s">
         <v>168</v>
-      </c>
-      <c r="H5" s="8" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="33" customHeight="1">
@@ -5402,7 +5544,7 @@
         <v>41</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C6" s="8">
         <v>5</v>
@@ -5414,13 +5556,13 @@
         <v>5</v>
       </c>
       <c r="F6" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="G6" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="H6" s="8" t="s">
         <v>172</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="16.5" customHeight="1">
@@ -5428,7 +5570,7 @@
         <v>35</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C7" s="8">
         <v>6</v>
@@ -5440,13 +5582,13 @@
         <v>6</v>
       </c>
       <c r="F7" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="G7" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="H7" s="8" t="s">
         <v>176</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="16.5" customHeight="1">
@@ -5454,7 +5596,7 @@
         <v>35</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C8" s="8">
         <v>2</v>
@@ -5466,13 +5608,13 @@
         <v>2</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G8" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="H8" s="8" t="s">
         <v>178</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="33" customHeight="1">
@@ -5480,7 +5622,7 @@
         <v>35</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C9" s="8">
         <v>4</v>
@@ -5492,13 +5634,13 @@
         <v>4</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="33" customHeight="1">
@@ -5506,7 +5648,7 @@
         <v>35</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C10" s="35">
         <v>6</v>
@@ -5518,13 +5660,13 @@
         <v>6</v>
       </c>
       <c r="F10" s="35" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G10" s="35" t="s">
+        <v>182</v>
+      </c>
+      <c r="H10" s="35" t="s">
         <v>183</v>
-      </c>
-      <c r="H10" s="35" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="16.5" customHeight="1">
@@ -5532,7 +5674,7 @@
         <v>49</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C11" s="8">
         <v>6</v>
@@ -5544,13 +5686,13 @@
         <v>6</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="33" customHeight="1">
@@ -5558,7 +5700,7 @@
         <v>49</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C12" s="8">
         <v>1</v>
@@ -5570,10 +5712,10 @@
         <v>1</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>11</v>
@@ -5581,10 +5723,10 @@
     </row>
     <row r="13" spans="1:8" ht="33" customHeight="1">
       <c r="A13" s="8" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C13" s="8">
         <v>0</v>
@@ -5596,13 +5738,13 @@
         <v>0</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G13" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="H13" s="8" t="s">
         <v>188</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="16.5" customHeight="1">
@@ -5610,7 +5752,7 @@
         <v>9</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C14" s="8">
         <v>2</v>
@@ -5622,13 +5764,13 @@
         <v>2</v>
       </c>
       <c r="F14" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="G14" s="8" t="s">
         <v>191</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="H14" s="8" t="s">
         <v>192</v>
-      </c>
-      <c r="H14" s="8" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="16.5" customHeight="1">
@@ -5636,32 +5778,32 @@
         <v>32</v>
       </c>
       <c r="B15" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="C15" s="8" t="s">
         <v>194</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>195</v>
       </c>
       <c r="D15" s="8">
         <v>0</v>
       </c>
       <c r="E15" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="F15" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="G15" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H15" s="8" t="s">
         <v>196</v>
       </c>
-      <c r="G15" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="H15" s="8" t="s">
+    </row>
+    <row r="16" spans="1:8" ht="16.5" customHeight="1">
+      <c r="A16" s="101" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A16" s="99" t="s">
-        <v>198</v>
-      </c>
-      <c r="B16" s="100"/>
+      <c r="B16" s="102"/>
       <c r="C16" s="8">
         <f>SUM(C5:C15)</f>
         <v>35</v>
@@ -5674,45 +5816,45 @@
         <f>SUM(E5:E15)</f>
         <v>35</v>
       </c>
-      <c r="F16" s="99" t="s">
-        <v>199</v>
-      </c>
-      <c r="G16" s="100"/>
+      <c r="F16" s="101" t="s">
+        <v>198</v>
+      </c>
+      <c r="G16" s="102"/>
       <c r="H16" s="21"/>
     </row>
     <row r="17" spans="1:8" ht="15" customHeight="1">
-      <c r="A17" s="90"/>
-      <c r="B17" s="90"/>
-      <c r="C17" s="90"/>
-      <c r="D17" s="90"/>
-      <c r="E17" s="90"/>
-      <c r="F17" s="90"/>
-      <c r="G17" s="90"/>
-      <c r="H17" s="90"/>
+      <c r="A17" s="92"/>
+      <c r="B17" s="92"/>
+      <c r="C17" s="92"/>
+      <c r="D17" s="92"/>
+      <c r="E17" s="92"/>
+      <c r="F17" s="92"/>
+      <c r="G17" s="92"/>
+      <c r="H17" s="92"/>
     </row>
     <row r="18" spans="1:8" ht="15" customHeight="1">
       <c r="A18" s="33" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="16.5" customHeight="1">
       <c r="A19" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D19" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="F19" s="1" t="s">
         <v>203</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>204</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>82</v>
@@ -5821,7 +5963,7 @@
     </row>
     <row r="32" spans="1:8" ht="14.25" customHeight="1">
       <c r="A32" s="29" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="15">
@@ -5832,22 +5974,22 @@
         <v>3</v>
       </c>
       <c r="C33" s="38" t="s">
+        <v>205</v>
+      </c>
+      <c r="D33" s="38" t="s">
         <v>206</v>
       </c>
-      <c r="D33" s="38" t="s">
+      <c r="E33" s="38" t="s">
         <v>207</v>
       </c>
-      <c r="E33" s="38" t="s">
+      <c r="F33" s="38" t="s">
+        <v>161</v>
+      </c>
+      <c r="G33" s="38" t="s">
         <v>208</v>
       </c>
-      <c r="F33" s="38" t="s">
-        <v>162</v>
-      </c>
-      <c r="G33" s="38" t="s">
+      <c r="H33" s="38" t="s">
         <v>209</v>
-      </c>
-      <c r="H33" s="38" t="s">
-        <v>210</v>
       </c>
       <c r="I33" t="s">
         <v>82</v>
@@ -5861,7 +6003,7 @@
         <v>58</v>
       </c>
       <c r="C34" s="35" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D34" s="35">
         <v>4</v>
@@ -5873,13 +6015,13 @@
         <v>4</v>
       </c>
       <c r="G34" s="35" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H34" s="35" t="s">
+        <v>211</v>
+      </c>
+      <c r="I34" t="s">
         <v>212</v>
-      </c>
-      <c r="I34" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="33">
@@ -5890,25 +6032,25 @@
         <v>58</v>
       </c>
       <c r="C35" s="35" t="s">
+        <v>213</v>
+      </c>
+      <c r="D35" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="E35" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="F35" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="G35" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="H35" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="I35" t="s">
         <v>214</v>
-      </c>
-      <c r="D35" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E35" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="F35" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="G35" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="H35" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="I35" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="36" spans="1:9" ht="16.5">
@@ -5919,7 +6061,7 @@
         <v>60</v>
       </c>
       <c r="C36" s="35" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D36" s="35">
         <v>6</v>
@@ -5931,10 +6073,10 @@
         <v>6</v>
       </c>
       <c r="G36" s="35" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H36" s="35" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="16.5">
@@ -5945,7 +6087,7 @@
         <v>60</v>
       </c>
       <c r="C37" s="35" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D37" s="35">
         <v>12</v>
@@ -5960,10 +6102,10 @@
         <v>11</v>
       </c>
       <c r="H37" s="35" t="s">
+        <v>217</v>
+      </c>
+      <c r="I37" t="s">
         <v>218</v>
-      </c>
-      <c r="I37" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="33">
@@ -5974,7 +6116,7 @@
         <v>62</v>
       </c>
       <c r="C38" s="35" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D38" s="35">
         <v>2</v>
@@ -5986,7 +6128,7 @@
         <v>2</v>
       </c>
       <c r="G38" s="35" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H38" s="35" t="s">
         <v>85</v>
@@ -6000,7 +6142,7 @@
         <v>62</v>
       </c>
       <c r="C39" s="35" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D39" s="35">
         <v>4</v>
@@ -6012,13 +6154,13 @@
         <v>4</v>
       </c>
       <c r="G39" s="35" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H39" s="35" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I39" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="33">
@@ -6029,7 +6171,7 @@
         <v>62</v>
       </c>
       <c r="C40" s="35" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D40" s="35">
         <v>6</v>
@@ -6044,7 +6186,7 @@
         <v>11</v>
       </c>
       <c r="H40" s="35" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -6085,147 +6227,147 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="91" t="s">
+        <v>222</v>
+      </c>
+      <c r="B1" s="92"/>
+      <c r="C1" s="92"/>
+      <c r="D1" s="92"/>
+      <c r="E1" s="92"/>
+      <c r="F1" s="92"/>
+      <c r="G1" s="92"/>
+      <c r="H1" s="92"/>
+    </row>
+    <row r="3" spans="1:8" ht="15" customHeight="1">
+      <c r="A3" s="100" t="s">
         <v>223</v>
       </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-    </row>
-    <row r="3" spans="1:8" ht="15" customHeight="1">
-      <c r="A3" s="98" t="s">
-        <v>224</v>
-      </c>
-      <c r="B3" s="90"/>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
+      <c r="B3" s="92"/>
+      <c r="C3" s="92"/>
+      <c r="D3" s="92"/>
+      <c r="E3" s="92"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>227</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="49.5" customHeight="1">
       <c r="A5" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>47</v>
       </c>
       <c r="C5" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="E5" s="8" t="s">
         <v>231</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="33" customHeight="1">
       <c r="A6" s="8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B6" s="8" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>234</v>
       </c>
-      <c r="D6" s="8" t="s">
-        <v>235</v>
-      </c>
       <c r="E6" s="8" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="33" customHeight="1">
       <c r="A7" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>25</v>
       </c>
       <c r="C7" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>237</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>238</v>
-      </c>
       <c r="E7" s="8" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="33" customHeight="1">
       <c r="A8" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="C8" s="8" t="s">
         <v>240</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="D8" s="8" t="s">
         <v>241</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="E8" s="8" t="s">
         <v>242</v>
       </c>
-      <c r="E8" s="8" t="s">
+    </row>
+    <row r="11" spans="1:8" ht="15" customHeight="1">
+      <c r="A11" s="100" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" ht="15" customHeight="1">
-      <c r="A11" s="98" t="s">
-        <v>244</v>
-      </c>
-      <c r="B11" s="90"/>
-      <c r="C11" s="90"/>
-      <c r="D11" s="90"/>
-      <c r="E11" s="90"/>
-      <c r="F11" s="90"/>
-      <c r="G11" s="90"/>
-      <c r="H11" s="90"/>
+      <c r="B11" s="92"/>
+      <c r="C11" s="92"/>
+      <c r="D11" s="92"/>
+      <c r="E11" s="92"/>
+      <c r="F11" s="92"/>
+      <c r="G11" s="92"/>
+      <c r="H11" s="92"/>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>249</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="16.5" customHeight="1">
@@ -6356,24 +6498,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="91" t="s">
+        <v>250</v>
+      </c>
+      <c r="B1" s="92"/>
+      <c r="C1" s="92"/>
+      <c r="D1" s="92"/>
+      <c r="E1" s="92"/>
+      <c r="F1" s="92"/>
+    </row>
+    <row r="3" spans="1:6" ht="15" customHeight="1">
+      <c r="A3" s="100" t="s">
         <v>251</v>
       </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-    </row>
-    <row r="3" spans="1:6" ht="15" customHeight="1">
-      <c r="A3" s="98" t="s">
-        <v>252</v>
-      </c>
-      <c r="B3" s="90"/>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
+      <c r="B3" s="92"/>
+      <c r="C3" s="92"/>
+      <c r="D3" s="92"/>
+      <c r="E3" s="92"/>
+      <c r="F3" s="92"/>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1">
       <c r="A4" s="5" t="s">
@@ -6383,13 +6525,13 @@
         <v>3</v>
       </c>
       <c r="C4" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>253</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>246</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>254</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>82</v>
@@ -6406,7 +6548,7 @@
         <v>480</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E5" s="8">
         <v>480</v>
@@ -6426,7 +6568,7 @@
         <v>500</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E6" s="8">
         <v>500</v>
@@ -6446,7 +6588,7 @@
         <v>900</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E7" s="8">
         <v>900</v>
@@ -6456,21 +6598,21 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A8" s="103" t="s">
+      <c r="A8" s="105" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="94"/>
+      <c r="B8" s="96"/>
       <c r="C8" s="35">
         <v>500</v>
       </c>
       <c r="D8" s="35" t="s">
+        <v>255</v>
+      </c>
+      <c r="E8" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="35" t="s">
         <v>256</v>
-      </c>
-      <c r="E8" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="35" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="16.5" customHeight="1">
@@ -6484,7 +6626,7 @@
         <v>1800</v>
       </c>
       <c r="D9" s="35" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E9" s="35" t="s">
         <v>11</v>
@@ -6494,18 +6636,18 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1">
-      <c r="A10" s="101"/>
-      <c r="B10" s="93"/>
-      <c r="C10" s="93"/>
-      <c r="D10" s="93"/>
-      <c r="E10" s="93"/>
-      <c r="F10" s="94"/>
+      <c r="A10" s="103"/>
+      <c r="B10" s="95"/>
+      <c r="C10" s="95"/>
+      <c r="D10" s="95"/>
+      <c r="E10" s="95"/>
+      <c r="F10" s="96"/>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1">
-      <c r="A11" s="99" t="s">
-        <v>198</v>
-      </c>
-      <c r="B11" s="94"/>
+      <c r="A11" s="101" t="s">
+        <v>197</v>
+      </c>
+      <c r="B11" s="96"/>
       <c r="C11" s="34">
         <f>SUM(C5:C9)</f>
         <v>4180</v>
@@ -6520,18 +6662,18 @@
     <row r="12" spans="1:6" ht="16.5" customHeight="1"/>
     <row r="13" spans="1:6" ht="16.5" customHeight="1">
       <c r="A13" s="33" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16.5" customHeight="1">
       <c r="A14" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="C14" s="6" t="s">
         <v>261</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>262</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>11</v>
@@ -6545,10 +6687,10 @@
     </row>
     <row r="15" spans="1:6" ht="16.5" customHeight="1">
       <c r="A15" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>263</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>264</v>
       </c>
       <c r="C15" s="8">
         <v>0</v>
@@ -6556,7 +6698,7 @@
     </row>
     <row r="16" spans="1:6" ht="16.5" customHeight="1">
       <c r="A16" s="8" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B16" s="8" t="s">
         <v>11</v>
@@ -6566,21 +6708,21 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="15" customHeight="1">
-      <c r="A17" s="102" t="s">
-        <v>266</v>
-      </c>
-      <c r="B17" s="93"/>
-      <c r="C17" s="93"/>
-      <c r="D17" s="93"/>
-      <c r="E17" s="93"/>
-      <c r="F17" s="94"/>
+      <c r="A17" s="104" t="s">
+        <v>265</v>
+      </c>
+      <c r="B17" s="95"/>
+      <c r="C17" s="95"/>
+      <c r="D17" s="95"/>
+      <c r="E17" s="95"/>
+      <c r="F17" s="96"/>
     </row>
     <row r="18" spans="1:6" ht="15" customHeight="1">
       <c r="A18" s="11" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C18" s="11">
         <v>0</v>
@@ -6592,15 +6734,15 @@
     <row r="19" spans="1:6" ht="16.5" customHeight="1"/>
     <row r="20" spans="1:6" ht="16.5" customHeight="1">
       <c r="A20" s="33" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="16.5" customHeight="1">
       <c r="A21" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>268</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>269</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>11</v>
@@ -6617,38 +6759,38 @@
     </row>
     <row r="22" spans="1:6" ht="16.5" customHeight="1">
       <c r="A22" s="22" t="s">
+        <v>269</v>
+      </c>
+      <c r="B22" s="23" t="s">
         <v>270</v>
       </c>
-      <c r="B22" s="23" t="s">
-        <v>271</v>
-      </c>
     </row>
     <row r="23" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A23" s="102" t="s">
-        <v>164</v>
-      </c>
-      <c r="B23" s="93"/>
-      <c r="C23" s="93"/>
-      <c r="D23" s="93"/>
-      <c r="E23" s="93"/>
-      <c r="F23" s="94"/>
+      <c r="A23" s="104" t="s">
+        <v>163</v>
+      </c>
+      <c r="B23" s="95"/>
+      <c r="C23" s="95"/>
+      <c r="D23" s="95"/>
+      <c r="E23" s="95"/>
+      <c r="F23" s="96"/>
     </row>
     <row r="24" spans="1:6" ht="16.5" customHeight="1">
       <c r="A24" s="8" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="15.75" customHeight="1">
       <c r="A26" s="31" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="14.25" customHeight="1">
       <c r="A29" s="29" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="15">
@@ -6659,13 +6801,13 @@
         <v>3</v>
       </c>
       <c r="C30" s="46" t="s">
+        <v>252</v>
+      </c>
+      <c r="D30" s="46" t="s">
+        <v>245</v>
+      </c>
+      <c r="E30" s="46" t="s">
         <v>253</v>
-      </c>
-      <c r="D30" s="46" t="s">
-        <v>246</v>
-      </c>
-      <c r="E30" s="46" t="s">
-        <v>254</v>
       </c>
       <c r="F30" s="46" t="s">
         <v>82</v>
@@ -6682,13 +6824,13 @@
         <v>980</v>
       </c>
       <c r="D31" s="35" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E31" s="35" t="s">
         <v>11</v>
       </c>
       <c r="F31" s="35" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="16.5">
@@ -6702,13 +6844,13 @@
         <v>500</v>
       </c>
       <c r="D32" s="35" t="s">
+        <v>275</v>
+      </c>
+      <c r="E32" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="F32" s="35" t="s">
         <v>276</v>
-      </c>
-      <c r="E32" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="F32" s="35" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="16.5">
@@ -6722,13 +6864,13 @@
         <v>580</v>
       </c>
       <c r="D33" s="35" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E33" s="35" t="s">
         <v>11</v>
       </c>
       <c r="F33" s="35" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="16.5">
@@ -6742,13 +6884,13 @@
         <v>11</v>
       </c>
       <c r="D34" s="35" t="s">
+        <v>278</v>
+      </c>
+      <c r="E34" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="F34" s="35" t="s">
         <v>279</v>
-      </c>
-      <c r="E34" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="F34" s="35" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="16.5">
@@ -6762,7 +6904,7 @@
         <v>11</v>
       </c>
       <c r="D35" s="35" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E35" s="35" t="s">
         <v>11</v>
@@ -6803,28 +6945,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="91" t="s">
+        <v>281</v>
+      </c>
+      <c r="B1" s="92"/>
+      <c r="C1" s="92"/>
+      <c r="D1" s="92"/>
+      <c r="E1" s="92"/>
+      <c r="F1" s="92"/>
+      <c r="G1" s="92"/>
+      <c r="H1" s="92"/>
+    </row>
+    <row r="2" spans="1:8" ht="15.75" customHeight="1">
+      <c r="A2" s="93" t="s">
         <v>282</v>
       </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-    </row>
-    <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" s="91" t="s">
-        <v>283</v>
-      </c>
-      <c r="B2" s="90"/>
-      <c r="C2" s="90"/>
-      <c r="D2" s="90"/>
-      <c r="E2" s="90"/>
-      <c r="F2" s="90"/>
-      <c r="G2" s="90"/>
-      <c r="H2" s="90"/>
+      <c r="B2" s="92"/>
+      <c r="C2" s="92"/>
+      <c r="D2" s="92"/>
+      <c r="E2" s="92"/>
+      <c r="F2" s="92"/>
+      <c r="G2" s="92"/>
+      <c r="H2" s="92"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -6834,22 +6976,22 @@
         <v>3</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>285</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>286</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>78</v>
       </c>
       <c r="G3" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>287</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="16.5" customHeight="1">
@@ -6860,7 +7002,7 @@
         <v>42</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>11</v>
@@ -6886,7 +7028,7 @@
         <v>36</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>11</v>
@@ -6912,7 +7054,7 @@
         <v>48</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>11</v>
@@ -6938,7 +7080,7 @@
         <v>33</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>11</v>
@@ -6964,19 +7106,19 @@
         <v>19</v>
       </c>
       <c r="C8" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="8" t="s">
         <v>289</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>290</v>
       </c>
       <c r="H8" s="8" t="s">
         <v>11</v>
@@ -6990,19 +7132,19 @@
         <v>45</v>
       </c>
       <c r="C9" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" s="8" t="s">
         <v>289</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>290</v>
       </c>
       <c r="H9" s="8" t="s">
         <v>11</v>
@@ -7016,7 +7158,7 @@
         <v>53</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>11</v>
@@ -7028,7 +7170,7 @@
         <v>11</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H10" s="8" t="s">
         <v>11</v>
@@ -7036,7 +7178,7 @@
     </row>
     <row r="13" spans="1:8" ht="14.25" customHeight="1">
       <c r="A13" s="29" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15">
@@ -7047,22 +7189,22 @@
         <v>3</v>
       </c>
       <c r="C14" s="38" t="s">
+        <v>283</v>
+      </c>
+      <c r="D14" s="38" t="s">
         <v>284</v>
       </c>
-      <c r="D14" s="38" t="s">
+      <c r="E14" s="38" t="s">
         <v>285</v>
-      </c>
-      <c r="E14" s="38" t="s">
-        <v>286</v>
       </c>
       <c r="F14" s="38" t="s">
         <v>78</v>
       </c>
       <c r="G14" s="38" t="s">
+        <v>286</v>
+      </c>
+      <c r="H14" s="38" t="s">
         <v>287</v>
-      </c>
-      <c r="H14" s="38" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="16.5">
@@ -7073,13 +7215,13 @@
         <v>58</v>
       </c>
       <c r="C15" s="35" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>11</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F15" s="35" t="s">
         <v>11</v>
@@ -7099,13 +7241,13 @@
         <v>60</v>
       </c>
       <c r="C16" s="35" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D16" s="35" t="s">
         <v>11</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F16" s="35" t="s">
         <v>11</v>
@@ -7125,13 +7267,13 @@
         <v>62</v>
       </c>
       <c r="C17" s="35" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D17" s="35" t="s">
         <v>11</v>
       </c>
       <c r="E17" s="35" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F17" s="35" t="s">
         <v>11</v>
@@ -7151,7 +7293,7 @@
         <v>53</v>
       </c>
       <c r="C18" s="35" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D18" s="35" t="s">
         <v>11</v>
@@ -7163,7 +7305,7 @@
         <v>11</v>
       </c>
       <c r="G18" s="35" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H18" s="35" t="s">
         <v>148</v>
@@ -7201,30 +7343,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="104" t="s">
-        <v>296</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
+      <c r="A1" s="106" t="s">
+        <v>295</v>
+      </c>
+      <c r="B1" s="92"/>
+      <c r="C1" s="92"/>
+      <c r="D1" s="92"/>
+      <c r="E1" s="92"/>
+      <c r="F1" s="92"/>
     </row>
     <row r="2" spans="1:6" ht="24.95" customHeight="1">
       <c r="A2" s="9" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="9" t="s">
+        <v>296</v>
+      </c>
+      <c r="D2" s="9" t="s">
         <v>297</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="E2" s="9" t="s">
         <v>298</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>299</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>82</v>
@@ -7232,59 +7374,59 @@
     </row>
     <row r="3" spans="1:6" ht="21.95" customHeight="1">
       <c r="A3" s="10" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>49</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>300</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="E3" s="18" t="s">
         <v>302</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="F3" s="10" t="s">
         <v>303</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="21.95" customHeight="1">
       <c r="A4" s="10" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>44</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D4" s="10" t="s">
+        <v>305</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="F4" s="10" t="s">
         <v>306</v>
-      </c>
-      <c r="E4" s="18" t="s">
-        <v>303</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="21.95" customHeight="1">
       <c r="A5" s="10" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>41</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F5" s="10" t="s">
         <v>11</v>
@@ -7298,13 +7440,13 @@
         <v>25</v>
       </c>
       <c r="C6" s="10" t="s">
+        <v>308</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="20" t="s">
         <v>309</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="20" t="s">
-        <v>310</v>
       </c>
       <c r="F6" s="10" t="s">
         <v>11</v>
@@ -7318,16 +7460,16 @@
         <v>28</v>
       </c>
       <c r="C7" s="54" t="s">
+        <v>308</v>
+      </c>
+      <c r="D7" s="54" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="55" t="s">
         <v>309</v>
       </c>
-      <c r="D7" s="54" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="55" t="s">
-        <v>310</v>
-      </c>
       <c r="F7" s="56" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="21.95" customHeight="1">
@@ -7338,13 +7480,13 @@
         <v>18</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D8" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="E8" s="19" t="s">
         <v>311</v>
-      </c>
-      <c r="E8" s="19" t="s">
-        <v>312</v>
       </c>
       <c r="F8" s="10" t="s">
         <v>11</v>
@@ -7358,13 +7500,13 @@
         <v>18</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="F9" s="10" t="s">
         <v>11</v>
@@ -7372,19 +7514,19 @@
     </row>
     <row r="10" spans="1:6" ht="21.95" customHeight="1">
       <c r="A10" s="10" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>18</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="F10" s="10" t="s">
         <v>11</v>
@@ -7398,13 +7540,13 @@
         <v>47</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F11" s="10" t="s">
         <v>11</v>
@@ -7418,13 +7560,13 @@
         <v>35</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E12" s="20" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F12" s="10" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
auto: modify 01-Projects (2)
</commit_message>
<xml_diff>
--- a/01-Projects/family-hub/credit-card-management/信用卡主控表.xlsx
+++ b/01-Projects/family-hub/credit-card-management/信用卡主控表.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="1-卡片信息" sheetId="1" r:id="rId1"/>
@@ -1853,7 +1853,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2097,6 +2097,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2125,8 +2128,8 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="3" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2614,15 +2617,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="94" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
+      <c r="B1" s="95"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="95"/>
+      <c r="G1" s="95"/>
     </row>
     <row r="2" spans="1:8" ht="24.95" customHeight="1">
       <c r="A2" s="1" t="s">
@@ -2654,22 +2657,22 @@
       <c r="A3" s="8">
         <v>1</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="57" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="2">
+      <c r="D3" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="110">
         <v>0</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="110">
         <v>0</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="57" t="s">
         <v>329</v>
       </c>
       <c r="H3" s="53" t="s">
@@ -3049,12 +3052,12 @@
       </c>
     </row>
     <row r="19" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A19" s="99" t="s">
+      <c r="A19" s="100" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="97"/>
-      <c r="C19" s="97"/>
-      <c r="D19" s="98"/>
+      <c r="B19" s="98"/>
+      <c r="C19" s="98"/>
+      <c r="D19" s="99"/>
       <c r="E19" s="3">
         <f>SUM(E3:E18)</f>
         <v>831000</v>
@@ -3067,26 +3070,26 @@
       <c r="H19" s="26"/>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A21" s="95" t="s">
+      <c r="A21" s="96" t="s">
         <v>56</v>
       </c>
-      <c r="B21" s="94"/>
-      <c r="C21" s="94"/>
-      <c r="D21" s="94"/>
-      <c r="E21" s="94"/>
-      <c r="F21" s="94"/>
-      <c r="G21" s="94"/>
+      <c r="B21" s="95"/>
+      <c r="C21" s="95"/>
+      <c r="D21" s="95"/>
+      <c r="E21" s="95"/>
+      <c r="F21" s="95"/>
+      <c r="G21" s="95"/>
     </row>
     <row r="24" spans="1:8" ht="21" customHeight="1">
-      <c r="A24" s="93" t="s">
+      <c r="A24" s="94" t="s">
         <v>57</v>
       </c>
-      <c r="B24" s="94"/>
-      <c r="C24" s="94"/>
-      <c r="D24" s="94"/>
-      <c r="E24" s="94"/>
-      <c r="F24" s="94"/>
-      <c r="G24" s="94"/>
+      <c r="B24" s="95"/>
+      <c r="C24" s="95"/>
+      <c r="D24" s="95"/>
+      <c r="E24" s="95"/>
+      <c r="F24" s="95"/>
+      <c r="G24" s="95"/>
     </row>
     <row r="25" spans="1:8" ht="21" customHeight="1">
       <c r="A25" s="38" t="s">
@@ -3373,12 +3376,12 @@
       <c r="H37" s="53"/>
     </row>
     <row r="38" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A38" s="96" t="s">
+      <c r="A38" s="97" t="s">
         <v>73</v>
       </c>
-      <c r="B38" s="97"/>
-      <c r="C38" s="97"/>
-      <c r="D38" s="98"/>
+      <c r="B38" s="98"/>
+      <c r="C38" s="98"/>
+      <c r="D38" s="99"/>
       <c r="E38" s="41">
         <f>SUM(E26:E37)</f>
         <v>44000</v>
@@ -3425,28 +3428,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="94" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
+      <c r="B1" s="95"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="95"/>
+      <c r="G1" s="95"/>
+      <c r="H1" s="95"/>
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1">
-      <c r="A3" s="101" t="s">
+      <c r="A3" s="102" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="97"/>
-      <c r="C3" s="97"/>
-      <c r="D3" s="97"/>
-      <c r="E3" s="97"/>
-      <c r="F3" s="97"/>
-      <c r="G3" s="97"/>
-      <c r="H3" s="98"/>
+      <c r="B3" s="98"/>
+      <c r="C3" s="98"/>
+      <c r="D3" s="98"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="99"/>
       <c r="I3" s="24"/>
     </row>
     <row r="4" spans="1:9" ht="33" customHeight="1">
@@ -3606,16 +3609,16 @@
       <c r="I9" s="13"/>
     </row>
     <row r="10" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A10" s="101" t="s">
+      <c r="A10" s="102" t="s">
         <v>94</v>
       </c>
-      <c r="B10" s="97"/>
-      <c r="C10" s="97"/>
-      <c r="D10" s="97"/>
-      <c r="E10" s="97"/>
-      <c r="F10" s="97"/>
-      <c r="G10" s="97"/>
-      <c r="H10" s="98"/>
+      <c r="B10" s="98"/>
+      <c r="C10" s="98"/>
+      <c r="D10" s="98"/>
+      <c r="E10" s="98"/>
+      <c r="F10" s="98"/>
+      <c r="G10" s="98"/>
+      <c r="H10" s="99"/>
       <c r="I10" s="24"/>
     </row>
     <row r="11" spans="1:9" ht="16.5" customHeight="1">
@@ -3848,16 +3851,16 @@
       <c r="I19" s="13"/>
     </row>
     <row r="20" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A20" s="101" t="s">
+      <c r="A20" s="102" t="s">
         <v>109</v>
       </c>
-      <c r="B20" s="97"/>
-      <c r="C20" s="97"/>
-      <c r="D20" s="97"/>
-      <c r="E20" s="97"/>
-      <c r="F20" s="97"/>
-      <c r="G20" s="97"/>
-      <c r="H20" s="98"/>
+      <c r="B20" s="98"/>
+      <c r="C20" s="98"/>
+      <c r="D20" s="98"/>
+      <c r="E20" s="98"/>
+      <c r="F20" s="98"/>
+      <c r="G20" s="98"/>
+      <c r="H20" s="99"/>
       <c r="I20" s="24"/>
     </row>
     <row r="21" spans="1:9" ht="16.5" customHeight="1">
@@ -3982,16 +3985,16 @@
       <c r="I25" s="13"/>
     </row>
     <row r="26" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A26" s="101" t="s">
+      <c r="A26" s="102" t="s">
         <v>117</v>
       </c>
-      <c r="B26" s="97"/>
-      <c r="C26" s="97"/>
-      <c r="D26" s="97"/>
-      <c r="E26" s="97"/>
-      <c r="F26" s="97"/>
-      <c r="G26" s="97"/>
-      <c r="H26" s="98"/>
+      <c r="B26" s="98"/>
+      <c r="C26" s="98"/>
+      <c r="D26" s="98"/>
+      <c r="E26" s="98"/>
+      <c r="F26" s="98"/>
+      <c r="G26" s="98"/>
+      <c r="H26" s="99"/>
       <c r="I26" s="24"/>
     </row>
     <row r="27" spans="1:9" ht="16.5" customHeight="1">
@@ -4107,16 +4110,16 @@
       </c>
     </row>
     <row r="33" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A33" s="100" t="s">
+      <c r="A33" s="101" t="s">
         <v>133</v>
       </c>
-      <c r="B33" s="94"/>
-      <c r="C33" s="94"/>
-      <c r="D33" s="94"/>
-      <c r="E33" s="94"/>
-      <c r="F33" s="94"/>
-      <c r="G33" s="94"/>
-      <c r="H33" s="94"/>
+      <c r="B33" s="95"/>
+      <c r="C33" s="95"/>
+      <c r="D33" s="95"/>
+      <c r="E33" s="95"/>
+      <c r="F33" s="95"/>
+      <c r="G33" s="95"/>
+      <c r="H33" s="95"/>
     </row>
     <row r="36" spans="1:9" ht="14.25" customHeight="1">
       <c r="A36" s="36" t="s">
@@ -4525,24 +4528,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="94" t="s">
         <v>392</v>
       </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
+      <c r="B1" s="95"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="95"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="96" t="s">
         <v>152</v>
       </c>
-      <c r="B2" s="94"/>
-      <c r="C2" s="94"/>
-      <c r="D2" s="94"/>
-      <c r="E2" s="94"/>
-      <c r="F2" s="94"/>
+      <c r="B2" s="95"/>
+      <c r="C2" s="95"/>
+      <c r="D2" s="95"/>
+      <c r="E2" s="95"/>
+      <c r="F2" s="95"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -5071,34 +5074,34 @@
       <c r="F30" s="72"/>
     </row>
     <row r="31" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A31" s="95" t="s">
+      <c r="A31" s="96" t="s">
         <v>153</v>
       </c>
-      <c r="B31" s="94"/>
-      <c r="C31" s="94"/>
-      <c r="D31" s="94"/>
-      <c r="E31" s="94"/>
-      <c r="F31" s="94"/>
+      <c r="B31" s="95"/>
+      <c r="C31" s="95"/>
+      <c r="D31" s="95"/>
+      <c r="E31" s="95"/>
+      <c r="F31" s="95"/>
     </row>
     <row r="32" spans="1:8" s="89" customFormat="1" ht="30" customHeight="1">
-      <c r="A32" s="93" t="s">
+      <c r="A32" s="94" t="s">
         <v>393</v>
       </c>
-      <c r="B32" s="94"/>
-      <c r="C32" s="94"/>
-      <c r="D32" s="94"/>
-      <c r="E32" s="94"/>
-      <c r="F32" s="94"/>
+      <c r="B32" s="95"/>
+      <c r="C32" s="95"/>
+      <c r="D32" s="95"/>
+      <c r="E32" s="95"/>
+      <c r="F32" s="95"/>
     </row>
     <row r="33" spans="1:8" s="89" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A33" s="95" t="s">
+      <c r="A33" s="96" t="s">
         <v>152</v>
       </c>
-      <c r="B33" s="94"/>
-      <c r="C33" s="94"/>
-      <c r="D33" s="94"/>
-      <c r="E33" s="94"/>
-      <c r="F33" s="94"/>
+      <c r="B33" s="95"/>
+      <c r="C33" s="95"/>
+      <c r="D33" s="95"/>
+      <c r="E33" s="95"/>
+      <c r="F33" s="95"/>
     </row>
     <row r="34" spans="1:8" s="89" customFormat="1" ht="15" customHeight="1">
       <c r="A34" s="1" t="s">
@@ -5191,7 +5194,7 @@
         <v>391</v>
       </c>
       <c r="G39" s="75"/>
-      <c r="H39" s="109" t="s">
+      <c r="H39" s="93" t="s">
         <v>398</v>
       </c>
     </row>
@@ -5499,28 +5502,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="94" t="s">
         <v>156</v>
       </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
+      <c r="B1" s="95"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="95"/>
+      <c r="G1" s="95"/>
+      <c r="H1" s="95"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
-      <c r="A3" s="102" t="s">
+      <c r="A3" s="103" t="s">
         <v>157</v>
       </c>
-      <c r="B3" s="94"/>
-      <c r="C3" s="94"/>
-      <c r="D3" s="94"/>
-      <c r="E3" s="94"/>
-      <c r="F3" s="94"/>
-      <c r="G3" s="94"/>
-      <c r="H3" s="94"/>
+      <c r="B3" s="95"/>
+      <c r="C3" s="95"/>
+      <c r="D3" s="95"/>
+      <c r="E3" s="95"/>
+      <c r="F3" s="95"/>
+      <c r="G3" s="95"/>
+      <c r="H3" s="95"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -5835,10 +5838,10 @@
       </c>
     </row>
     <row r="16" spans="1:8" ht="16.5" customHeight="1">
-      <c r="A16" s="103" t="s">
+      <c r="A16" s="104" t="s">
         <v>197</v>
       </c>
-      <c r="B16" s="104"/>
+      <c r="B16" s="105"/>
       <c r="C16" s="8">
         <f>SUM(C5:C15)</f>
         <v>35</v>
@@ -5851,21 +5854,21 @@
         <f>SUM(E5:E15)</f>
         <v>35</v>
       </c>
-      <c r="F16" s="103" t="s">
+      <c r="F16" s="104" t="s">
         <v>198</v>
       </c>
-      <c r="G16" s="104"/>
+      <c r="G16" s="105"/>
       <c r="H16" s="21"/>
     </row>
     <row r="17" spans="1:8" ht="15" customHeight="1">
-      <c r="A17" s="94"/>
-      <c r="B17" s="94"/>
-      <c r="C17" s="94"/>
-      <c r="D17" s="94"/>
-      <c r="E17" s="94"/>
-      <c r="F17" s="94"/>
-      <c r="G17" s="94"/>
-      <c r="H17" s="94"/>
+      <c r="A17" s="95"/>
+      <c r="B17" s="95"/>
+      <c r="C17" s="95"/>
+      <c r="D17" s="95"/>
+      <c r="E17" s="95"/>
+      <c r="F17" s="95"/>
+      <c r="G17" s="95"/>
+      <c r="H17" s="95"/>
     </row>
     <row r="18" spans="1:8" ht="15" customHeight="1">
       <c r="A18" s="33" t="s">
@@ -6262,25 +6265,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="94" t="s">
         <v>222</v>
       </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
+      <c r="B1" s="95"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="95"/>
+      <c r="G1" s="95"/>
+      <c r="H1" s="95"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
-      <c r="A3" s="102" t="s">
+      <c r="A3" s="103" t="s">
         <v>223</v>
       </c>
-      <c r="B3" s="94"/>
-      <c r="C3" s="94"/>
-      <c r="D3" s="94"/>
-      <c r="E3" s="94"/>
+      <c r="B3" s="95"/>
+      <c r="C3" s="95"/>
+      <c r="D3" s="95"/>
+      <c r="E3" s="95"/>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -6368,16 +6371,16 @@
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
-      <c r="A11" s="102" t="s">
+      <c r="A11" s="103" t="s">
         <v>243</v>
       </c>
-      <c r="B11" s="94"/>
-      <c r="C11" s="94"/>
-      <c r="D11" s="94"/>
-      <c r="E11" s="94"/>
-      <c r="F11" s="94"/>
-      <c r="G11" s="94"/>
-      <c r="H11" s="94"/>
+      <c r="B11" s="95"/>
+      <c r="C11" s="95"/>
+      <c r="D11" s="95"/>
+      <c r="E11" s="95"/>
+      <c r="F11" s="95"/>
+      <c r="G11" s="95"/>
+      <c r="H11" s="95"/>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
       <c r="A12" s="1" t="s">
@@ -6533,24 +6536,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="94" t="s">
         <v>250</v>
       </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
+      <c r="B1" s="95"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="95"/>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1">
-      <c r="A3" s="102" t="s">
+      <c r="A3" s="103" t="s">
         <v>251</v>
       </c>
-      <c r="B3" s="94"/>
-      <c r="C3" s="94"/>
-      <c r="D3" s="94"/>
-      <c r="E3" s="94"/>
-      <c r="F3" s="94"/>
+      <c r="B3" s="95"/>
+      <c r="C3" s="95"/>
+      <c r="D3" s="95"/>
+      <c r="E3" s="95"/>
+      <c r="F3" s="95"/>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1">
       <c r="A4" s="5" t="s">
@@ -6633,10 +6636,10 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A8" s="107" t="s">
+      <c r="A8" s="108" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="98"/>
+      <c r="B8" s="99"/>
       <c r="C8" s="35">
         <v>500</v>
       </c>
@@ -6671,18 +6674,18 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1">
-      <c r="A10" s="105"/>
-      <c r="B10" s="97"/>
-      <c r="C10" s="97"/>
-      <c r="D10" s="97"/>
-      <c r="E10" s="97"/>
-      <c r="F10" s="98"/>
+      <c r="A10" s="106"/>
+      <c r="B10" s="98"/>
+      <c r="C10" s="98"/>
+      <c r="D10" s="98"/>
+      <c r="E10" s="98"/>
+      <c r="F10" s="99"/>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1">
-      <c r="A11" s="103" t="s">
+      <c r="A11" s="104" t="s">
         <v>197</v>
       </c>
-      <c r="B11" s="98"/>
+      <c r="B11" s="99"/>
       <c r="C11" s="34">
         <f>SUM(C5:C9)</f>
         <v>4180</v>
@@ -6743,14 +6746,14 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="15" customHeight="1">
-      <c r="A17" s="106" t="s">
+      <c r="A17" s="107" t="s">
         <v>265</v>
       </c>
-      <c r="B17" s="97"/>
-      <c r="C17" s="97"/>
-      <c r="D17" s="97"/>
-      <c r="E17" s="97"/>
-      <c r="F17" s="98"/>
+      <c r="B17" s="98"/>
+      <c r="C17" s="98"/>
+      <c r="D17" s="98"/>
+      <c r="E17" s="98"/>
+      <c r="F17" s="99"/>
     </row>
     <row r="18" spans="1:6" ht="15" customHeight="1">
       <c r="A18" s="11" t="s">
@@ -6801,14 +6804,14 @@
       </c>
     </row>
     <row r="23" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A23" s="106" t="s">
+      <c r="A23" s="107" t="s">
         <v>163</v>
       </c>
-      <c r="B23" s="97"/>
-      <c r="C23" s="97"/>
-      <c r="D23" s="97"/>
-      <c r="E23" s="97"/>
-      <c r="F23" s="98"/>
+      <c r="B23" s="98"/>
+      <c r="C23" s="98"/>
+      <c r="D23" s="98"/>
+      <c r="E23" s="98"/>
+      <c r="F23" s="99"/>
     </row>
     <row r="24" spans="1:6" ht="16.5" customHeight="1">
       <c r="A24" s="8" t="s">
@@ -6980,28 +6983,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="94" t="s">
         <v>281</v>
       </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="94"/>
+      <c r="B1" s="95"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="95"/>
+      <c r="G1" s="95"/>
+      <c r="H1" s="95"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="96" t="s">
         <v>282</v>
       </c>
-      <c r="B2" s="94"/>
-      <c r="C2" s="94"/>
-      <c r="D2" s="94"/>
-      <c r="E2" s="94"/>
-      <c r="F2" s="94"/>
-      <c r="G2" s="94"/>
-      <c r="H2" s="94"/>
+      <c r="B2" s="95"/>
+      <c r="C2" s="95"/>
+      <c r="D2" s="95"/>
+      <c r="E2" s="95"/>
+      <c r="F2" s="95"/>
+      <c r="G2" s="95"/>
+      <c r="H2" s="95"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -7378,14 +7381,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="108" t="s">
+      <c r="A1" s="109" t="s">
         <v>295</v>
       </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
+      <c r="B1" s="95"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="95"/>
     </row>
     <row r="2" spans="1:6" ht="24.95" customHeight="1">
       <c r="A2" s="9" t="s">

</xml_diff>